<commit_message>
Split poisons and bait stations into their own lines
The staff materials table now carries Zernocid and Pest Killer as separate
quantity-and-cost pairs beside the glue stations, and the one-off bait
station purchase is broken out by contour: 179 on contour 1 and 1 198 on
contour 2, 1 377 in total at 2 160 each, 2 974 320.

Object sheets list the one-off purchase as two rows rather than one.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLozcDkCvYTXvP2yAkyMFB
</commit_message>
<xml_diff>
--- a/reports/УКПФ_дератизация_сравнение_КП.xlsx
+++ b/reports/УКПФ_дератизация_сравнение_КП.xlsx
@@ -201,13 +201,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1179,7 +1179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="B19" s="29" t="inlineStr">
         <is>
-          <t>Приманочные станции 1-го и 2-го контура — разовая закупка, в ежемесячную себестоимость не входит</t>
+          <t>Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
       <c r="C19" s="22" t="inlineStr">
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="D19" s="6">
-        <f>(Данные!$B$20+Данные!$C$20)*Данные!$B$9</f>
+        <f>Данные!$B$20*Данные!$B$9</f>
         <v/>
       </c>
       <c r="E19" s="30" t="n">
@@ -1530,106 +1530,134 @@
       </c>
     </row>
     <row r="20">
-      <c r="E20" s="31" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Штат УКПФ</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>Приманочные станции 2-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="6">
+        <f>Данные!$C$20*Данные!$B$9</f>
+        <v/>
+      </c>
+      <c r="E20" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="12">
+        <f>D20*E20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" s="31" t="inlineStr">
         <is>
           <t>Итого блока</t>
         </is>
       </c>
-      <c r="F20" s="9">
-        <f>SUM(F19:F19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="F21" s="9">
+        <f>SUM(F19:F20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
         </is>
       </c>
-      <c r="B22" s="16" t="n"/>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="16" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="16" t="n"/>
+      <c r="F23" s="16" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="inlineStr">
         <is>
           <t>Вариант</t>
         </is>
       </c>
-      <c r="B23" s="27" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>Что входит</t>
         </is>
       </c>
-      <c r="C23" s="28" t="inlineStr">
+      <c r="C24" s="28" t="inlineStr">
         <is>
           <t>Обходов в месяц</t>
         </is>
       </c>
-      <c r="D23" s="28" t="inlineStr">
+      <c r="D24" s="28" t="inlineStr">
         <is>
           <t>Цена в месяц</t>
         </is>
       </c>
-      <c r="E23" s="28" t="inlineStr">
+      <c r="E24" s="28" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F23" s="28" t="inlineStr">
+      <c r="F24" s="28" t="inlineStr">
         <is>
           <t>За год</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="B25" s="29" t="inlineStr">
         <is>
           <t>дезинсекция</t>
         </is>
       </c>
-      <c r="C24" s="22" t="n">
+      <c r="C25" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D25" s="6">
         <f>Данные!$B$54</f>
         <v/>
       </c>
-      <c r="E24" s="30" t="n">
+      <c r="E25" s="30" t="n">
         <v>12</v>
       </c>
-      <c r="F24" s="12">
-        <f>D24*E24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="E25" s="31" t="inlineStr">
+      <c r="F25" s="12">
+        <f>D25*E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" s="31" t="inlineStr">
         <is>
           <t>Итого блока</t>
         </is>
       </c>
-      <c r="F25" s="9">
-        <f>SUM(F24:F24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="23" t="inlineStr">
-        <is>
-          <t>Зерноцид по ККЗ в нормах не заявлен, поэтому строка Зерноцида даёт ноль.</t>
-        </is>
+      <c r="F26" s="9">
+        <f>SUM(F25:F25)</f>
+        <v/>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>Зерноцид по ККЗ в нормах не заявлен, поэтому строка Зерноцида даёт ноль.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>Зарплата дератизаторов по объектам не делится — она на листе «Штат УКПФ».</t>
         </is>
@@ -1638,8 +1666,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A29:F29"/>
     <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A27:F27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1651,7 +1679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2258,7 +2286,7 @@
       </c>
       <c r="B31" s="29" t="inlineStr">
         <is>
-          <t>Приманочные станции 1-го и 2-го контура — разовая закупка, в ежемесячную себестоимость не входит</t>
+          <t>Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
       <c r="C31" s="22" t="inlineStr">
@@ -2267,7 +2295,7 @@
         </is>
       </c>
       <c r="D31" s="6">
-        <f>(SUM(Данные!$B$23:$B$30)+SUM(Данные!$C$23:$C$30))*Данные!$B$9</f>
+        <f>SUM(Данные!$B$23:$B$30)*Данные!$B$9</f>
         <v/>
       </c>
       <c r="E31" s="30" t="n">
@@ -2279,86 +2307,86 @@
       </c>
     </row>
     <row r="32">
-      <c r="E32" s="31" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Штат УКПФ</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="inlineStr">
+        <is>
+          <t>Приманочные станции 2-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D32" s="6">
+        <f>SUM(Данные!$C$23:$C$30)*Данные!$B$9</f>
+        <v/>
+      </c>
+      <c r="E32" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="12">
+        <f>D32*E32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="E33" s="31" t="inlineStr">
         <is>
           <t>Итого блока</t>
         </is>
       </c>
-      <c r="F32" s="9">
-        <f>SUM(F31:F31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="15" t="inlineStr">
+      <c r="F33" s="9">
+        <f>SUM(F31:F32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
         </is>
       </c>
-      <c r="B34" s="16" t="n"/>
-      <c r="C34" s="16" t="n"/>
-      <c r="D34" s="16" t="n"/>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="16" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="27" t="inlineStr">
+      <c r="B35" s="16" t="n"/>
+      <c r="C35" s="16" t="n"/>
+      <c r="D35" s="16" t="n"/>
+      <c r="E35" s="16" t="n"/>
+      <c r="F35" s="16" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="27" t="inlineStr">
         <is>
           <t>Вариант</t>
         </is>
       </c>
-      <c r="B35" s="27" t="inlineStr">
+      <c r="B36" s="27" t="inlineStr">
         <is>
           <t>Что входит</t>
         </is>
       </c>
-      <c r="C35" s="28" t="inlineStr">
+      <c r="C36" s="28" t="inlineStr">
         <is>
           <t>Обходов в месяц</t>
         </is>
       </c>
-      <c r="D35" s="28" t="inlineStr">
+      <c r="D36" s="28" t="inlineStr">
         <is>
           <t>Цена в месяц</t>
         </is>
       </c>
-      <c r="E35" s="28" t="inlineStr">
+      <c r="E36" s="28" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F35" s="28" t="inlineStr">
+      <c r="F36" s="28" t="inlineStr">
         <is>
           <t>За год</t>
         </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B36" s="29" t="inlineStr">
-        <is>
-          <t>Айыртау БП</t>
-        </is>
-      </c>
-      <c r="C36" s="22" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D36" s="6">
-        <f>Данные!$B$48</f>
-        <v/>
-      </c>
-      <c r="E36" s="30" t="n">
-        <v>12</v>
-      </c>
-      <c r="F36" s="12">
-        <f>D36*E36</f>
-        <v/>
       </c>
     </row>
     <row r="37">
@@ -2369,7 +2397,7 @@
       </c>
       <c r="B37" s="29" t="inlineStr">
         <is>
-          <t>Многоэтажки Д и Г</t>
+          <t>Айыртау БП</t>
         </is>
       </c>
       <c r="C37" s="22" t="inlineStr">
@@ -2378,7 +2406,7 @@
         </is>
       </c>
       <c r="D37" s="6">
-        <f>Данные!$B$49</f>
+        <f>Данные!$B$48</f>
         <v/>
       </c>
       <c r="E37" s="30" t="n">
@@ -2397,7 +2425,7 @@
       </c>
       <c r="B38" s="29" t="inlineStr">
         <is>
-          <t>Площадки А, Б, Е, Ж, В (РМ), В</t>
+          <t>Многоэтажки Д и Г</t>
         </is>
       </c>
       <c r="C38" s="22" t="inlineStr">
@@ -2406,7 +2434,7 @@
         </is>
       </c>
       <c r="D38" s="6">
-        <f>Данные!$B$50</f>
+        <f>Данные!$B$49</f>
         <v/>
       </c>
       <c r="E38" s="30" t="n">
@@ -2418,35 +2446,63 @@
       </c>
     </row>
     <row r="39">
-      <c r="E39" s="31" t="inlineStr">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Indigo Solutions</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="inlineStr">
+        <is>
+          <t>Площадки А, Б, Е, Ж, В (РМ), В</t>
+        </is>
+      </c>
+      <c r="C39" s="22" t="inlineStr">
+        <is>
+          <t>в КП не указана</t>
+        </is>
+      </c>
+      <c r="D39" s="6">
+        <f>Данные!$B$50</f>
+        <v/>
+      </c>
+      <c r="E39" s="30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F39" s="12">
+        <f>D39*E39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" s="31" t="inlineStr">
         <is>
           <t>Итого блока</t>
         </is>
       </c>
-      <c r="F39" s="9">
-        <f>SUM(F36:F38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="23" t="inlineStr">
-        <is>
-          <t>Состав площадок у Indigo и в нашем расчёте описан по-разному: у них шесть напольных площадок плюс «В (рем. молод)», у нас восемь площадок по контурам. Сопоставлять построчно нельзя, только суммарно.</t>
-        </is>
+      <c r="F40" s="9">
+        <f>SUM(F37:F39)</f>
+        <v/>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="23" t="inlineStr">
         <is>
+          <t>Состав площадок у Indigo и в нашем расчёте описан по-разному: у них шесть напольных площадок плюс «В (рем. молод)», у нас восемь площадок по контурам. Сопоставлять построчно нельзя, только суммарно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="23" t="inlineStr">
+        <is>
           <t>Разовая закупка приманочных станций 1-го и 2-го контура показана справочно и в годовой итог не входит.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2458,7 +2514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2872,7 +2928,7 @@
       </c>
       <c r="B24" s="29" t="inlineStr">
         <is>
-          <t>Приманочные станции 1-го и 2-го контура — разовая закупка, в ежемесячную себестоимость не входит</t>
+          <t>Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
       <c r="C24" s="22" t="inlineStr">
@@ -2881,7 +2937,7 @@
         </is>
       </c>
       <c r="D24" s="6">
-        <f>(Данные!$B$21+Данные!$C$21)*Данные!$B$9</f>
+        <f>Данные!$B$21*Данные!$B$9</f>
         <v/>
       </c>
       <c r="E24" s="30" t="n">
@@ -2893,101 +2949,129 @@
       </c>
     </row>
     <row r="25">
-      <c r="E25" s="31" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Штат УКПФ</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>Приманочные станции 2-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D25" s="6">
+        <f>Данные!$C$21*Данные!$B$9</f>
+        <v/>
+      </c>
+      <c r="E25" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="12">
+        <f>D25*E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" s="31" t="inlineStr">
         <is>
           <t>Итого блока</t>
         </is>
       </c>
-      <c r="F25" s="9">
-        <f>SUM(F24:F24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="F26" s="9">
+        <f>SUM(F24:F25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
         </is>
       </c>
-      <c r="B27" s="16" t="n"/>
-      <c r="C27" s="16" t="n"/>
-      <c r="D27" s="16" t="n"/>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="16" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="27" t="inlineStr">
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="16" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
         <is>
           <t>Вариант</t>
         </is>
       </c>
-      <c r="B28" s="27" t="inlineStr">
+      <c r="B29" s="27" t="inlineStr">
         <is>
           <t>Что входит</t>
         </is>
       </c>
-      <c r="C28" s="28" t="inlineStr">
+      <c r="C29" s="28" t="inlineStr">
         <is>
           <t>Обходов в месяц</t>
         </is>
       </c>
-      <c r="D28" s="28" t="inlineStr">
+      <c r="D29" s="28" t="inlineStr">
         <is>
           <t>Цена в месяц</t>
         </is>
       </c>
-      <c r="E28" s="28" t="inlineStr">
+      <c r="E29" s="28" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F28" s="28" t="inlineStr">
+      <c r="F29" s="28" t="inlineStr">
         <is>
           <t>За год</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="B29" s="29" t="inlineStr">
+      <c r="B30" s="29" t="inlineStr">
         <is>
           <t>дезинсекция</t>
         </is>
       </c>
-      <c r="C29" s="22" t="inlineStr">
+      <c r="C30" s="22" t="inlineStr">
         <is>
           <t>в КП не указана</t>
         </is>
       </c>
-      <c r="D29" s="6">
+      <c r="D30" s="6">
         <f>Данные!$B$51</f>
         <v/>
       </c>
-      <c r="E29" s="30" t="n">
+      <c r="E30" s="30" t="n">
         <v>12</v>
       </c>
-      <c r="F29" s="12">
-        <f>D29*E29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="E30" s="31" t="inlineStr">
+      <c r="F30" s="12">
+        <f>D30*E30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" s="31" t="inlineStr">
         <is>
           <t>Итого блока</t>
         </is>
       </c>
-      <c r="F30" s="9">
-        <f>SUM(F29:F29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="23" t="inlineStr">
+      <c r="F31" s="9">
+        <f>SUM(F30:F30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>Нормы штата по инкубаторию: 18 точек 1-го контура, 34 второго, 12 клеевых третьего; 1 кг брикетов Pest Killer и 1 кг Зерноцида на обработку.</t>
         </is>
@@ -2996,7 +3080,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A33:F33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3616,7 +3700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3946,7 +4030,7 @@
       </c>
       <c r="B19" s="29" t="inlineStr">
         <is>
-          <t>Приманочные станции 1-го и 2-го контура — разовая закупка, в ежемесячную себестоимость не входит</t>
+          <t>Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
       <c r="C19" s="22" t="inlineStr">
@@ -3955,7 +4039,7 @@
         </is>
       </c>
       <c r="D19" s="6">
-        <f>(Данные!$B$22+Данные!$C$22)*Данные!$B$9</f>
+        <f>Данные!$B$22*Данные!$B$9</f>
         <v/>
       </c>
       <c r="E19" s="30" t="n">
@@ -3967,34 +4051,62 @@
       </c>
     </row>
     <row r="20">
-      <c r="E20" s="31" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Штат УКПФ</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>Приманочные станции 2-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="6">
+        <f>Данные!$C$22*Данные!$B$9</f>
+        <v/>
+      </c>
+      <c r="E20" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="12">
+        <f>D20*E20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" s="31" t="inlineStr">
         <is>
           <t>Итого блока</t>
         </is>
       </c>
-      <c r="F20" s="9">
-        <f>SUM(F19:F19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="23" t="inlineStr">
-        <is>
-          <t>Клеевые станции по корпусам: Б — 11, Ж — 5, Е — 6, В — 6, В (РМ) — 6, Д — 3, Г — 3, БП-12 — 6, БП-13 — 6, БП-14 — 6, А — 5. Приманочные: 4, 2, 3, 3, 3, 4, 3, 5, 5, 5, 2.</t>
-        </is>
+      <c r="F21" s="9">
+        <f>SUM(F19:F20)</f>
+        <v/>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="23" t="inlineStr">
         <is>
+          <t>Клеевые станции по корпусам: Б — 11, Ж — 5, Е — 6, В — 6, В (РМ) — 6, Д — 3, Г — 3, БП-12 — 6, БП-13 — 6, БП-14 — 6, А — 5. Приманочные: 4, 2, 3, 3, 3, 4, 3, 5, 5, 5, 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
           <t>Норма 1,3 кг брикетов Pest Killer по АБК — приблизительная оценка, требует подтверждения. Зерноцид по АБК не заявлен.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A23:F23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4007,16 +4119,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4124,7 +4238,7 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>МАТЕРИАЛЫ ПО ОБЪЕКТАМ — СТАНЦИИ И ЯДЫ РАЗДЕЛЬНО</t>
+          <t>МАТЕРИАЛЫ ПО ОБЪЕКТАМ — СТАНЦИИ, ЗЕРНОЦИД И БРИКЕТЫ РАЗДЕЛЬНО</t>
         </is>
       </c>
       <c r="B11" s="16" t="n"/>
@@ -4133,6 +4247,8 @@
       <c r="E11" s="16" t="n"/>
       <c r="F11" s="16" t="n"/>
       <c r="G11" s="16" t="n"/>
+      <c r="H11" s="16" t="n"/>
+      <c r="I11" s="16" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="34" t="inlineStr">
@@ -4157,15 +4273,25 @@
       </c>
       <c r="E12" s="35" t="inlineStr">
         <is>
+          <t>Зерноцид, кг/мес</t>
+        </is>
+      </c>
+      <c r="F12" s="35" t="inlineStr">
+        <is>
           <t>Зерноцид за год, ₸</t>
         </is>
       </c>
-      <c r="F12" s="35" t="inlineStr">
+      <c r="G12" s="35" t="inlineStr">
+        <is>
+          <t>Pest Killer, кг/мес</t>
+        </is>
+      </c>
+      <c r="H12" s="35" t="inlineStr">
         <is>
           <t>Pest Killer за год, ₸</t>
         </is>
       </c>
-      <c r="G12" s="35" t="inlineStr">
+      <c r="I12" s="35" t="inlineStr">
         <is>
           <t>Материалы за год, ₸</t>
         </is>
@@ -4189,16 +4315,24 @@
         <f>B13*Данные!$B$8*Данные!$B$15+C13*Данные!$B$8*Данные!$B$16</f>
         <v/>
       </c>
-      <c r="E13" s="12">
-        <f>Данные!$G$20*Данные!$B$6*Данные!$B$15</f>
+      <c r="E13" s="37">
+        <f>Данные!$G$20</f>
         <v/>
       </c>
       <c r="F13" s="12">
-        <f>Данные!$F$20*Данные!$B$7*Данные!$B$15</f>
-        <v/>
-      </c>
-      <c r="G13" s="17">
-        <f>D13+E13+F13</f>
+        <f>E13*Данные!$B$6*Данные!$B$15</f>
+        <v/>
+      </c>
+      <c r="G13" s="37">
+        <f>Данные!$F$20</f>
+        <v/>
+      </c>
+      <c r="H13" s="12">
+        <f>G13*Данные!$B$7*Данные!$B$15</f>
+        <v/>
+      </c>
+      <c r="I13" s="17">
+        <f>D13+F13+H13</f>
         <v/>
       </c>
     </row>
@@ -4220,16 +4354,24 @@
         <f>B14*Данные!$B$8*Данные!$B$15+C14*Данные!$B$8*Данные!$B$16</f>
         <v/>
       </c>
-      <c r="E14" s="12">
-        <f>SUM(Данные!$G$23:$G$30)*Данные!$B$6*Данные!$B$15</f>
+      <c r="E14" s="37">
+        <f>SUM(Данные!$G$23:$G$30)</f>
         <v/>
       </c>
       <c r="F14" s="12">
-        <f>SUM(Данные!$F$23:$F$30)*Данные!$B$7*Данные!$B$15</f>
-        <v/>
-      </c>
-      <c r="G14" s="17">
-        <f>D14+E14+F14</f>
+        <f>E14*Данные!$B$6*Данные!$B$15</f>
+        <v/>
+      </c>
+      <c r="G14" s="37">
+        <f>SUM(Данные!$F$23:$F$30)</f>
+        <v/>
+      </c>
+      <c r="H14" s="12">
+        <f>G14*Данные!$B$7*Данные!$B$15</f>
+        <v/>
+      </c>
+      <c r="I14" s="17">
+        <f>D14+F14+H14</f>
         <v/>
       </c>
     </row>
@@ -4251,16 +4393,24 @@
         <f>B15*Данные!$B$8*Данные!$B$15+C15*Данные!$B$8*Данные!$B$16</f>
         <v/>
       </c>
-      <c r="E15" s="12">
-        <f>Данные!$G$21*Данные!$B$6*Данные!$B$15</f>
+      <c r="E15" s="37">
+        <f>Данные!$G$21</f>
         <v/>
       </c>
       <c r="F15" s="12">
-        <f>Данные!$F$21*Данные!$B$7*Данные!$B$15</f>
-        <v/>
-      </c>
-      <c r="G15" s="17">
-        <f>D15+E15+F15</f>
+        <f>E15*Данные!$B$6*Данные!$B$15</f>
+        <v/>
+      </c>
+      <c r="G15" s="37">
+        <f>Данные!$F$21</f>
+        <v/>
+      </c>
+      <c r="H15" s="12">
+        <f>G15*Данные!$B$7*Данные!$B$15</f>
+        <v/>
+      </c>
+      <c r="I15" s="17">
+        <f>D15+F15+H15</f>
         <v/>
       </c>
     </row>
@@ -4282,16 +4432,24 @@
         <f>B16*Данные!$B$8*Данные!$B$15+C16*Данные!$B$8*Данные!$B$16</f>
         <v/>
       </c>
-      <c r="E16" s="12">
-        <f>Данные!$G$22*Данные!$B$6*Данные!$B$15</f>
+      <c r="E16" s="37">
+        <f>Данные!$G$22</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>Данные!$F$22*Данные!$B$7*Данные!$B$15</f>
-        <v/>
-      </c>
-      <c r="G16" s="17">
-        <f>D16+E16+F16</f>
+        <f>E16*Данные!$B$6*Данные!$B$15</f>
+        <v/>
+      </c>
+      <c r="G16" s="37">
+        <f>Данные!$F$22</f>
+        <v/>
+      </c>
+      <c r="H16" s="12">
+        <f>G16*Данные!$B$7*Данные!$B$15</f>
+        <v/>
+      </c>
+      <c r="I16" s="17">
+        <f>D16+F16+H16</f>
         <v/>
       </c>
     </row>
@@ -4306,7 +4464,9 @@
       <c r="D17" s="11" t="n"/>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="11" t="n"/>
-      <c r="G17" s="17">
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="11" t="n"/>
+      <c r="I17" s="17">
         <f>Данные!$B$11*Данные!$B$10*Данные!$B$15</f>
         <v/>
       </c>
@@ -4323,7 +4483,7 @@
         <f>SUM(D13:D17)</f>
         <v/>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="38">
         <f>SUM(E13:E17)</f>
         <v/>
       </c>
@@ -4331,20 +4491,30 @@
         <f>SUM(F13:F17)</f>
         <v/>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="38">
         <f>SUM(G13:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="9">
+        <f>SUM(H13:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="9">
+        <f>SUM(I13:I17)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>РАЗОВАЯ ЗАКУПКА ПРИМАНОЧНЫХ СТАНЦИЙ 1-го И 2-го КОНТУРА</t>
+          <t>РАЗОВАЯ ЗАКУПКА ПРИМАНОЧНЫХ СТАНЦИЙ</t>
         </is>
       </c>
       <c r="B20" s="16" t="n"/>
       <c r="C20" s="16" t="n"/>
       <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
@@ -4354,15 +4524,25 @@
       </c>
       <c r="B21" s="28" t="inlineStr">
         <is>
-          <t>Точек 1-го и 2-го контура, шт</t>
+          <t>1-й контур, шт</t>
         </is>
       </c>
       <c r="C21" s="28" t="inlineStr">
         <is>
+          <t>2-й контур, шт</t>
+        </is>
+      </c>
+      <c r="D21" s="28" t="inlineStr">
+        <is>
+          <t>Всего, шт</t>
+        </is>
+      </c>
+      <c r="E21" s="28" t="inlineStr">
+        <is>
           <t>Цена, ₸/шт</t>
         </is>
       </c>
-      <c r="D21" s="28" t="inlineStr">
+      <c r="F21" s="28" t="inlineStr">
         <is>
           <t>Разово, ₸</t>
         </is>
@@ -4375,15 +4555,23 @@
         </is>
       </c>
       <c r="B22" s="36">
-        <f>Данные!$B$20+Данные!$C$20</f>
-        <v/>
-      </c>
-      <c r="C22" s="6">
+        <f>Данные!$B$20</f>
+        <v/>
+      </c>
+      <c r="C22" s="36">
+        <f>Данные!$C$20</f>
+        <v/>
+      </c>
+      <c r="D22" s="36">
+        <f>B22+C22</f>
+        <v/>
+      </c>
+      <c r="E22" s="6">
         <f>Данные!$B$9</f>
         <v/>
       </c>
-      <c r="D22" s="17">
-        <f>B22*C22</f>
+      <c r="F22" s="17">
+        <f>D22*E22</f>
         <v/>
       </c>
     </row>
@@ -4394,15 +4582,23 @@
         </is>
       </c>
       <c r="B23" s="36">
-        <f>SUM(Данные!$B$23:$B$30)+SUM(Данные!$C$23:$C$30)</f>
-        <v/>
-      </c>
-      <c r="C23" s="6">
+        <f>SUM(Данные!$B$23:$B$30)</f>
+        <v/>
+      </c>
+      <c r="C23" s="36">
+        <f>SUM(Данные!$C$23:$C$30)</f>
+        <v/>
+      </c>
+      <c r="D23" s="36">
+        <f>B23+C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="6">
         <f>Данные!$B$9</f>
         <v/>
       </c>
-      <c r="D23" s="17">
-        <f>B23*C23</f>
+      <c r="F23" s="17">
+        <f>D23*E23</f>
         <v/>
       </c>
     </row>
@@ -4413,15 +4609,23 @@
         </is>
       </c>
       <c r="B24" s="36">
-        <f>Данные!$B$21+Данные!$C$21</f>
-        <v/>
-      </c>
-      <c r="C24" s="6">
+        <f>Данные!$B$21</f>
+        <v/>
+      </c>
+      <c r="C24" s="36">
+        <f>Данные!$C$21</f>
+        <v/>
+      </c>
+      <c r="D24" s="36">
+        <f>B24+C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="6">
         <f>Данные!$B$9</f>
         <v/>
       </c>
-      <c r="D24" s="17">
-        <f>B24*C24</f>
+      <c r="F24" s="17">
+        <f>D24*E24</f>
         <v/>
       </c>
     </row>
@@ -4432,15 +4636,23 @@
         </is>
       </c>
       <c r="B25" s="36">
-        <f>Данные!$B$22+Данные!$C$22</f>
-        <v/>
-      </c>
-      <c r="C25" s="6">
+        <f>Данные!$B$22</f>
+        <v/>
+      </c>
+      <c r="C25" s="36">
+        <f>Данные!$C$22</f>
+        <v/>
+      </c>
+      <c r="D25" s="36">
+        <f>B25+C25</f>
+        <v/>
+      </c>
+      <c r="E25" s="6">
         <f>Данные!$B$9</f>
         <v/>
       </c>
-      <c r="D25" s="17">
-        <f>B25*C25</f>
+      <c r="F25" s="17">
+        <f>D25*E25</f>
         <v/>
       </c>
     </row>
@@ -4450,13 +4662,21 @@
           <t>ИТОГО РАЗОВО</t>
         </is>
       </c>
-      <c r="B26" s="37">
+      <c r="B26" s="39">
         <f>SUM(B22:B25)</f>
         <v/>
       </c>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="9">
+      <c r="C26" s="39">
+        <f>SUM(C22:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="39">
         <f>SUM(D22:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="9">
+        <f>SUM(F22:F25)</f>
         <v/>
       </c>
     </row>
@@ -4517,7 +4737,7 @@
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>'Штат УКПФ'!$G$18</f>
+        <f>'Штат УКПФ'!$I$18</f>
         <v/>
       </c>
       <c r="E30" s="17">
@@ -4542,7 +4762,7 @@
         <v/>
       </c>
       <c r="D31" s="12">
-        <f>'Штат УКПФ'!$G$18</f>
+        <f>'Штат УКПФ'!$I$18</f>
         <v/>
       </c>
       <c r="E31" s="17">
@@ -4567,7 +4787,7 @@
         <v/>
       </c>
       <c r="D32" s="12">
-        <f>'Штат УКПФ'!$G$18</f>
+        <f>'Штат УКПФ'!$I$18</f>
         <v/>
       </c>
       <c r="E32" s="17">
@@ -4592,7 +4812,7 @@
         <v/>
       </c>
       <c r="D33" s="12">
-        <f>'Штат УКПФ'!$G$18</f>
+        <f>'Штат УКПФ'!$I$18</f>
         <v/>
       </c>
       <c r="E33" s="17">
@@ -4617,7 +4837,7 @@
         <v/>
       </c>
       <c r="D34" s="12">
-        <f>'Штат УКПФ'!$G$18</f>
+        <f>'Штат УКПФ'!$I$18</f>
         <v/>
       </c>
       <c r="E34" s="17">
@@ -4642,7 +4862,7 @@
         <v/>
       </c>
       <c r="D35" s="12">
-        <f>'Штат УКПФ'!$G$18</f>
+        <f>'Штат УКПФ'!$I$18</f>
         <v/>
       </c>
       <c r="E35" s="17">
@@ -4667,7 +4887,7 @@
         <v/>
       </c>
       <c r="D36" s="12">
-        <f>'Штат УКПФ'!$G$18</f>
+        <f>'Штат УКПФ'!$I$18</f>
         <v/>
       </c>
       <c r="E36" s="17">
@@ -4692,7 +4912,7 @@
         <v/>
       </c>
       <c r="D37" s="12">
-        <f>'Штат УКПФ'!$G$18</f>
+        <f>'Штат УКПФ'!$I$18</f>
         <v/>
       </c>
       <c r="E37" s="17">
@@ -4717,7 +4937,7 @@
         <v/>
       </c>
       <c r="D38" s="12">
-        <f>'Штат УКПФ'!$G$18</f>
+        <f>'Штат УКПФ'!$I$18</f>
         <v/>
       </c>
       <c r="E38" s="17">
@@ -4824,7 +5044,7 @@
           <t>Зерноцид</t>
         </is>
       </c>
-      <c r="B6" s="38" t="n">
+      <c r="B6" s="40" t="n">
         <v>740</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -4844,7 +5064,7 @@
           <t>Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="40" t="n">
         <v>3642.5</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -4864,7 +5084,7 @@
           <t>Клеевая станция 3-го контура</t>
         </is>
       </c>
-      <c r="B8" s="38" t="n">
+      <c r="B8" s="40" t="n">
         <v>160</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -4884,7 +5104,7 @@
           <t>Приманочная станция 1–2 контура</t>
         </is>
       </c>
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="40" t="n">
         <v>2160</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -4904,7 +5124,7 @@
           <t>Бутылка</t>
         </is>
       </c>
-      <c r="B10" s="38" t="n">
+      <c r="B10" s="40" t="n">
         <v>68</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -4924,7 +5144,7 @@
           <t>Бутылки, расход</t>
         </is>
       </c>
-      <c r="B11" s="39" t="n">
+      <c r="B11" s="41" t="n">
         <v>40</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -4944,7 +5164,7 @@
           <t>Оклад дератизатора · вариант 1</t>
         </is>
       </c>
-      <c r="B12" s="38" t="n">
+      <c r="B12" s="40" t="n">
         <v>258488</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -4964,7 +5184,7 @@
           <t>Оклад дератизатора · вариант 2</t>
         </is>
       </c>
-      <c r="B13" s="38" t="n">
+      <c r="B13" s="40" t="n">
         <v>350000</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -4984,7 +5204,7 @@
           <t>Численность штата</t>
         </is>
       </c>
-      <c r="B14" s="39" t="n">
+      <c r="B14" s="41" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -5004,7 +5224,7 @@
           <t>Тёплых месяцев (апрель — октябрь)</t>
         </is>
       </c>
-      <c r="B15" s="39" t="n">
+      <c r="B15" s="41" t="n">
         <v>7</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -5024,7 +5244,7 @@
           <t>Зимних месяцев (ноябрь — март)</t>
         </is>
       </c>
-      <c r="B16" s="39" t="n">
+      <c r="B16" s="41" t="n">
         <v>5</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -5100,23 +5320,23 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B20" s="39" t="n">
+      <c r="B20" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="39" t="n">
+      <c r="C20" s="41" t="n">
         <v>29</v>
       </c>
-      <c r="D20" s="39" t="n">
+      <c r="D20" s="41" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="32">
         <f>SUM(B20:D20)</f>
         <v/>
       </c>
-      <c r="F20" s="40" t="n">
+      <c r="F20" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="40" t="n">
+      <c r="G20" s="42" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -5131,23 +5351,23 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B21" s="39" t="n">
+      <c r="B21" s="41" t="n">
         <v>18</v>
       </c>
-      <c r="C21" s="39" t="n">
+      <c r="C21" s="41" t="n">
         <v>34</v>
       </c>
-      <c r="D21" s="39" t="n">
+      <c r="D21" s="41" t="n">
         <v>12</v>
       </c>
       <c r="E21" s="32">
         <f>SUM(B21:D21)</f>
         <v/>
       </c>
-      <c r="F21" s="40" t="n">
+      <c r="F21" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="40" t="n">
+      <c r="G21" s="42" t="n">
         <v>1</v>
       </c>
       <c r="H21" s="7" t="inlineStr"/>
@@ -5158,23 +5378,23 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B22" s="39" t="n">
+      <c r="B22" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="39" t="n">
+      <c r="C22" s="41" t="n">
         <v>39</v>
       </c>
-      <c r="D22" s="39" t="n">
+      <c r="D22" s="41" t="n">
         <v>63</v>
       </c>
       <c r="E22" s="32">
         <f>SUM(B22:D22)</f>
         <v/>
       </c>
-      <c r="F22" s="40" t="n">
+      <c r="F22" s="42" t="n">
         <v>1.3</v>
       </c>
-      <c r="G22" s="40" t="n">
+      <c r="G22" s="42" t="n">
         <v>0</v>
       </c>
       <c r="H22" s="7" t="inlineStr">
@@ -5189,23 +5409,23 @@
           <t>Площадка А</t>
         </is>
       </c>
-      <c r="B23" s="39" t="n">
+      <c r="B23" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="C23" s="39" t="n">
+      <c r="C23" s="41" t="n">
         <v>147</v>
       </c>
-      <c r="D23" s="39" t="n">
+      <c r="D23" s="41" t="n">
         <v>20</v>
       </c>
       <c r="E23" s="32">
         <f>SUM(B23:D23)</f>
         <v/>
       </c>
-      <c r="F23" s="40" t="n">
+      <c r="F23" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="40" t="n">
+      <c r="G23" s="42" t="n">
         <v>2</v>
       </c>
       <c r="H23" s="7" t="inlineStr"/>
@@ -5216,23 +5436,23 @@
           <t>Площадка Б</t>
         </is>
       </c>
-      <c r="B24" s="39" t="n">
+      <c r="B24" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C24" s="39" t="n">
+      <c r="C24" s="41" t="n">
         <v>146</v>
       </c>
-      <c r="D24" s="39" t="n">
+      <c r="D24" s="41" t="n">
         <v>20</v>
       </c>
       <c r="E24" s="32">
         <f>SUM(B24:D24)</f>
         <v/>
       </c>
-      <c r="F24" s="40" t="n">
+      <c r="F24" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="40" t="n">
+      <c r="G24" s="42" t="n">
         <v>2</v>
       </c>
       <c r="H24" s="7" t="inlineStr"/>
@@ -5243,23 +5463,23 @@
           <t>В / Восточка</t>
         </is>
       </c>
-      <c r="B25" s="39" t="n">
+      <c r="B25" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="C25" s="39" t="n">
+      <c r="C25" s="41" t="n">
         <v>239</v>
       </c>
-      <c r="D25" s="39" t="n">
+      <c r="D25" s="41" t="n">
         <v>30</v>
       </c>
       <c r="E25" s="32">
         <f>SUM(B25:D25)</f>
         <v/>
       </c>
-      <c r="F25" s="40" t="n">
+      <c r="F25" s="42" t="n">
         <v>3.5</v>
       </c>
-      <c r="G25" s="40" t="n">
+      <c r="G25" s="42" t="n">
         <v>3</v>
       </c>
       <c r="H25" s="7" t="inlineStr"/>
@@ -5270,23 +5490,23 @@
           <t>Площадка Г</t>
         </is>
       </c>
-      <c r="B26" s="39" t="n">
+      <c r="B26" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C26" s="39" t="n">
+      <c r="C26" s="41" t="n">
         <v>88</v>
       </c>
-      <c r="D26" s="39" t="n">
+      <c r="D26" s="41" t="n">
         <v>80</v>
       </c>
       <c r="E26" s="32">
         <f>SUM(B26:D26)</f>
         <v/>
       </c>
-      <c r="F26" s="40" t="n">
+      <c r="F26" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="40" t="n">
+      <c r="G26" s="42" t="n">
         <v>1</v>
       </c>
       <c r="H26" s="7" t="inlineStr"/>
@@ -5297,23 +5517,23 @@
           <t>Площадка Д</t>
         </is>
       </c>
-      <c r="B27" s="39" t="n">
+      <c r="B27" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="C27" s="39" t="n">
+      <c r="C27" s="41" t="n">
         <v>69</v>
       </c>
-      <c r="D27" s="39" t="n">
+      <c r="D27" s="41" t="n">
         <v>64</v>
       </c>
       <c r="E27" s="32">
         <f>SUM(B27:D27)</f>
         <v/>
       </c>
-      <c r="F27" s="40" t="n">
+      <c r="F27" s="42" t="n">
         <v>1.5</v>
       </c>
-      <c r="G27" s="40" t="n">
+      <c r="G27" s="42" t="n">
         <v>1</v>
       </c>
       <c r="H27" s="7" t="inlineStr"/>
@@ -5324,23 +5544,23 @@
           <t>Площадка Е</t>
         </is>
       </c>
-      <c r="B28" s="39" t="n">
+      <c r="B28" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="C28" s="39" t="n">
+      <c r="C28" s="41" t="n">
         <v>147</v>
       </c>
-      <c r="D28" s="39" t="n">
+      <c r="D28" s="41" t="n">
         <v>20</v>
       </c>
       <c r="E28" s="32">
         <f>SUM(B28:D28)</f>
         <v/>
       </c>
-      <c r="F28" s="40" t="n">
+      <c r="F28" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="40" t="n">
+      <c r="G28" s="42" t="n">
         <v>2</v>
       </c>
       <c r="H28" s="7" t="inlineStr"/>
@@ -5351,23 +5571,23 @@
           <t>Площадка Ж</t>
         </is>
       </c>
-      <c r="B29" s="39" t="n">
+      <c r="B29" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C29" s="39" t="n">
+      <c r="C29" s="41" t="n">
         <v>73</v>
       </c>
-      <c r="D29" s="39" t="n">
+      <c r="D29" s="41" t="n">
         <v>10</v>
       </c>
       <c r="E29" s="32">
         <f>SUM(B29:D29)</f>
         <v/>
       </c>
-      <c r="F29" s="40" t="n">
+      <c r="F29" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="40" t="n">
+      <c r="G29" s="42" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="7" t="inlineStr"/>
@@ -5378,23 +5598,23 @@
           <t>Айыртау (БП)</t>
         </is>
       </c>
-      <c r="B30" s="39" t="n">
+      <c r="B30" s="41" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="39" t="n">
+      <c r="C30" s="41" t="n">
         <v>187</v>
       </c>
-      <c r="D30" s="39" t="n">
+      <c r="D30" s="41" t="n">
         <v>24</v>
       </c>
       <c r="E30" s="32">
         <f>SUM(B30:D30)</f>
         <v/>
       </c>
-      <c r="F30" s="40" t="n">
+      <c r="F30" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="G30" s="40" t="n">
+      <c r="G30" s="42" t="n">
         <v>3</v>
       </c>
       <c r="H30" s="7" t="inlineStr"/>
@@ -5409,8 +5629,8 @@
       <c r="C31" s="32" t="n"/>
       <c r="D31" s="32" t="n"/>
       <c r="E31" s="32" t="n"/>
-      <c r="F31" s="41" t="n"/>
-      <c r="G31" s="41" t="n"/>
+      <c r="F31" s="37" t="n"/>
+      <c r="G31" s="37" t="n"/>
       <c r="H31" s="7" t="inlineStr">
         <is>
           <t>нормы расхода не заданы</t>
@@ -5427,8 +5647,8 @@
       <c r="C32" s="32" t="n"/>
       <c r="D32" s="32" t="n"/>
       <c r="E32" s="32" t="n"/>
-      <c r="F32" s="41" t="n"/>
-      <c r="G32" s="41" t="n"/>
+      <c r="F32" s="37" t="n"/>
+      <c r="G32" s="37" t="n"/>
       <c r="H32" s="7" t="inlineStr">
         <is>
           <t>нормы расхода не заданы</t>
@@ -5441,27 +5661,27 @@
           <t>ИТОГО ПО ФАБРИКЕ</t>
         </is>
       </c>
-      <c r="B33" s="42">
+      <c r="B33" s="43">
         <f>SUM(B20:B32)</f>
         <v/>
       </c>
-      <c r="C33" s="42">
+      <c r="C33" s="43">
         <f>SUM(C20:C32)</f>
         <v/>
       </c>
-      <c r="D33" s="42">
+      <c r="D33" s="43">
         <f>SUM(D20:D32)</f>
         <v/>
       </c>
-      <c r="E33" s="42">
+      <c r="E33" s="43">
         <f>SUM(E20:E32)</f>
         <v/>
       </c>
-      <c r="F33" s="43">
+      <c r="F33" s="38">
         <f>SUM(F20:F32)</f>
         <v/>
       </c>
-      <c r="G33" s="43">
+      <c r="G33" s="38">
         <f>SUM(G20:G32)</f>
         <v/>
       </c>
@@ -5513,7 +5733,7 @@
           <t>Indigo · ККЗ, дератизация</t>
         </is>
       </c>
-      <c r="B37" s="38" t="n">
+      <c r="B37" s="40" t="n">
         <v>96600</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -5533,7 +5753,7 @@
           <t>Indigo · Айыртау БП, полная замена</t>
         </is>
       </c>
-      <c r="B38" s="38" t="n">
+      <c r="B38" s="40" t="n">
         <v>618400</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -5553,7 +5773,7 @@
           <t>Indigo · Айыртау БП, частичная замена</t>
         </is>
       </c>
-      <c r="B39" s="38" t="n">
+      <c r="B39" s="40" t="n">
         <v>478400</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -5573,7 +5793,7 @@
           <t>Indigo · Многоэтажки Д и Г, полная замена</t>
         </is>
       </c>
-      <c r="B40" s="38" t="n">
+      <c r="B40" s="40" t="n">
         <v>569800</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -5593,7 +5813,7 @@
           <t>Indigo · Многоэтажки Д и Г, частичная замена</t>
         </is>
       </c>
-      <c r="B41" s="38" t="n">
+      <c r="B41" s="40" t="n">
         <v>440700</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -5613,7 +5833,7 @@
           <t>Indigo · Площадки А,Б,Е,Ж,В,В(РМ), полная</t>
         </is>
       </c>
-      <c r="B42" s="38" t="n">
+      <c r="B42" s="40" t="n">
         <v>2599100</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -5633,7 +5853,7 @@
           <t>Indigo · Площадки А,Б,Е,Ж,В,В(РМ), частичная</t>
         </is>
       </c>
-      <c r="B43" s="38" t="n">
+      <c r="B43" s="40" t="n">
         <v>2010300</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -5653,7 +5873,7 @@
           <t>Indigo · Инкубаторий, полная замена</t>
         </is>
       </c>
-      <c r="B44" s="38" t="n">
+      <c r="B44" s="40" t="n">
         <v>126200</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
@@ -5673,7 +5893,7 @@
           <t>Indigo · Инкубаторий, частичная замена</t>
         </is>
       </c>
-      <c r="B45" s="38" t="n">
+      <c r="B45" s="40" t="n">
         <v>106800</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -5693,7 +5913,7 @@
           <t>Indigo · ЗПП, полная замена</t>
         </is>
       </c>
-      <c r="B46" s="38" t="n">
+      <c r="B46" s="40" t="n">
         <v>126200</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -5713,7 +5933,7 @@
           <t>Indigo · ЗПП, частичная замена</t>
         </is>
       </c>
-      <c r="B47" s="38" t="n">
+      <c r="B47" s="40" t="n">
         <v>106800</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -5733,7 +5953,7 @@
           <t>Indigo · дезинсекция, Айыртау БП</t>
         </is>
       </c>
-      <c r="B48" s="38" t="n">
+      <c r="B48" s="40" t="n">
         <v>720000</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -5753,7 +5973,7 @@
           <t>Indigo · дезинсекция, Многоэтажки</t>
         </is>
       </c>
-      <c r="B49" s="38" t="n">
+      <c r="B49" s="40" t="n">
         <v>1080000</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -5773,7 +5993,7 @@
           <t>Indigo · дезинсекция, Площадки</t>
         </is>
       </c>
-      <c r="B50" s="38" t="n">
+      <c r="B50" s="40" t="n">
         <v>3000000</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -5793,7 +6013,7 @@
           <t>Indigo · дезинсекция, Инкубаторий</t>
         </is>
       </c>
-      <c r="B51" s="38" t="n">
+      <c r="B51" s="40" t="n">
         <v>100800</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -5813,7 +6033,7 @@
           <t>Indigo · дезинсекция, ЗПП</t>
         </is>
       </c>
-      <c r="B52" s="38" t="n">
+      <c r="B52" s="40" t="n">
         <v>160800</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -5833,7 +6053,7 @@
           <t>Pest Hunters · ККЗ, дератизация</t>
         </is>
       </c>
-      <c r="B53" s="38" t="n">
+      <c r="B53" s="40" t="n">
         <v>75000</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -5853,7 +6073,7 @@
           <t>Pest Hunters · ККЗ, дезинсекция</t>
         </is>
       </c>
-      <c r="B54" s="38" t="n">
+      <c r="B54" s="40" t="n">
         <v>70000</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
@@ -5873,7 +6093,7 @@
           <t>Pest Hunters · площадки, март — ноябрь</t>
         </is>
       </c>
-      <c r="B55" s="38" t="n">
+      <c r="B55" s="40" t="n">
         <v>3172000</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
@@ -5893,7 +6113,7 @@
           <t>Pest Hunters · площадки, декабрь — февраль</t>
         </is>
       </c>
-      <c r="B56" s="38" t="n">
+      <c r="B56" s="40" t="n">
         <v>2074000</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -5913,7 +6133,7 @@
           <t>Pest Hunters · площадки альт., март — ноябрь</t>
         </is>
       </c>
-      <c r="B57" s="38" t="n">
+      <c r="B57" s="40" t="n">
         <v>2806000</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -5933,7 +6153,7 @@
           <t>Pest Hunters · площадки альт., дек. — февраль</t>
         </is>
       </c>
-      <c r="B58" s="38" t="n">
+      <c r="B58" s="40" t="n">
         <v>1830000</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
@@ -5953,7 +6173,7 @@
           <t>Pest Hunters · ЗПП</t>
         </is>
       </c>
-      <c r="B59" s="38" t="n">
+      <c r="B59" s="40" t="n">
         <v>180000</v>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -5973,7 +6193,7 @@
           <t>Pest Hunters · склад ТМЦ</t>
         </is>
       </c>
-      <c r="B60" s="38" t="n">
+      <c r="B60" s="40" t="n">
         <v>80000</v>
       </c>
       <c r="C60" s="5" t="inlineStr">
@@ -5993,7 +6213,7 @@
           <t>Месяцев высокого тарифа площадок (мар — ноя)</t>
         </is>
       </c>
-      <c r="B61" s="39" t="n">
+      <c r="B61" s="41" t="n">
         <v>9</v>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -6013,7 +6233,7 @@
           <t>Месяцев низкого тарифа площадок (дек — фев)</t>
         </is>
       </c>
-      <c r="B62" s="39" t="n">
+      <c r="B62" s="41" t="n">
         <v>3</v>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -6033,7 +6253,7 @@
           <t>Месяцев действия договора по складу ТМЦ</t>
         </is>
       </c>
-      <c r="B63" s="39" t="n">
+      <c r="B63" s="41" t="n">
         <v>9</v>
       </c>
       <c r="C63" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Drop the "what is included" column from the object sheets
Each object sheet is now a four-column table - item, price per month,
months, year - matching the shape of the lead comparison matrix. The
service description is folded into the item label where it adds anything.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLozcDkCvYTXvP2yAkyMFB
</commit_message>
<xml_diff>
--- a/reports/УКПФ_дератизация_сравнение_КП.xlsx
+++ b/reports/УКПФ_дератизация_сравнение_КП.xlsx
@@ -263,12 +263,6 @@
     <xf numFmtId="164" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -287,6 +281,12 @@
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1515,15 +1515,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1559,21 +1557,21 @@
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>Штат УКПФ · материалы</t>
+          <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="26">
-        <f>F9</f>
+        <f>D9</f>
         <v>1159200</v>
       </c>
       <c r="C5" s="26">
-        <f>F10</f>
+        <f>D10</f>
         <v>900000</v>
       </c>
       <c r="D5" s="26">
-        <f>F11+F12+F13+F14</f>
+        <f>D11+D12+D13+D14</f>
         <v>25497.5</v>
       </c>
     </row>
@@ -1587,211 +1585,149 @@
       <c r="B7" s="16" t="n"/>
       <c r="C7" s="16" t="n"/>
       <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>барьер вокруг периметра кормоцеха и грязный барьер</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D9" s="30">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · барьер вокруг периметра кормоцеха и грязный барьер</t>
+        </is>
+      </c>
+      <c r="B9" s="28">
         <f>Данные!$B$37</f>
         <v>96600</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="C9" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F9" s="8">
-        <f>D9*E9</f>
+      <c r="D9" s="8">
+        <f>B9*C9</f>
         <v>1159200</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Pest Hunters</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>дератизация</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="30">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Pest Hunters · дератизация</t>
+        </is>
+      </c>
+      <c r="B10" s="28">
         <f>Данные!$B$53</f>
         <v>75000</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="C10" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F10" s="8">
-        <f>D10*E10</f>
+      <c r="D10" s="8">
+        <f>B10*C10</f>
         <v>900000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>Клеевые станции 3-го контура, тёплый сезон</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D11" s="30">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
+        </is>
+      </c>
+      <c r="B11" s="28">
         <f>Данные!$D$20*Данные!$B$8</f>
         <v>0</v>
       </c>
-      <c r="E11" s="30">
+      <c r="C11" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F11" s="8">
-        <f>D11*E11</f>
+      <c r="D11" s="8">
+        <f>B11*C11</f>
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D12" s="30">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
+        </is>
+      </c>
+      <c r="B12" s="28">
         <f>Данные!$D$20*2*Данные!$B$8</f>
         <v>0</v>
       </c>
-      <c r="E12" s="30">
+      <c r="C12" s="28">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
-      <c r="F12" s="8">
-        <f>D12*E12</f>
+      <c r="D12" s="8">
+        <f>B12*C12</f>
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>Зерноцид, 2-й контур</t>
-        </is>
-      </c>
-      <c r="C13" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D13" s="30">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Зерноцид, 2-й контур</t>
+        </is>
+      </c>
+      <c r="B13" s="28">
         <f>Данные!$G$20*Данные!$B$6</f>
         <v>0</v>
       </c>
-      <c r="E13" s="30">
+      <c r="C13" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F13" s="8">
-        <f>D13*E13</f>
+      <c r="D13" s="8">
+        <f>B13*C13</f>
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>Pest Killer, брикеты</t>
-        </is>
-      </c>
-      <c r="C14" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D14" s="30">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Pest Killer, брикеты</t>
+        </is>
+      </c>
+      <c r="B14" s="28">
         <f>Данные!$F$20*Данные!$B$7</f>
         <v>3642.5</v>
       </c>
-      <c r="E14" s="30">
+      <c r="C14" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F14" s="8">
-        <f>D14*E14</f>
+      <c r="D14" s="8">
+        <f>B14*C14</f>
         <v>25497.5</v>
       </c>
     </row>
     <row r="15">
-      <c r="E15" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F15" s="12">
-        <f>SUM(F9:F14)</f>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D15" s="12">
+        <f>SUM(D9:D14)</f>
         <v>2084697.5</v>
       </c>
     </row>
@@ -1805,105 +1741,73 @@
       <c r="B17" s="16" t="n"/>
       <c r="C17" s="16" t="n"/>
       <c r="D17" s="16" t="n"/>
-      <c r="E17" s="16" t="n"/>
-      <c r="F17" s="16" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C18" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D18" s="28" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E18" s="28" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F18" s="28" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B19" s="29" t="inlineStr">
-        <is>
-          <t>Приманочные станции 1-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D19" s="30">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B19" s="28">
         <f>Данные!$B$20*Данные!$B$9</f>
         <v>0</v>
       </c>
-      <c r="E19" s="30" t="n">
+      <c r="C19" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="7">
-        <f>D19*E19</f>
+      <c r="D19" s="7">
+        <f>B19*C19</f>
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B20" s="29" t="inlineStr">
-        <is>
-          <t>Приманочные станции 2-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D20" s="30">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B20" s="28">
         <f>Данные!$C$20*Данные!$B$9</f>
         <v>62640</v>
       </c>
-      <c r="E20" s="30" t="n">
+      <c r="C20" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="7">
-        <f>D20*E20</f>
+      <c r="D20" s="7">
+        <f>B20*C20</f>
         <v>62640</v>
       </c>
     </row>
     <row r="21">
-      <c r="E21" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F21" s="12">
-        <f>SUM(F19:F20)</f>
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D21" s="12">
+        <f>SUM(D19:D20)</f>
         <v>62640</v>
       </c>
     </row>
@@ -1917,87 +1821,67 @@
       <c r="B23" s="16" t="n"/>
       <c r="C23" s="16" t="n"/>
       <c r="D23" s="16" t="n"/>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="16" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B24" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D24" s="28" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E24" s="28" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F24" s="28" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Pest Hunters</t>
-        </is>
-      </c>
-      <c r="B25" s="29" t="inlineStr">
-        <is>
-          <t>дезинсекция</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="30">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>Pest Hunters · дезинсекция</t>
+        </is>
+      </c>
+      <c r="B25" s="28">
         <f>Данные!$B$54</f>
         <v>70000</v>
       </c>
-      <c r="E25" s="30" t="n">
+      <c r="C25" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F25" s="7">
-        <f>D25*E25</f>
+      <c r="D25" s="7">
+        <f>B25*C25</f>
         <v>840000</v>
       </c>
     </row>
     <row r="26">
-      <c r="E26" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F26" s="12">
-        <f>SUM(F25:F25)</f>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D26" s="12">
+        <f>SUM(D25:D25)</f>
         <v>840000</v>
       </c>
     </row>
     <row r="27"/>
-    <row r="28" ht="28" customHeight="1">
+    <row r="28" ht="26" customHeight="1">
       <c r="A28" s="23" t="inlineStr">
         <is>
           <t>Зерноцид по ККЗ в нормах не заявлен, поэтому строка Зерноцида даёт ноль.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="26" customHeight="1">
       <c r="A29" s="23" t="inlineStr">
         <is>
           <t>Зарплата дератизаторов по объектам не делится — она на листе «Штат УКПФ».</t>
@@ -2006,9 +1890,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2020,15 +1904,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2064,21 +1946,21 @@
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>Штат УКПФ · материалы</t>
+          <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="26">
-        <f>F9+F10+F11</f>
+        <f>D9+D10+D11</f>
         <v>45447600</v>
       </c>
       <c r="C5" s="26">
-        <f>F12+F13</f>
+        <f>D12+D13</f>
         <v>34770000</v>
       </c>
       <c r="D5" s="26">
-        <f>F14+F15+F16+F17</f>
+        <f>D14+D15+D16+D17</f>
         <v>1240117.5</v>
       </c>
     </row>
@@ -2092,295 +1974,205 @@
       <c r="B7" s="16" t="n"/>
       <c r="C7" s="16" t="n"/>
       <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>Айыртау БП (БП-12, БП-13, БП-14) — полная замена, 180 ед.</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D9" s="30">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Айыртау БП (БП-12, БП-13, БП-14) — полная замена, 180 ед.</t>
+        </is>
+      </c>
+      <c r="B9" s="28">
         <f>Данные!$B$38</f>
         <v>618400</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="C9" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F9" s="8">
-        <f>D9*E9</f>
+      <c r="D9" s="8">
+        <f>B9*C9</f>
         <v>7420800</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>Многоэтажки, площадки Д и Г — полная замена, 166 ед.</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D10" s="30">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Многоэтажки, площадки Д и Г — полная замена, 166 ед.</t>
+        </is>
+      </c>
+      <c r="B10" s="28">
         <f>Данные!$B$40</f>
         <v>569800</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="C10" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F10" s="8">
-        <f>D10*E10</f>
+      <c r="D10" s="8">
+        <f>B10*C10</f>
         <v>6837600</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>Площадки А, Б, Е, Ж, В (рем. молод), В — полная замена, 793 ед.</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D11" s="30">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (рем. молод), В — полная замена, 793 ед.</t>
+        </is>
+      </c>
+      <c r="B11" s="28">
         <f>Данные!$B$42</f>
         <v>2599100</v>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="C11" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F11" s="8">
-        <f>D11*E11</f>
+      <c r="D11" s="8">
+        <f>B11*C11</f>
         <v>31189200</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Pest Hunters</t>
-        </is>
-      </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>122 объекта, март — ноябрь, оборудование подрядчика</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="30">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Pest Hunters · 122 объекта, март — ноябрь, оборудование подрядчика</t>
+        </is>
+      </c>
+      <c r="B12" s="28">
         <f>Данные!$B$55</f>
         <v>3172000</v>
       </c>
-      <c r="E12" s="30">
+      <c r="C12" s="28">
         <f>Данные!$B$61</f>
         <v>9</v>
       </c>
-      <c r="F12" s="8">
-        <f>D12*E12</f>
+      <c r="D12" s="8">
+        <f>B12*C12</f>
         <v>28548000</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Pest Hunters</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>122 объекта, декабрь — февраль, оборудование подрядчика</t>
-        </is>
-      </c>
-      <c r="C13" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="30">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Pest Hunters · 122 объекта, декабрь — февраль, оборудование подрядчика</t>
+        </is>
+      </c>
+      <c r="B13" s="28">
         <f>Данные!$B$56</f>
         <v>2074000</v>
       </c>
-      <c r="E13" s="30">
+      <c r="C13" s="28">
         <f>Данные!$B$62</f>
         <v>3</v>
       </c>
-      <c r="F13" s="8">
-        <f>D13*E13</f>
+      <c r="D13" s="8">
+        <f>B13*C13</f>
         <v>6222000</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>Клеевые станции 3-го контура, тёплый сезон</t>
-        </is>
-      </c>
-      <c r="C14" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D14" s="30">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
+        </is>
+      </c>
+      <c r="B14" s="28">
         <f>SUM(Данные!$D$23:$D$30)*Данные!$B$8</f>
         <v>42880</v>
       </c>
-      <c r="E14" s="30">
+      <c r="C14" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F14" s="8">
-        <f>D14*E14</f>
+      <c r="D14" s="8">
+        <f>B14*C14</f>
         <v>300160</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B15" s="29" t="inlineStr">
-        <is>
-          <t>Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
-        </is>
-      </c>
-      <c r="C15" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D15" s="30">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
+        </is>
+      </c>
+      <c r="B15" s="28">
         <f>SUM(Данные!$D$23:$D$30)*2*Данные!$B$8</f>
         <v>85760</v>
       </c>
-      <c r="E15" s="30">
+      <c r="C15" s="28">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
-      <c r="F15" s="8">
-        <f>D15*E15</f>
+      <c r="D15" s="8">
+        <f>B15*C15</f>
         <v>428800</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B16" s="29" t="inlineStr">
-        <is>
-          <t>Зерноцид, 2-й контур</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D16" s="30">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Зерноцид, 2-й контур</t>
+        </is>
+      </c>
+      <c r="B16" s="28">
         <f>SUM(Данные!$G$23:$G$30)*Данные!$B$6</f>
         <v>11100</v>
       </c>
-      <c r="E16" s="30">
+      <c r="C16" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F16" s="8">
-        <f>D16*E16</f>
+      <c r="D16" s="8">
+        <f>B16*C16</f>
         <v>77700</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B17" s="29" t="inlineStr">
-        <is>
-          <t>Pest Killer, брикеты</t>
-        </is>
-      </c>
-      <c r="C17" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D17" s="30">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Pest Killer, брикеты</t>
+        </is>
+      </c>
+      <c r="B17" s="28">
         <f>SUM(Данные!$F$23:$F$30)*Данные!$B$7</f>
         <v>61922.5</v>
       </c>
-      <c r="E17" s="30">
+      <c r="C17" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F17" s="8">
-        <f>D17*E17</f>
+      <c r="D17" s="8">
+        <f>B17*C17</f>
         <v>433457.5</v>
       </c>
     </row>
     <row r="18">
-      <c r="E18" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F18" s="12">
-        <f>SUM(F9:F17)</f>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D18" s="12">
+        <f>SUM(D9:D17)</f>
         <v>81457717.5</v>
       </c>
     </row>
@@ -2394,187 +2186,129 @@
       <c r="B20" s="16" t="n"/>
       <c r="C20" s="16" t="n"/>
       <c r="D20" s="16" t="n"/>
-      <c r="E20" s="16" t="n"/>
-      <c r="F20" s="16" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B21" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C21" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D21" s="28" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E21" s="28" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F21" s="28" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B22" s="29" t="inlineStr">
-        <is>
-          <t>Айыртау БП — частичная замена</t>
-        </is>
-      </c>
-      <c r="C22" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D22" s="30">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Айыртау БП — частичная замена</t>
+        </is>
+      </c>
+      <c r="B22" s="28">
         <f>Данные!$B$39</f>
         <v>478400</v>
       </c>
-      <c r="E22" s="30" t="n">
+      <c r="C22" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F22" s="7">
-        <f>D22*E22</f>
+      <c r="D22" s="7">
+        <f>B22*C22</f>
         <v>5740800</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B23" s="29" t="inlineStr">
-        <is>
-          <t>Многоэтажки Д и Г — частичная замена</t>
-        </is>
-      </c>
-      <c r="C23" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D23" s="30">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Многоэтажки Д и Г — частичная замена</t>
+        </is>
+      </c>
+      <c r="B23" s="28">
         <f>Данные!$B$41</f>
         <v>440700</v>
       </c>
-      <c r="E23" s="30" t="n">
+      <c r="C23" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F23" s="7">
-        <f>D23*E23</f>
+      <c r="D23" s="7">
+        <f>B23*C23</f>
         <v>5288400</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B24" s="29" t="inlineStr">
-        <is>
-          <t>Площадки А, Б, Е, Ж, В (РМ), В — частичная замена</t>
-        </is>
-      </c>
-      <c r="C24" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D24" s="30">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (РМ), В — частичная замена</t>
+        </is>
+      </c>
+      <c r="B24" s="28">
         <f>Данные!$B$43</f>
         <v>2010300</v>
       </c>
-      <c r="E24" s="30" t="n">
+      <c r="C24" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F24" s="7">
-        <f>D24*E24</f>
+      <c r="D24" s="7">
+        <f>B24*C24</f>
         <v>24123600</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Pest Hunters</t>
-        </is>
-      </c>
-      <c r="B25" s="29" t="inlineStr">
-        <is>
-          <t>122 объекта, март — ноябрь, оборудование заказчика</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="30">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>Pest Hunters · 122 объекта, март — ноябрь, оборудование заказчика</t>
+        </is>
+      </c>
+      <c r="B25" s="28">
         <f>Данные!$B$57</f>
         <v>2806000</v>
       </c>
-      <c r="E25" s="30">
+      <c r="C25" s="28">
         <f>Данные!$B$61</f>
         <v>9</v>
       </c>
-      <c r="F25" s="7">
-        <f>D25*E25</f>
+      <c r="D25" s="7">
+        <f>B25*C25</f>
         <v>25254000</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Pest Hunters</t>
-        </is>
-      </c>
-      <c r="B26" s="29" t="inlineStr">
-        <is>
-          <t>122 объекта, декабрь — февраль, оборудование заказчика</t>
-        </is>
-      </c>
-      <c r="C26" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="30">
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>Pest Hunters · 122 объекта, декабрь — февраль, оборудование заказчика</t>
+        </is>
+      </c>
+      <c r="B26" s="28">
         <f>Данные!$B$58</f>
         <v>1830000</v>
       </c>
-      <c r="E26" s="30">
+      <c r="C26" s="28">
         <f>Данные!$B$62</f>
         <v>3</v>
       </c>
-      <c r="F26" s="7">
-        <f>D26*E26</f>
+      <c r="D26" s="7">
+        <f>B26*C26</f>
         <v>5490000</v>
       </c>
     </row>
     <row r="27">
-      <c r="E27" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F27" s="12">
-        <f>SUM(F22:F26)</f>
+      <c r="C27" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D27" s="12">
+        <f>SUM(D22:D26)</f>
         <v>65896800</v>
       </c>
     </row>
@@ -2588,105 +2322,73 @@
       <c r="B29" s="16" t="n"/>
       <c r="C29" s="16" t="n"/>
       <c r="D29" s="16" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="16" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B30" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C30" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D30" s="28" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E30" s="28" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F30" s="28" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B31" s="29" t="inlineStr">
-        <is>
-          <t>Приманочные станции 1-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D31" s="30">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B31" s="28">
         <f>SUM(Данные!$B$23:$B$30)*Данные!$B$9</f>
         <v>347760</v>
       </c>
-      <c r="E31" s="30" t="n">
+      <c r="C31" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F31" s="7">
-        <f>D31*E31</f>
+      <c r="D31" s="7">
+        <f>B31*C31</f>
         <v>347760</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B32" s="29" t="inlineStr">
-        <is>
-          <t>Приманочные станции 2-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="C32" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D32" s="30">
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B32" s="28">
         <f>SUM(Данные!$C$23:$C$30)*Данные!$B$9</f>
         <v>2367360</v>
       </c>
-      <c r="E32" s="30" t="n">
+      <c r="C32" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F32" s="7">
-        <f>D32*E32</f>
+      <c r="D32" s="7">
+        <f>B32*C32</f>
         <v>2367360</v>
       </c>
     </row>
     <row r="33">
-      <c r="E33" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F33" s="12">
-        <f>SUM(F31:F32)</f>
+      <c r="C33" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D33" s="12">
+        <f>SUM(D31:D32)</f>
         <v>2715120</v>
       </c>
     </row>
@@ -2700,145 +2402,103 @@
       <c r="B35" s="16" t="n"/>
       <c r="C35" s="16" t="n"/>
       <c r="D35" s="16" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="16" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B36" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C36" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D36" s="28" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E36" s="28" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F36" s="28" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B37" s="29" t="inlineStr">
-        <is>
-          <t>Айыртау БП</t>
-        </is>
-      </c>
-      <c r="C37" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D37" s="30">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Айыртау БП</t>
+        </is>
+      </c>
+      <c r="B37" s="28">
         <f>Данные!$B$48</f>
         <v>720000</v>
       </c>
-      <c r="E37" s="30" t="n">
+      <c r="C37" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F37" s="7">
-        <f>D37*E37</f>
+      <c r="D37" s="7">
+        <f>B37*C37</f>
         <v>8640000</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B38" s="29" t="inlineStr">
-        <is>
-          <t>Многоэтажки Д и Г</t>
-        </is>
-      </c>
-      <c r="C38" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D38" s="30">
+      <c r="A38" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Многоэтажки Д и Г</t>
+        </is>
+      </c>
+      <c r="B38" s="28">
         <f>Данные!$B$49</f>
         <v>1080000</v>
       </c>
-      <c r="E38" s="30" t="n">
+      <c r="C38" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F38" s="7">
-        <f>D38*E38</f>
+      <c r="D38" s="7">
+        <f>B38*C38</f>
         <v>12960000</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B39" s="29" t="inlineStr">
-        <is>
-          <t>Площадки А, Б, Е, Ж, В (РМ), В</t>
-        </is>
-      </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D39" s="30">
+      <c r="A39" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (РМ), В</t>
+        </is>
+      </c>
+      <c r="B39" s="28">
         <f>Данные!$B$50</f>
         <v>3000000</v>
       </c>
-      <c r="E39" s="30" t="n">
+      <c r="C39" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F39" s="7">
-        <f>D39*E39</f>
+      <c r="D39" s="7">
+        <f>B39*C39</f>
         <v>36000000</v>
       </c>
     </row>
     <row r="40">
-      <c r="E40" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F40" s="12">
-        <f>SUM(F37:F39)</f>
+      <c r="C40" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D40" s="12">
+        <f>SUM(D37:D39)</f>
         <v>57600000</v>
       </c>
     </row>
     <row r="41"/>
-    <row r="42" ht="28" customHeight="1">
+    <row r="42" ht="26" customHeight="1">
       <c r="A42" s="23" t="inlineStr">
         <is>
           <t>Состав площадок у Indigo и в нашем расчёте описан по-разному: у них шесть напольных площадок плюс «В (рем. молод)», у нас восемь площадок по контурам. Сопоставлять построчно нельзя, только суммарно.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="28" customHeight="1">
+    <row r="43" ht="26" customHeight="1">
       <c r="A43" s="23" t="inlineStr">
         <is>
           <t>Разовая закупка приманочных станций 1-го и 2-го контура показана справочно и в годовой итог не входит.</t>
@@ -2847,9 +2507,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2861,15 +2521,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2905,21 +2563,21 @@
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>Штат УКПФ · материалы</t>
+          <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="26">
-        <f>F9</f>
+        <f>D9</f>
         <v>1514400</v>
       </c>
       <c r="C5" s="26">
-        <f>F10</f>
+        <f>D10</f>
         <v>0</v>
       </c>
       <c r="D5" s="26">
-        <f>F11+F12+F13+F14</f>
+        <f>D11+D12+D13+D14</f>
         <v>63317.5</v>
       </c>
     </row>
@@ -2933,212 +2591,148 @@
       <c r="B7" s="16" t="n"/>
       <c r="C7" s="16" t="n"/>
       <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>полная замена оборудования, 48 ед.</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D9" s="30">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · полная замена оборудования, 48 ед.</t>
+        </is>
+      </c>
+      <c r="B9" s="28">
         <f>Данные!$B$44</f>
         <v>126200</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="C9" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F9" s="8">
-        <f>D9*E9</f>
+      <c r="D9" s="8">
+        <f>B9*C9</f>
         <v>1514400</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>нет в КП</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D10" s="30" t="n">
+      <c r="B10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="C10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="8">
-        <f>D10*E10</f>
+      <c r="D10" s="8">
+        <f>B10*C10</f>
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>Клеевые станции 3-го контура, тёплый сезон</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D11" s="30">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
+        </is>
+      </c>
+      <c r="B11" s="28">
         <f>Данные!$D$21*Данные!$B$8</f>
         <v>1920</v>
       </c>
-      <c r="E11" s="30">
+      <c r="C11" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F11" s="8">
-        <f>D11*E11</f>
+      <c r="D11" s="8">
+        <f>B11*C11</f>
         <v>13440</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D12" s="30">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
+        </is>
+      </c>
+      <c r="B12" s="28">
         <f>Данные!$D$21*2*Данные!$B$8</f>
         <v>3840</v>
       </c>
-      <c r="E12" s="30">
+      <c r="C12" s="28">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
-      <c r="F12" s="8">
-        <f>D12*E12</f>
+      <c r="D12" s="8">
+        <f>B12*C12</f>
         <v>19200</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>Зерноцид, 2-й контур</t>
-        </is>
-      </c>
-      <c r="C13" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D13" s="30">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Зерноцид, 2-й контур</t>
+        </is>
+      </c>
+      <c r="B13" s="28">
         <f>Данные!$G$21*Данные!$B$6</f>
         <v>740</v>
       </c>
-      <c r="E13" s="30">
+      <c r="C13" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F13" s="8">
-        <f>D13*E13</f>
+      <c r="D13" s="8">
+        <f>B13*C13</f>
         <v>5180</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>Pest Killer, брикеты</t>
-        </is>
-      </c>
-      <c r="C14" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D14" s="30">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Pest Killer, брикеты</t>
+        </is>
+      </c>
+      <c r="B14" s="28">
         <f>Данные!$F$21*Данные!$B$7</f>
         <v>3642.5</v>
       </c>
-      <c r="E14" s="30">
+      <c r="C14" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F14" s="8">
-        <f>D14*E14</f>
+      <c r="D14" s="8">
+        <f>B14*C14</f>
         <v>25497.5</v>
       </c>
     </row>
     <row r="15">
-      <c r="E15" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F15" s="12">
-        <f>SUM(F9:F14)</f>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D15" s="12">
+        <f>SUM(D9:D14)</f>
         <v>1577717.5</v>
       </c>
     </row>
@@ -3152,77 +2746,55 @@
       <c r="B17" s="16" t="n"/>
       <c r="C17" s="16" t="n"/>
       <c r="D17" s="16" t="n"/>
-      <c r="E17" s="16" t="n"/>
-      <c r="F17" s="16" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C18" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D18" s="28" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E18" s="28" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F18" s="28" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B19" s="29" t="inlineStr">
-        <is>
-          <t>частичная замена оборудования</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D19" s="30">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · частичная замена оборудования</t>
+        </is>
+      </c>
+      <c r="B19" s="28">
         <f>Данные!$B$45</f>
         <v>106800</v>
       </c>
-      <c r="E19" s="30" t="n">
+      <c r="C19" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F19" s="7">
-        <f>D19*E19</f>
+      <c r="D19" s="7">
+        <f>B19*C19</f>
         <v>1281600</v>
       </c>
     </row>
     <row r="20">
-      <c r="E20" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F20" s="12">
-        <f>SUM(F19:F19)</f>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D20" s="12">
+        <f>SUM(D19:D19)</f>
         <v>1281600</v>
       </c>
     </row>
@@ -3236,105 +2808,73 @@
       <c r="B22" s="16" t="n"/>
       <c r="C22" s="16" t="n"/>
       <c r="D22" s="16" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="16" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B23" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C23" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D23" s="28" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E23" s="28" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F23" s="28" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B24" s="29" t="inlineStr">
-        <is>
-          <t>Приманочные станции 1-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="C24" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D24" s="30">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B24" s="28">
         <f>Данные!$B$21*Данные!$B$9</f>
         <v>38880</v>
       </c>
-      <c r="E24" s="30" t="n">
+      <c r="C24" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="7">
-        <f>D24*E24</f>
+      <c r="D24" s="7">
+        <f>B24*C24</f>
         <v>38880</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B25" s="29" t="inlineStr">
-        <is>
-          <t>Приманочные станции 2-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D25" s="30">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B25" s="28">
         <f>Данные!$C$21*Данные!$B$9</f>
         <v>73440</v>
       </c>
-      <c r="E25" s="30" t="n">
+      <c r="C25" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="7">
-        <f>D25*E25</f>
+      <c r="D25" s="7">
+        <f>B25*C25</f>
         <v>73440</v>
       </c>
     </row>
     <row r="26">
-      <c r="E26" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F26" s="12">
-        <f>SUM(F24:F25)</f>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D26" s="12">
+        <f>SUM(D24:D25)</f>
         <v>112320</v>
       </c>
     </row>
@@ -3348,82 +2888,60 @@
       <c r="B28" s="16" t="n"/>
       <c r="C28" s="16" t="n"/>
       <c r="D28" s="16" t="n"/>
-      <c r="E28" s="16" t="n"/>
-      <c r="F28" s="16" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B29" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C29" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D29" s="28" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E29" s="28" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F29" s="28" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B30" s="29" t="inlineStr">
-        <is>
-          <t>дезинсекция</t>
-        </is>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D30" s="30">
+      <c r="A30" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · дезинсекция</t>
+        </is>
+      </c>
+      <c r="B30" s="28">
         <f>Данные!$B$51</f>
         <v>100800</v>
       </c>
-      <c r="E30" s="30" t="n">
+      <c r="C30" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F30" s="7">
-        <f>D30*E30</f>
+      <c r="D30" s="7">
+        <f>B30*C30</f>
         <v>1209600</v>
       </c>
     </row>
     <row r="31">
-      <c r="E31" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F31" s="12">
-        <f>SUM(F30:F30)</f>
+      <c r="C31" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D31" s="12">
+        <f>SUM(D30:D30)</f>
         <v>1209600</v>
       </c>
     </row>
     <row r="32"/>
-    <row r="33" ht="28" customHeight="1">
+    <row r="33" ht="26" customHeight="1">
       <c r="A33" s="23" t="inlineStr">
         <is>
           <t>Нормы штата по инкубаторию: 18 точек 1-го контура, 34 второго, 12 клеевых третьего; 1 кг брикетов Pest Killer и 1 кг Зерноцида на обработку.</t>
@@ -3432,8 +2950,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3445,15 +2963,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3489,21 +3005,21 @@
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>Штат УКПФ · материалы</t>
+          <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="26">
-        <f>F9</f>
+        <f>D9</f>
         <v>1514400</v>
       </c>
       <c r="C5" s="26">
-        <f>F10</f>
+        <f>D10</f>
         <v>2160000</v>
       </c>
       <c r="D5" s="26">
-        <f>F11</f>
+        <f>D11</f>
         <v>0</v>
       </c>
     </row>
@@ -3517,128 +3033,90 @@
       <c r="B7" s="16" t="n"/>
       <c r="C7" s="16" t="n"/>
       <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>полная замена оборудования</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D9" s="30">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · полная замена оборудования</t>
+        </is>
+      </c>
+      <c r="B9" s="28">
         <f>Данные!$B$46</f>
         <v>126200</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="C9" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F9" s="8">
-        <f>D9*E9</f>
+      <c r="D9" s="8">
+        <f>B9*C9</f>
         <v>1514400</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Pest Hunters</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>договор №88 от 01.01.2026: дератизация и дезинсекция вместе</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="30">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Pest Hunters · договор №88 от 01.01.2026: дератизация и дезинсекция вместе</t>
+        </is>
+      </c>
+      <c r="B10" s="28">
         <f>Данные!$B$59</f>
         <v>180000</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="C10" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F10" s="8">
-        <f>D10*E10</f>
+      <c r="D10" s="8">
+        <f>B10*C10</f>
         <v>2160000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>нормы расхода по ЗПП не заданы</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D11" s="30" t="n">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · нормы расхода по ЗПП не заданы</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="C11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="8">
-        <f>D11*E11</f>
+      <c r="D11" s="8">
+        <f>B11*C11</f>
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="E12" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F12" s="12">
-        <f>SUM(F9:F11)</f>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D12" s="12">
+        <f>SUM(D9:D11)</f>
         <v>3674400</v>
       </c>
     </row>
@@ -3652,77 +3130,55 @@
       <c r="B14" s="16" t="n"/>
       <c r="C14" s="16" t="n"/>
       <c r="D14" s="16" t="n"/>
-      <c r="E14" s="16" t="n"/>
-      <c r="F14" s="16" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C15" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D15" s="28" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E15" s="28" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F15" s="28" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B16" s="29" t="inlineStr">
-        <is>
-          <t>частичная замена оборудования</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D16" s="30">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · частичная замена оборудования</t>
+        </is>
+      </c>
+      <c r="B16" s="28">
         <f>Данные!$B$47</f>
         <v>106800</v>
       </c>
-      <c r="E16" s="30" t="n">
+      <c r="C16" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F16" s="7">
-        <f>D16*E16</f>
+      <c r="D16" s="7">
+        <f>B16*C16</f>
         <v>1281600</v>
       </c>
     </row>
     <row r="17">
-      <c r="E17" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F17" s="12">
-        <f>SUM(F16:F16)</f>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D17" s="12">
+        <f>SUM(D16:D16)</f>
         <v>1281600</v>
       </c>
     </row>
@@ -3736,89 +3192,67 @@
       <c r="B19" s="16" t="n"/>
       <c r="C19" s="16" t="n"/>
       <c r="D19" s="16" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="16" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B20" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C20" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D20" s="28" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E20" s="28" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F20" s="28" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B21" s="29" t="inlineStr">
-        <is>
-          <t>дезинсекция</t>
-        </is>
-      </c>
-      <c r="C21" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D21" s="30">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · дезинсекция</t>
+        </is>
+      </c>
+      <c r="B21" s="28">
         <f>Данные!$B$52</f>
         <v>160800</v>
       </c>
-      <c r="E21" s="30" t="n">
+      <c r="C21" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="F21" s="7">
-        <f>D21*E21</f>
+      <c r="D21" s="7">
+        <f>B21*C21</f>
         <v>1929600</v>
       </c>
     </row>
     <row r="22">
-      <c r="E22" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F22" s="12">
-        <f>SUM(F21:F21)</f>
+      <c r="C22" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D22" s="12">
+        <f>SUM(D21:D21)</f>
         <v>1929600</v>
       </c>
     </row>
     <row r="23"/>
-    <row r="24" ht="28" customHeight="1">
+    <row r="24" ht="26" customHeight="1">
       <c r="A24" s="23" t="inlineStr">
         <is>
           <t>Строки не полностью сопоставимы: у Pest Hunters 180 000 ₸ включают и дератизацию, и дезинсекцию, у Indigo эти услуги разделены — 126 200 ₸ дератизация и 160 800 ₸ дезинсекция.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="26" customHeight="1">
       <c r="A25" s="23" t="inlineStr">
         <is>
           <t>По штату УКПФ нормы расхода на ЗПП не заданы, поэтому в расчёте ноль.</t>
@@ -3827,9 +3261,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3841,15 +3275,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3885,21 +3317,21 @@
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>Штат УКПФ · материалы</t>
+          <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="26">
-        <f>F9</f>
+        <f>D9</f>
         <v>0</v>
       </c>
       <c r="C5" s="26">
-        <f>F10</f>
+        <f>D10</f>
         <v>720000</v>
       </c>
       <c r="D5" s="26">
-        <f>F11</f>
+        <f>D11</f>
         <v>0</v>
       </c>
     </row>
@@ -3913,133 +3345,95 @@
       <c r="B7" s="16" t="n"/>
       <c r="C7" s="16" t="n"/>
       <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>нет в КП</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D9" s="30" t="n">
+      <c r="B9" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="C9" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="8">
-        <f>D9*E9</f>
+      <c r="D9" s="8">
+        <f>B9*C9</f>
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Pest Hunters</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>договор №921: дератизация и дезинсекция, выезд по рекламации за 2 рабочих дня</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="30">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Pest Hunters · договор №921: дератизация и дезинсекция, выезд по рекламации за 2 рабочих дня</t>
+        </is>
+      </c>
+      <c r="B10" s="28">
         <f>Данные!$B$60</f>
         <v>80000</v>
       </c>
-      <c r="E10" s="30">
+      <c r="C10" s="28">
         <f>Данные!$B$63</f>
         <v>9</v>
       </c>
-      <c r="F10" s="8">
-        <f>D10*E10</f>
+      <c r="D10" s="8">
+        <f>B10*C10</f>
         <v>720000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>нормы расхода по складу не заданы</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D11" s="30" t="n">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · нормы расхода по складу не заданы</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="C11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="8">
-        <f>D11*E11</f>
+      <c r="D11" s="8">
+        <f>B11*C11</f>
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="E12" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F12" s="12">
-        <f>SUM(F9:F11)</f>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D12" s="12">
+        <f>SUM(D9:D11)</f>
         <v>720000</v>
       </c>
     </row>
     <row r="13"/>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="26" customHeight="1">
       <c r="A14" s="23" t="inlineStr">
         <is>
           <t>С января по март договор не действует, поэтому в году девять оплачиваемых месяцев.</t>
@@ -4048,8 +3442,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4061,15 +3455,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4105,21 +3497,21 @@
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>Штат УКПФ · материалы</t>
+          <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="26">
-        <f>F9</f>
+        <f>D9</f>
         <v>0</v>
       </c>
       <c r="C5" s="26">
-        <f>F10</f>
+        <f>D10</f>
         <v>0</v>
       </c>
       <c r="D5" s="26">
-        <f>F11+F12+F13+F14</f>
+        <f>D11+D12+D13+D14</f>
         <v>204506.75</v>
       </c>
     </row>
@@ -4133,211 +3525,147 @@
       <c r="B7" s="16" t="n"/>
       <c r="C7" s="16" t="n"/>
       <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>нет в КП</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D9" s="30" t="n">
+      <c r="B9" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="C9" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="8">
-        <f>D9*E9</f>
+      <c r="D9" s="8">
+        <f>B9*C9</f>
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>нет в КП</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D10" s="30" t="n">
+      <c r="B10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="C10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="8">
-        <f>D10*E10</f>
+      <c r="D10" s="8">
+        <f>B10*C10</f>
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>Клеевые станции 3-го контура, тёплый сезон</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D11" s="30">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
+        </is>
+      </c>
+      <c r="B11" s="28">
         <f>Данные!$D$22*Данные!$B$8</f>
         <v>10080</v>
       </c>
-      <c r="E11" s="30">
+      <c r="C11" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F11" s="8">
-        <f>D11*E11</f>
+      <c r="D11" s="8">
+        <f>B11*C11</f>
         <v>70560</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D12" s="30">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
+        </is>
+      </c>
+      <c r="B12" s="28">
         <f>Данные!$D$22*2*Данные!$B$8</f>
         <v>20160</v>
       </c>
-      <c r="E12" s="30">
+      <c r="C12" s="28">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
-      <c r="F12" s="8">
-        <f>D12*E12</f>
+      <c r="D12" s="8">
+        <f>B12*C12</f>
         <v>100800</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>Зерноцид, 2-й контур</t>
-        </is>
-      </c>
-      <c r="C13" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D13" s="30">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Зерноцид, 2-й контур</t>
+        </is>
+      </c>
+      <c r="B13" s="28">
         <f>Данные!$G$22*Данные!$B$6</f>
         <v>0</v>
       </c>
-      <c r="E13" s="30">
+      <c r="C13" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F13" s="8">
-        <f>D13*E13</f>
+      <c r="D13" s="8">
+        <f>B13*C13</f>
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>Pest Killer, брикеты</t>
-        </is>
-      </c>
-      <c r="C14" s="21" t="n">
-        <v>8</v>
-      </c>
-      <c r="D14" s="30">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Pest Killer, брикеты</t>
+        </is>
+      </c>
+      <c r="B14" s="28">
         <f>Данные!$F$22*Данные!$B$7</f>
         <v>4735.25</v>
       </c>
-      <c r="E14" s="30">
+      <c r="C14" s="28">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
-      <c r="F14" s="8">
-        <f>D14*E14</f>
+      <c r="D14" s="8">
+        <f>B14*C14</f>
         <v>33146.75</v>
       </c>
     </row>
     <row r="15">
-      <c r="E15" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F15" s="12">
-        <f>SUM(F9:F14)</f>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D15" s="12">
+        <f>SUM(D9:D14)</f>
         <v>204506.75</v>
       </c>
     </row>
@@ -4351,117 +3679,85 @@
       <c r="B17" s="16" t="n"/>
       <c r="C17" s="16" t="n"/>
       <c r="D17" s="16" t="n"/>
-      <c r="E17" s="16" t="n"/>
-      <c r="F17" s="16" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>Вариант</t>
-        </is>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>Что входит</t>
-        </is>
-      </c>
-      <c r="C18" s="28" t="inlineStr">
-        <is>
-          <t>Обходов в месяц</t>
-        </is>
-      </c>
-      <c r="D18" s="28" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="E18" s="28" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="F18" s="28" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B19" s="29" t="inlineStr">
-        <is>
-          <t>Приманочные станции 1-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D19" s="30">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B19" s="28">
         <f>Данные!$B$22*Данные!$B$9</f>
         <v>0</v>
       </c>
-      <c r="E19" s="30" t="n">
+      <c r="C19" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="7">
-        <f>D19*E19</f>
+      <c r="D19" s="7">
+        <f>B19*C19</f>
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Штат УКПФ</t>
-        </is>
-      </c>
-      <c r="B20" s="29" t="inlineStr">
-        <is>
-          <t>Приманочные станции 2-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D20" s="30">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B20" s="28">
         <f>Данные!$C$22*Данные!$B$9</f>
         <v>84240</v>
       </c>
-      <c r="E20" s="30" t="n">
+      <c r="C20" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="7">
-        <f>D20*E20</f>
+      <c r="D20" s="7">
+        <f>B20*C20</f>
         <v>84240</v>
       </c>
     </row>
     <row r="21">
-      <c r="E21" s="31" t="inlineStr">
-        <is>
-          <t>Итого блока</t>
-        </is>
-      </c>
-      <c r="F21" s="12">
-        <f>SUM(F19:F20)</f>
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>Итого</t>
+        </is>
+      </c>
+      <c r="D21" s="12">
+        <f>SUM(D19:D20)</f>
         <v>84240</v>
       </c>
     </row>
     <row r="22"/>
-    <row r="23" ht="28" customHeight="1">
+    <row r="23" ht="26" customHeight="1">
       <c r="A23" s="23" t="inlineStr">
         <is>
           <t>Клеевые станции по корпусам: Б — 11, Ж — 5, Е — 6, В — 6, В (РМ) — 6, Д — 3, Г — 3, БП-12 — 6, БП-13 — 6, БП-14 — 6, А — 5. Приманочные: 4, 2, 3, 3, 3, 4, 3, 5, 5, 5, 2.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
+    <row r="24" ht="26" customHeight="1">
       <c r="A24" s="23" t="inlineStr">
         <is>
           <t>Норма 1,3 кг брикетов Pest Killer по АБК — приблизительная оценка, требует подтверждения. Зерноцид по АБК не заявлен.</t>
@@ -4470,9 +3766,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4587,7 +3883,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Зарплата за год</t>
         </is>
@@ -4618,47 +3914,47 @@
       <c r="I11" s="16" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B12" s="34" t="inlineStr">
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>Клеевых 3-го к., шт/мес лето</t>
         </is>
       </c>
-      <c r="C12" s="34" t="inlineStr">
+      <c r="C12" s="32" t="inlineStr">
         <is>
           <t>Клеевых 3-го к., шт/мес зима</t>
         </is>
       </c>
-      <c r="D12" s="34" t="inlineStr">
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>Клеевые за год, ₸</t>
         </is>
       </c>
-      <c r="E12" s="34" t="inlineStr">
+      <c r="E12" s="32" t="inlineStr">
         <is>
           <t>Зерноцид, кг/мес</t>
         </is>
       </c>
-      <c r="F12" s="34" t="inlineStr">
+      <c r="F12" s="32" t="inlineStr">
         <is>
           <t>Зерноцид за год, ₸</t>
         </is>
       </c>
-      <c r="G12" s="34" t="inlineStr">
+      <c r="G12" s="32" t="inlineStr">
         <is>
           <t>Pest Killer, кг/мес</t>
         </is>
       </c>
-      <c r="H12" s="34" t="inlineStr">
+      <c r="H12" s="32" t="inlineStr">
         <is>
           <t>Pest Killer за год, ₸</t>
         </is>
       </c>
-      <c r="I12" s="34" t="inlineStr">
+      <c r="I12" s="32" t="inlineStr">
         <is>
           <t>Материалы за год, ₸</t>
         </is>
@@ -4670,11 +3966,11 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B13" s="35">
+      <c r="B13" s="33">
         <f>Данные!$D$20</f>
         <v>0</v>
       </c>
-      <c r="C13" s="35">
+      <c r="C13" s="33">
         <f>Данные!$D$20*2</f>
         <v>0</v>
       </c>
@@ -4709,11 +4005,11 @@
           <t>Бройлерные площадки · 8 шт</t>
         </is>
       </c>
-      <c r="B14" s="35">
+      <c r="B14" s="33">
         <f>SUM(Данные!$D$23:$D$30)</f>
         <v>268</v>
       </c>
-      <c r="C14" s="35">
+      <c r="C14" s="33">
         <f>SUM(Данные!$D$23:$D$30)*2</f>
         <v>536</v>
       </c>
@@ -4748,11 +4044,11 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B15" s="35">
+      <c r="B15" s="33">
         <f>Данные!$D$21</f>
         <v>12</v>
       </c>
-      <c r="C15" s="35">
+      <c r="C15" s="33">
         <f>Данные!$D$21*2</f>
         <v>24</v>
       </c>
@@ -4787,11 +4083,11 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B16" s="35">
+      <c r="B16" s="33">
         <f>Данные!$D$22</f>
         <v>63</v>
       </c>
-      <c r="C16" s="35">
+      <c r="C16" s="33">
         <f>Данные!$D$22*2</f>
         <v>126</v>
       </c>
@@ -4844,8 +4140,8 @@
           <t>МАТЕРИАЛЫ ЗА ГОД, ИТОГО</t>
         </is>
       </c>
-      <c r="B18" s="37" t="n"/>
-      <c r="C18" s="37" t="n"/>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
       <c r="D18" s="12">
         <f>SUM(D13:D17)</f>
         <v>932960</v>
@@ -4885,32 +4181,32 @@
       <c r="F20" s="16" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B21" s="28" t="inlineStr">
+      <c r="B21" s="38" t="inlineStr">
         <is>
           <t>1-й контур, шт</t>
         </is>
       </c>
-      <c r="C21" s="28" t="inlineStr">
+      <c r="C21" s="38" t="inlineStr">
         <is>
           <t>2-й контур, шт</t>
         </is>
       </c>
-      <c r="D21" s="28" t="inlineStr">
+      <c r="D21" s="38" t="inlineStr">
         <is>
           <t>Всего, шт</t>
         </is>
       </c>
-      <c r="E21" s="28" t="inlineStr">
+      <c r="E21" s="38" t="inlineStr">
         <is>
           <t>Цена, ₸/шт</t>
         </is>
       </c>
-      <c r="F21" s="28" t="inlineStr">
+      <c r="F21" s="38" t="inlineStr">
         <is>
           <t>Разово, ₸</t>
         </is>
@@ -4922,19 +4218,19 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B22" s="35">
+      <c r="B22" s="33">
         <f>Данные!$B$20</f>
         <v>0</v>
       </c>
-      <c r="C22" s="35">
+      <c r="C22" s="33">
         <f>Данные!$C$20</f>
         <v>29</v>
       </c>
-      <c r="D22" s="35">
+      <c r="D22" s="33">
         <f>B22+C22</f>
         <v>29</v>
       </c>
-      <c r="E22" s="30">
+      <c r="E22" s="28">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4949,19 +4245,19 @@
           <t>Бройлерные площадки · 8 шт</t>
         </is>
       </c>
-      <c r="B23" s="35">
+      <c r="B23" s="33">
         <f>SUM(Данные!$B$23:$B$30)</f>
         <v>161</v>
       </c>
-      <c r="C23" s="35">
+      <c r="C23" s="33">
         <f>SUM(Данные!$C$23:$C$30)</f>
         <v>1096</v>
       </c>
-      <c r="D23" s="35">
+      <c r="D23" s="33">
         <f>B23+C23</f>
         <v>1257</v>
       </c>
-      <c r="E23" s="30">
+      <c r="E23" s="28">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4976,19 +4272,19 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B24" s="35">
+      <c r="B24" s="33">
         <f>Данные!$B$21</f>
         <v>18</v>
       </c>
-      <c r="C24" s="35">
+      <c r="C24" s="33">
         <f>Данные!$C$21</f>
         <v>34</v>
       </c>
-      <c r="D24" s="35">
+      <c r="D24" s="33">
         <f>B24+C24</f>
         <v>52</v>
       </c>
-      <c r="E24" s="30">
+      <c r="E24" s="28">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -5003,19 +4299,19 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B25" s="35">
+      <c r="B25" s="33">
         <f>Данные!$B$22</f>
         <v>0</v>
       </c>
-      <c r="C25" s="35">
+      <c r="C25" s="33">
         <f>Данные!$C$22</f>
         <v>39</v>
       </c>
-      <c r="D25" s="35">
+      <c r="D25" s="33">
         <f>B25+C25</f>
         <v>39</v>
       </c>
-      <c r="E25" s="30">
+      <c r="E25" s="28">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -5042,7 +4338,7 @@
         <f>SUM(D22:D25)</f>
         <v>1377</v>
       </c>
-      <c r="E26" s="37" t="n"/>
+      <c r="E26" s="35" t="n"/>
       <c r="F26" s="12">
         <f>SUM(F22:F25)</f>
         <v>2974320</v>
@@ -5062,32 +4358,32 @@
       <c r="F28" s="16" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="33" t="inlineStr">
+      <c r="A29" s="31" t="inlineStr">
         <is>
           <t>Численность, чел.</t>
         </is>
       </c>
-      <c r="B29" s="34" t="inlineStr">
+      <c r="B29" s="32" t="inlineStr">
         <is>
           <t>ЗП в месяц, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="C29" s="34" t="inlineStr">
+      <c r="C29" s="32" t="inlineStr">
         <is>
           <t>ЗП за год, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="D29" s="34" t="inlineStr">
+      <c r="D29" s="32" t="inlineStr">
         <is>
           <t>Материалы за год, ₸</t>
         </is>
       </c>
-      <c r="E29" s="34" t="inlineStr">
+      <c r="E29" s="32" t="inlineStr">
         <is>
           <t>Итого за год, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="F29" s="34" t="inlineStr">
+      <c r="F29" s="32" t="inlineStr">
         <is>
           <t>Итого за год, ₸ · оклад 350 000</t>
         </is>
@@ -5645,42 +4941,42 @@
       <c r="H18" s="16" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="33" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B19" s="34" t="inlineStr">
+      <c r="B19" s="32" t="inlineStr">
         <is>
           <t>1-й контур, шт</t>
         </is>
       </c>
-      <c r="C19" s="34" t="inlineStr">
+      <c r="C19" s="32" t="inlineStr">
         <is>
           <t>2-й контур, шт</t>
         </is>
       </c>
-      <c r="D19" s="34" t="inlineStr">
+      <c r="D19" s="32" t="inlineStr">
         <is>
           <t>3-й контур, шт</t>
         </is>
       </c>
-      <c r="E19" s="34" t="inlineStr">
+      <c r="E19" s="32" t="inlineStr">
         <is>
           <t>Всего точек, шт</t>
         </is>
       </c>
-      <c r="F19" s="34" t="inlineStr">
+      <c r="F19" s="32" t="inlineStr">
         <is>
           <t>Pest Killer, кг</t>
         </is>
       </c>
-      <c r="G19" s="34" t="inlineStr">
+      <c r="G19" s="32" t="inlineStr">
         <is>
           <t>Зерноцид, кг</t>
         </is>
       </c>
-      <c r="H19" s="34" t="inlineStr">
+      <c r="H19" s="32" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
@@ -6057,7 +5353,7 @@
         <f>SUM(G20:G32)</f>
         <v>16</v>
       </c>
-      <c r="H33" s="37" t="n"/>
+      <c r="H33" s="35" t="n"/>
     </row>
     <row r="34"/>
     <row r="35">

</xml_diff>

<commit_message>
Spell out the in-house cost in full on the lead sheet
New block lists headcount, the per-person salary, the payroll it produces,
each material with quantity, unit and unit price, the running total, the
one-off bait station purchase by contour and the first-year total. Payroll
and bottles are separate rows in the matrix rather than one merged line,
so every figure states what it covers and for how many people.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLozcDkCvYTXvP2yAkyMFB
</commit_message>
<xml_diff>
--- a/reports/УКПФ_дератизация_сравнение_КП.xlsx
+++ b/reports/УКПФ_дератизация_сравнение_КП.xlsx
@@ -213,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -245,17 +245,27 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -279,14 +289,7 @@
     </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -668,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -690,7 +693,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Все суммы в тенге. Только дератизация: дезинсекция у подрядчиков идёт отдельно. Цены Indigo включают НДС, цены Pest Hunters — без НДС.</t>
+          <t>Все суммы в тенге. Только дератизация: дезинсекция у подрядчиков идёт отдельно. Цены Indigo включают НДС, цены Pest Hunters — без НДС. Колонка «Штат УКПФ» — материалы по объектам; фонд оплаты труда идёт отдельной строкой ниже, его величина зависит от численности, заданной на листе «Данные».</t>
         </is>
       </c>
     </row>
@@ -718,7 +721,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="44" t="n"/>
+      <c r="A5" s="45" t="n"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
           <t>в месяц</t>
@@ -831,7 +834,7 @@
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="E8" s="45" t="n"/>
+      <c r="E8" s="46" t="n"/>
       <c r="F8" s="7">
         <f>G8/12</f>
         <v>5276.458333</v>
@@ -868,7 +871,7 @@
           <t>нормы не заданы</t>
         </is>
       </c>
-      <c r="G9" s="45" t="n"/>
+      <c r="G9" s="46" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -881,7 +884,7 @@
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="C10" s="45" t="n"/>
+      <c r="C10" s="46" t="n"/>
       <c r="D10" s="7">
         <f>E10/12</f>
         <v>60000</v>
@@ -895,7 +898,7 @@
           <t>нормы не заданы</t>
         </is>
       </c>
-      <c r="G10" s="45" t="n"/>
+      <c r="G10" s="46" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -908,13 +911,13 @@
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="C11" s="45" t="n"/>
+      <c r="C11" s="46" t="n"/>
       <c r="D11" s="9" t="inlineStr">
         <is>
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="E11" s="45" t="n"/>
+      <c r="E11" s="46" t="n"/>
       <c r="F11" s="7">
         <f>G11/12</f>
         <v>17042.22917</v>
@@ -958,7 +961,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Штат УКПФ: зарплата и бутылки</t>
+          <t>Фонд оплаты труда дератизаторов</t>
         </is>
       </c>
       <c r="B13" s="10" t="n"/>
@@ -967,543 +970,806 @@
       <c r="E13" s="10" t="n"/>
       <c r="F13" s="7">
         <f>G13/12</f>
-        <v>1035538.667</v>
+        <v>1033952</v>
       </c>
       <c r="G13" s="7">
-        <f>Данные!$B$14*Данные!$B$12*12+Данные!$B$11*Данные!$B$10*Данные!$B$15</f>
-        <v>12426464</v>
+        <f>Данные!$B$14*Данные!$B$12*12</f>
+        <v>12407424</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Бутылки</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="7">
+        <f>G14/12</f>
+        <v>1586.666667</v>
+      </c>
+      <c r="G14" s="7">
+        <f>Данные!$B$11*Данные!$B$10*Данные!$B$15</f>
+        <v>19040</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>ВСЕГО ЗА ГОД</t>
         </is>
       </c>
-      <c r="B14" s="14">
-        <f>C14/12</f>
+      <c r="B15" s="14">
+        <f>C15/12</f>
         <v>4136300</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C15" s="14">
         <f>C12</f>
         <v>49635600</v>
       </c>
-      <c r="D14" s="14">
-        <f>E14/12</f>
+      <c r="D15" s="14">
+        <f>E15/12</f>
         <v>3212500</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E15" s="14">
         <f>E12</f>
         <v>38550000</v>
       </c>
-      <c r="F14" s="14">
-        <f>G14/12</f>
+      <c r="F15" s="14">
+        <f>G15/12</f>
         <v>1163325.271</v>
       </c>
-      <c r="G14" s="14">
-        <f>G12+G13</f>
+      <c r="G15" s="14">
+        <f>G12+G13+G14</f>
         <v>13959903.25</v>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>РАЗНИЦА С СОБСТВЕННЫМ ШТАТОМ</t>
         </is>
       </c>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="16" t="n"/>
-      <c r="D16" s="16" t="n"/>
-      <c r="E16" s="16" t="n"/>
-      <c r="F16" s="16" t="n"/>
-      <c r="G16" s="16" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="n"/>
+      <c r="G17" s="16" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>в месяц</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>за год</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>во сколько раз</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions дороже штата</t>
-        </is>
-      </c>
-      <c r="B18" s="7">
-        <f>C18/12</f>
-        <v>2972974.729</v>
-      </c>
-      <c r="C18" s="8">
-        <f>C14-G14</f>
-        <v>35675696.75</v>
-      </c>
-      <c r="D18" s="46">
-        <f>IF(G14=0,0,C14/G14)</f>
-        <v>3.555583381</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Pest Hunters дороже штата</t>
+          <t>Indigo Solutions дороже штата</t>
         </is>
       </c>
       <c r="B19" s="7">
         <f>C19/12</f>
+        <v>2972974.729</v>
+      </c>
+      <c r="C19" s="8">
+        <f>C15-G15</f>
+        <v>35675696.75</v>
+      </c>
+      <c r="D19" s="47">
+        <f>IF(G15=0,0,C15/G15)</f>
+        <v>3.555583381</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Pest Hunters дороже штата</t>
+        </is>
+      </c>
+      <c r="B20" s="7">
+        <f>C20/12</f>
         <v>2049174.729</v>
       </c>
-      <c r="C19" s="8">
-        <f>E14-G14</f>
+      <c r="C20" s="8">
+        <f>E15-G15</f>
         <v>24590096.75</v>
       </c>
-      <c r="D19" s="46">
-        <f>IF(G14=0,0,E14/G14)</f>
+      <c r="D20" s="47">
+        <f>IF(G15=0,0,E15/G15)</f>
         <v>2.761480457</v>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>ШТАТ УКПФ · ИЗ ЧЕГО СКЛАДЫВАЕТСЯ</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="n"/>
-      <c r="C21" s="16" t="n"/>
-      <c r="D21" s="16" t="n"/>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="16" t="n"/>
-      <c r="G21" s="16" t="n"/>
-    </row>
+    <row r="21"/>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>ШТАТ УКПФ · ПОЛНАЯ РАСШИФРОВКА</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="16" t="n"/>
+      <c r="G22" s="16" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Статья</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>в месяц</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>за год</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>Количество</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>Ед. изм.</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>Цена за ед., ₸</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="F23" s="20" t="inlineStr">
+        <is>
+          <t>за год, ₸</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Численность штата</t>
+        </is>
+      </c>
+      <c r="B24" s="7">
+        <f>Данные!$B$14</f>
+        <v>4</v>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>чел.</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Оклад одного дератизатора</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>₸/мес</t>
+        </is>
+      </c>
+      <c r="D25" s="7">
+        <f>Данные!$B$12</f>
+        <v>258488</v>
+      </c>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Фонд оплаты труда</t>
         </is>
       </c>
-      <c r="B23" s="7">
-        <f>C23/12</f>
+      <c r="B26" s="7">
+        <f>Данные!$B$14</f>
+        <v>4</v>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>чел.</t>
+        </is>
+      </c>
+      <c r="D26" s="7">
+        <f>Данные!$B$12</f>
+        <v>258488</v>
+      </c>
+      <c r="E26" s="7">
+        <f>Данные!$B$14*Данные!$B$12</f>
         <v>1033952</v>
       </c>
-      <c r="C23" s="8">
+      <c r="F26" s="8">
         <f>Данные!$B$14*Данные!$B$12*12</f>
         <v>12407424</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Клеевые станции 3-го контура</t>
-        </is>
-      </c>
-      <c r="B24" s="7">
-        <f>C24/12</f>
-        <v>77746.66667</v>
-      </c>
-      <c r="C24" s="8">
-        <f>'Штат УКПФ'!D18</f>
-        <v>932960</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Зерноцид</t>
-        </is>
-      </c>
-      <c r="B25" s="7">
-        <f>C25/12</f>
-        <v>6906.666667</v>
-      </c>
-      <c r="C25" s="8">
-        <f>'Штат УКПФ'!F18</f>
-        <v>82880</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Pest Killer, брикеты</t>
-        </is>
-      </c>
-      <c r="B26" s="7">
-        <f>C26/12</f>
-        <v>43133.27083</v>
-      </c>
-      <c r="C26" s="8">
-        <f>'Штат УКПФ'!H18</f>
-        <v>517599.25</v>
-      </c>
-    </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Бутылки</t>
+          <t>Клеевые станции 3-го контура · апрель — октябрь</t>
         </is>
       </c>
       <c r="B27" s="7">
-        <f>C27/12</f>
-        <v>1586.666667</v>
-      </c>
-      <c r="C27" s="8">
+        <f>Данные!$D$33</f>
+        <v>343</v>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>шт/мес</t>
+        </is>
+      </c>
+      <c r="D27" s="7">
+        <f>Данные!$B$8</f>
+        <v>160</v>
+      </c>
+      <c r="E27" s="7">
+        <f>Данные!$D$33*Данные!$B$8</f>
+        <v>54880</v>
+      </c>
+      <c r="F27" s="8">
+        <f>Данные!$D$33*Данные!$B$8*Данные!$B$15</f>
+        <v>384160</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Клеевые станции 3-го контура · ноябрь — март, объём вдвое</t>
+        </is>
+      </c>
+      <c r="B28" s="7">
+        <f>Данные!$D$33*2</f>
+        <v>686</v>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>шт/мес</t>
+        </is>
+      </c>
+      <c r="D28" s="7">
+        <f>Данные!$B$8</f>
+        <v>160</v>
+      </c>
+      <c r="E28" s="7">
+        <f>Данные!$D$33*2*Данные!$B$8</f>
+        <v>109760</v>
+      </c>
+      <c r="F28" s="8">
+        <f>Данные!$D$33*2*Данные!$B$8*Данные!$B$16</f>
+        <v>548800</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Зерноцид · 2-й контур, тёплый сезон</t>
+        </is>
+      </c>
+      <c r="B29" s="7">
+        <f>Данные!$G$33</f>
+        <v>16</v>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>кг/мес</t>
+        </is>
+      </c>
+      <c r="D29" s="7">
+        <f>Данные!$B$6</f>
+        <v>740</v>
+      </c>
+      <c r="E29" s="7">
+        <f>Данные!$G$33*Данные!$B$6</f>
+        <v>11840</v>
+      </c>
+      <c r="F29" s="8">
+        <f>Данные!$G$33*Данные!$B$6*Данные!$B$15</f>
+        <v>82880</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Pest Killer, брикеты · тёплый сезон</t>
+        </is>
+      </c>
+      <c r="B30" s="7">
+        <f>Данные!$F$33</f>
+        <v>20.3</v>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>кг/мес</t>
+        </is>
+      </c>
+      <c r="D30" s="7">
+        <f>Данные!$B$7</f>
+        <v>3642.5</v>
+      </c>
+      <c r="E30" s="7">
+        <f>Данные!$F$33*Данные!$B$7</f>
+        <v>73942.75</v>
+      </c>
+      <c r="F30" s="8">
+        <f>Данные!$F$33*Данные!$B$7*Данные!$B$15</f>
+        <v>517599.25</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Бутылки · тёплый сезон</t>
+        </is>
+      </c>
+      <c r="B31" s="7">
+        <f>Данные!$B$11</f>
+        <v>40</v>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>шт/мес</t>
+        </is>
+      </c>
+      <c r="D31" s="7">
+        <f>Данные!$B$10</f>
+        <v>68</v>
+      </c>
+      <c r="E31" s="7">
+        <f>Данные!$B$11*Данные!$B$10</f>
+        <v>2720</v>
+      </c>
+      <c r="F31" s="8">
         <f>Данные!$B$11*Данные!$B$10*Данные!$B$15</f>
         <v>19040</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>ИТОГО ШТАТ</t>
-        </is>
-      </c>
-      <c r="B28" s="12">
-        <f>C28/12</f>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>ИТОГО ТЕКУЩИЕ РАСХОДЫ ШТАТА</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="14">
+        <f>F32/12</f>
         <v>1163325.271</v>
       </c>
-      <c r="C28" s="12">
-        <f>SUM(C23:C27)</f>
+      <c r="F32" s="14">
+        <f>F26+F27+F28+F29+F30+F31</f>
         <v>13959903.25</v>
       </c>
-    </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>СКИДКИ INDIGO ИЗ КП ОТ 19.08.2026</t>
-        </is>
-      </c>
-      <c r="B30" s="16" t="n"/>
-      <c r="C30" s="16" t="n"/>
-      <c r="D30" s="16" t="n"/>
-      <c r="E30" s="16" t="n"/>
-      <c r="F30" s="16" t="n"/>
-      <c r="G30" s="16" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="17" t="inlineStr">
-        <is>
-          <t>Условие</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>в месяц</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>за год</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Ставка</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>Цена КП без скидок</t>
-        </is>
-      </c>
-      <c r="B32" s="7">
-        <f>C32/12</f>
-        <v>4136300</v>
-      </c>
-      <c r="C32" s="8">
-        <f>C14</f>
-        <v>49635600</v>
-      </c>
-      <c r="D32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
+          <t>Приманочные станции 1-го контура · разовая закупка</t>
+        </is>
+      </c>
+      <c r="B33" s="7">
+        <f>Данные!$B$33</f>
+        <v>179</v>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D33" s="7">
+        <f>Данные!$B$9</f>
+        <v>2160</v>
+      </c>
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="8">
+        <f>Данные!$B$33*Данные!$B$9</f>
+        <v>386640</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Приманочные станции 2-го контура · разовая закупка</t>
+        </is>
+      </c>
+      <c r="B34" s="7">
+        <f>Данные!$C$33</f>
+        <v>1198</v>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D34" s="7">
+        <f>Данные!$B$9</f>
+        <v>2160</v>
+      </c>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="8">
+        <f>Данные!$C$33*Данные!$B$9</f>
+        <v>2587680</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>ИТОГО РАЗОВАЯ ЗАКУПКА ОБОРУДОВАНИЯ</t>
+        </is>
+      </c>
+      <c r="B35" s="12">
+        <f>Данные!$B$33+Данные!$C$33</f>
+        <v>1377</v>
+      </c>
+      <c r="C35" s="23" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="22" t="n"/>
+      <c r="F35" s="12">
+        <f>F33+F34</f>
+        <v>2974320</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>ИТОГО ПЕРВЫЙ ГОД · с разовой закупкой</t>
+        </is>
+      </c>
+      <c r="B36" s="22" t="n"/>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="22" t="n"/>
+      <c r="E36" s="22" t="n"/>
+      <c r="F36" s="14">
+        <f>F32+F35</f>
+        <v>16934223.25</v>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>Материалы от численности не зависят: норма ядов и станций привязана к точкам, а не к людям. Каждый дополнительный дератизатор добавляет только фонд оплаты труда.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>СКИДКИ INDIGO ИЗ КП ОТ 19.08.2026</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="n"/>
+      <c r="C39" s="16" t="n"/>
+      <c r="D39" s="16" t="n"/>
+      <c r="E39" s="16" t="n"/>
+      <c r="F39" s="16" t="n"/>
+      <c r="G39" s="16" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Условие</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>в месяц</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>за год</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Ставка</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Цена КП без скидок</t>
+        </is>
+      </c>
+      <c r="B41" s="7">
+        <f>C41/12</f>
+        <v>4136300</v>
+      </c>
+      <c r="C41" s="8">
+        <f>C15</f>
+        <v>49635600</v>
+      </c>
+      <c r="D41" s="10" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
           <t>Вся территория фабрики</t>
         </is>
       </c>
-      <c r="B33" s="7">
-        <f>C33/12</f>
+      <c r="B42" s="7">
+        <f>C42/12</f>
         <v>3515855</v>
       </c>
-      <c r="C33" s="8">
-        <f>C14*(1-Данные!$B$64)</f>
+      <c r="C42" s="8">
+        <f>C15*(1-Данные!$B$64)</f>
         <v>42190260</v>
       </c>
-      <c r="D33" s="19">
+      <c r="D42" s="25">
         <f>Данные!$B$64</f>
         <v>0.15</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Вся территория + 100 % предоплата</t>
         </is>
       </c>
-      <c r="B34" s="7">
-        <f>C34/12</f>
+      <c r="B43" s="7">
+        <f>C43/12</f>
         <v>2988476.75</v>
       </c>
-      <c r="C34" s="8">
-        <f>C14*(1-Данные!$B$64)*(1-Данные!$B$65)</f>
+      <c r="C43" s="8">
+        <f>C15*(1-Данные!$B$64)*(1-Данные!$B$65)</f>
         <v>35861721</v>
       </c>
-      <c r="D34" s="19">
+      <c r="D43" s="25">
         <f>Данные!$B$65</f>
         <v>0.15</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>Вся территория + предоплата + неплательщик НДС</t>
         </is>
       </c>
-      <c r="B35" s="7">
-        <f>C35/12</f>
+      <c r="B44" s="7">
+        <f>C44/12</f>
         <v>2510320.47</v>
       </c>
-      <c r="C35" s="8">
-        <f>C14*(1-Данные!$B$64)*(1-Данные!$B$65)*(1-Данные!$B$66)</f>
+      <c r="C44" s="8">
+        <f>C15*(1-Данные!$B$64)*(1-Данные!$B$65)*(1-Данные!$B$66)</f>
         <v>30123845.64</v>
       </c>
-      <c r="D35" s="19">
+      <c r="D44" s="25">
         <f>Данные!$B$66</f>
         <v>0.16</v>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>ПЕРИОДИЧНОСТЬ ОБХОДОВ</t>
         </is>
       </c>
-      <c r="B37" s="16" t="n"/>
-      <c r="C37" s="16" t="n"/>
-      <c r="D37" s="16" t="n"/>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="16" t="n"/>
-      <c r="G37" s="16" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+      <c r="B46" s="16" t="n"/>
+      <c r="C46" s="16" t="n"/>
+      <c r="D46" s="16" t="n"/>
+      <c r="E46" s="16" t="n"/>
+      <c r="F46" s="16" t="n"/>
+      <c r="G46" s="16" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="inlineStr">
         <is>
           <t>Вариант</t>
         </is>
       </c>
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B47" s="26" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="C38" s="20" t="inlineStr">
+      <c r="C47" s="26" t="inlineStr">
         <is>
           <t>Обходов в месяц</t>
         </is>
       </c>
-      <c r="D38" s="20" t="inlineStr">
+      <c r="D47" s="26" t="inlineStr">
         <is>
           <t>Что зафиксировано в документах</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>все объекты</t>
         </is>
       </c>
-      <c r="C39" s="21" t="inlineStr">
+      <c r="C48" s="21" t="inlineStr">
         <is>
           <t>в КП не указана</t>
         </is>
       </c>
-      <c r="D39" s="22" t="inlineStr">
+      <c r="D48" s="27" t="inlineStr">
         <is>
           <t>ответ по заявке ≤ 2 ч, выезд ≤ 24 ч, вызовы без ограничений</t>
         </is>
       </c>
-      <c r="E39" s="47" t="n"/>
-      <c r="F39" s="47" t="n"/>
-      <c r="G39" s="45" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="E48" s="48" t="n"/>
+      <c r="F48" s="48" t="n"/>
+      <c r="G48" s="46" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>ККЗ</t>
         </is>
       </c>
-      <c r="C40" s="21" t="n">
+      <c r="C49" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="D40" s="22" t="inlineStr">
+      <c r="D49" s="27" t="inlineStr">
         <is>
           <t>выезд по запросу</t>
         </is>
       </c>
-      <c r="E40" s="47" t="n"/>
-      <c r="F40" s="47" t="n"/>
-      <c r="G40" s="45" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="E49" s="48" t="n"/>
+      <c r="F49" s="48" t="n"/>
+      <c r="G49" s="46" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>бройлерные площадки</t>
         </is>
       </c>
-      <c r="C41" s="21" t="n">
+      <c r="C50" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="D41" s="22" t="inlineStr">
+      <c r="D50" s="27" t="inlineStr">
         <is>
           <t>дополнительные визиты по вызову</t>
         </is>
       </c>
-      <c r="E41" s="47" t="n"/>
-      <c r="F41" s="47" t="n"/>
-      <c r="G41" s="45" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="E50" s="48" t="n"/>
+      <c r="F50" s="48" t="n"/>
+      <c r="G50" s="46" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>ЗПП</t>
         </is>
       </c>
-      <c r="C42" s="21" t="n">
+      <c r="C51" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="D42" s="22" t="inlineStr">
+      <c r="D51" s="27" t="inlineStr">
         <is>
           <t>по графику на 2026 год, бригада из трёх человек</t>
         </is>
       </c>
-      <c r="E42" s="47" t="n"/>
-      <c r="F42" s="47" t="n"/>
-      <c r="G42" s="45" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+      <c r="E51" s="48" t="n"/>
+      <c r="F51" s="48" t="n"/>
+      <c r="G51" s="46" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>склад ТМЦ</t>
         </is>
       </c>
-      <c r="C43" s="21" t="n">
+      <c r="C52" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D52" s="27" t="inlineStr">
         <is>
           <t>выезд по рекламации за два рабочих дня</t>
         </is>
       </c>
-      <c r="E43" s="47" t="n"/>
-      <c r="F43" s="47" t="n"/>
-      <c r="G43" s="45" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="E52" s="48" t="n"/>
+      <c r="F52" s="48" t="n"/>
+      <c r="G52" s="46" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>все объекты</t>
         </is>
       </c>
-      <c r="C44" s="21" t="n">
+      <c r="C53" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="D44" s="22" t="inlineStr">
+      <c r="D53" s="27" t="inlineStr">
         <is>
           <t>присутствие 5/2, реакция в тот же день</t>
         </is>
       </c>
-      <c r="E44" s="47" t="n"/>
-      <c r="F44" s="47" t="n"/>
-      <c r="G44" s="45" t="n"/>
+      <c r="E53" s="48" t="n"/>
+      <c r="F53" s="48" t="n"/>
+      <c r="G53" s="46" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="D41:G41"/>
-    <mergeCell ref="D40:G40"/>
+    <mergeCell ref="D48:G48"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D39:G39"/>
-    <mergeCell ref="D44:G44"/>
+    <mergeCell ref="D50:G50"/>
+    <mergeCell ref="D53:G53"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D52:G52"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D43:G43"/>
-    <mergeCell ref="D42:G42"/>
+    <mergeCell ref="D49:G49"/>
+    <mergeCell ref="D51:G51"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1532,7 +1798,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Кормоцех. Indigo — КП от 19.08.2026, цены с НДС. Pest Hunters — КП №26/12, без НДС. Штат УКПФ — 29 приманочных станций 2-го контура, 1 кг брикетов Pest Killer на обработку.</t>
         </is>
@@ -1540,37 +1806,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="26">
+      <c r="B5" s="30">
         <f>D9</f>
         <v>1159200</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="30">
         <f>D10</f>
         <v>900000</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="30">
         <f>D11+D12+D13+D14</f>
         <v>25497.5</v>
       </c>
@@ -1609,16 +1875,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · барьер вокруг периметра кормоцеха и грязный барьер</t>
         </is>
       </c>
-      <c r="B9" s="28">
+      <c r="B9" s="32">
         <f>Данные!$B$37</f>
         <v>96600</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="8">
@@ -1627,16 +1893,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters · дератизация</t>
         </is>
       </c>
-      <c r="B10" s="28">
+      <c r="B10" s="32">
         <f>Данные!$B$53</f>
         <v>75000</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="8">
@@ -1645,16 +1911,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
         </is>
       </c>
-      <c r="B11" s="28">
+      <c r="B11" s="32">
         <f>Данные!$D$20*Данные!$B$8</f>
         <v>0</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -1664,16 +1930,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
         </is>
       </c>
-      <c r="B12" s="28">
+      <c r="B12" s="32">
         <f>Данные!$D$20*2*Данные!$B$8</f>
         <v>0</v>
       </c>
-      <c r="C12" s="28">
+      <c r="C12" s="32">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
@@ -1683,16 +1949,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Зерноцид, 2-й контур</t>
         </is>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="32">
         <f>Данные!$G$20*Данные!$B$6</f>
         <v>0</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -1702,16 +1968,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B14" s="28">
+      <c r="B14" s="32">
         <f>Данные!$F$20*Данные!$B$7</f>
         <v>3642.5</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -1721,7 +1987,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -1765,16 +2031,16 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B19" s="28">
+      <c r="B19" s="32">
         <f>Данные!$B$20*Данные!$B$9</f>
         <v>0</v>
       </c>
-      <c r="C19" s="28" t="n">
+      <c r="C19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="7">
@@ -1783,16 +2049,16 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B20" s="28">
+      <c r="B20" s="32">
         <f>Данные!$C$20*Данные!$B$9</f>
         <v>62640</v>
       </c>
-      <c r="C20" s="28" t="n">
+      <c r="C20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="7">
@@ -1801,7 +2067,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="29" t="inlineStr">
+      <c r="C21" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -1845,16 +2111,16 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters · дезинсекция</t>
         </is>
       </c>
-      <c r="B25" s="28">
+      <c r="B25" s="32">
         <f>Данные!$B$54</f>
         <v>70000</v>
       </c>
-      <c r="C25" s="28" t="n">
+      <c r="C25" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D25" s="7">
@@ -1863,7 +2129,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="29" t="inlineStr">
+      <c r="C26" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -1875,14 +2141,14 @@
     </row>
     <row r="27"/>
     <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="23" t="inlineStr">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>Зерноцид по ККЗ в нормах не заявлен, поэтому строка Зерноцида даёт ноль.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="23" t="inlineStr">
+      <c r="A29" s="24" t="inlineStr">
         <is>
           <t>Зарплата дератизаторов по объектам не делится — она на листе «Штат УКПФ».</t>
         </is>
@@ -1921,7 +2187,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Восемь площадок: А, Б, В (Восточка), Г, Д, Е, Ж, Айыртау. У Indigo они разбиты на три группы, у Pest Hunters — 122 объекта с сезонным тарифом.</t>
         </is>
@@ -1929,37 +2195,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="26">
+      <c r="B5" s="30">
         <f>D9+D10+D11</f>
         <v>45447600</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="30">
         <f>D12+D13</f>
         <v>34770000</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="30">
         <f>D14+D15+D16+D17</f>
         <v>1240117.5</v>
       </c>
@@ -1998,16 +2264,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · Айыртау БП (БП-12, БП-13, БП-14) — полная замена, 180 ед.</t>
         </is>
       </c>
-      <c r="B9" s="28">
+      <c r="B9" s="32">
         <f>Данные!$B$38</f>
         <v>618400</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="8">
@@ -2016,16 +2282,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · Многоэтажки, площадки Д и Г — полная замена, 166 ед.</t>
         </is>
       </c>
-      <c r="B10" s="28">
+      <c r="B10" s="32">
         <f>Данные!$B$40</f>
         <v>569800</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="8">
@@ -2034,16 +2300,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (рем. молод), В — полная замена, 793 ед.</t>
         </is>
       </c>
-      <c r="B11" s="28">
+      <c r="B11" s="32">
         <f>Данные!$B$42</f>
         <v>2599100</v>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D11" s="8">
@@ -2052,16 +2318,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters · 122 объекта, март — ноябрь, оборудование подрядчика</t>
         </is>
       </c>
-      <c r="B12" s="28">
+      <c r="B12" s="32">
         <f>Данные!$B$55</f>
         <v>3172000</v>
       </c>
-      <c r="C12" s="28">
+      <c r="C12" s="32">
         <f>Данные!$B$61</f>
         <v>9</v>
       </c>
@@ -2071,16 +2337,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters · 122 объекта, декабрь — февраль, оборудование подрядчика</t>
         </is>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="32">
         <f>Данные!$B$56</f>
         <v>2074000</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="32">
         <f>Данные!$B$62</f>
         <v>3</v>
       </c>
@@ -2090,16 +2356,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
         </is>
       </c>
-      <c r="B14" s="28">
+      <c r="B14" s="32">
         <f>SUM(Данные!$D$23:$D$30)*Данные!$B$8</f>
         <v>42880</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2109,16 +2375,16 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
         </is>
       </c>
-      <c r="B15" s="28">
+      <c r="B15" s="32">
         <f>SUM(Данные!$D$23:$D$30)*2*Данные!$B$8</f>
         <v>85760</v>
       </c>
-      <c r="C15" s="28">
+      <c r="C15" s="32">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
@@ -2128,16 +2394,16 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Зерноцид, 2-й контур</t>
         </is>
       </c>
-      <c r="B16" s="28">
+      <c r="B16" s="32">
         <f>SUM(Данные!$G$23:$G$30)*Данные!$B$6</f>
         <v>11100</v>
       </c>
-      <c r="C16" s="28">
+      <c r="C16" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2147,16 +2413,16 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B17" s="28">
+      <c r="B17" s="32">
         <f>SUM(Данные!$F$23:$F$30)*Данные!$B$7</f>
         <v>61922.5</v>
       </c>
-      <c r="C17" s="28">
+      <c r="C17" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2166,7 +2432,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="29" t="inlineStr">
+      <c r="C18" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2210,16 +2476,16 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+      <c r="A22" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · Айыртау БП — частичная замена</t>
         </is>
       </c>
-      <c r="B22" s="28">
+      <c r="B22" s="32">
         <f>Данные!$B$39</f>
         <v>478400</v>
       </c>
-      <c r="C22" s="28" t="n">
+      <c r="C22" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D22" s="7">
@@ -2228,16 +2494,16 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · Многоэтажки Д и Г — частичная замена</t>
         </is>
       </c>
-      <c r="B23" s="28">
+      <c r="B23" s="32">
         <f>Данные!$B$41</f>
         <v>440700</v>
       </c>
-      <c r="C23" s="28" t="n">
+      <c r="C23" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D23" s="7">
@@ -2246,16 +2512,16 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="inlineStr">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (РМ), В — частичная замена</t>
         </is>
       </c>
-      <c r="B24" s="28">
+      <c r="B24" s="32">
         <f>Данные!$B$43</f>
         <v>2010300</v>
       </c>
-      <c r="C24" s="28" t="n">
+      <c r="C24" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D24" s="7">
@@ -2264,16 +2530,16 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters · 122 объекта, март — ноябрь, оборудование заказчика</t>
         </is>
       </c>
-      <c r="B25" s="28">
+      <c r="B25" s="32">
         <f>Данные!$B$57</f>
         <v>2806000</v>
       </c>
-      <c r="C25" s="28">
+      <c r="C25" s="32">
         <f>Данные!$B$61</f>
         <v>9</v>
       </c>
@@ -2283,16 +2549,16 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr">
+      <c r="A26" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters · 122 объекта, декабрь — февраль, оборудование заказчика</t>
         </is>
       </c>
-      <c r="B26" s="28">
+      <c r="B26" s="32">
         <f>Данные!$B$58</f>
         <v>1830000</v>
       </c>
-      <c r="C26" s="28">
+      <c r="C26" s="32">
         <f>Данные!$B$62</f>
         <v>3</v>
       </c>
@@ -2302,7 +2568,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="C27" s="29" t="inlineStr">
+      <c r="C27" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2346,16 +2612,16 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="inlineStr">
+      <c r="A31" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B31" s="28">
+      <c r="B31" s="32">
         <f>SUM(Данные!$B$23:$B$30)*Данные!$B$9</f>
         <v>347760</v>
       </c>
-      <c r="C31" s="28" t="n">
+      <c r="C31" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="7">
@@ -2364,16 +2630,16 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="27" t="inlineStr">
+      <c r="A32" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B32" s="28">
+      <c r="B32" s="32">
         <f>SUM(Данные!$C$23:$C$30)*Данные!$B$9</f>
         <v>2367360</v>
       </c>
-      <c r="C32" s="28" t="n">
+      <c r="C32" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="7">
@@ -2382,7 +2648,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="C33" s="29" t="inlineStr">
+      <c r="C33" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2426,16 +2692,16 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="27" t="inlineStr">
+      <c r="A37" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · Айыртау БП</t>
         </is>
       </c>
-      <c r="B37" s="28">
+      <c r="B37" s="32">
         <f>Данные!$B$48</f>
         <v>720000</v>
       </c>
-      <c r="C37" s="28" t="n">
+      <c r="C37" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D37" s="7">
@@ -2444,16 +2710,16 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="27" t="inlineStr">
+      <c r="A38" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · Многоэтажки Д и Г</t>
         </is>
       </c>
-      <c r="B38" s="28">
+      <c r="B38" s="32">
         <f>Данные!$B$49</f>
         <v>1080000</v>
       </c>
-      <c r="C38" s="28" t="n">
+      <c r="C38" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D38" s="7">
@@ -2462,16 +2728,16 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="27" t="inlineStr">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (РМ), В</t>
         </is>
       </c>
-      <c r="B39" s="28">
+      <c r="B39" s="32">
         <f>Данные!$B$50</f>
         <v>3000000</v>
       </c>
-      <c r="C39" s="28" t="n">
+      <c r="C39" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D39" s="7">
@@ -2480,7 +2746,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="29" t="inlineStr">
+      <c r="C40" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2492,14 +2758,14 @@
     </row>
     <row r="41"/>
     <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="23" t="inlineStr">
+      <c r="A42" s="24" t="inlineStr">
         <is>
           <t>Состав площадок у Indigo и в нашем расчёте описан по-разному: у них шесть напольных площадок плюс «В (рем. молод)», у нас восемь площадок по контурам. Сопоставлять построчно нельзя, только суммарно.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="23" t="inlineStr">
+      <c r="A43" s="24" t="inlineStr">
         <is>
           <t>Разовая закупка приманочных станций 1-го и 2-го контура показана справочно и в годовой итог не входит.</t>
         </is>
@@ -2538,7 +2804,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>У Indigo появился в КП от 19.08.2026: 48 ед. оборудования. У Pest Hunters предложения нет.</t>
         </is>
@@ -2546,37 +2812,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="26">
+      <c r="B5" s="30">
         <f>D9</f>
         <v>1514400</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="30">
         <f>D10</f>
         <v>0</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="30">
         <f>D11+D12+D13+D14</f>
         <v>63317.5</v>
       </c>
@@ -2615,16 +2881,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · полная замена оборудования, 48 ед.</t>
         </is>
       </c>
-      <c r="B9" s="28">
+      <c r="B9" s="32">
         <f>Данные!$B$44</f>
         <v>126200</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="8">
@@ -2633,15 +2899,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B10" s="28" t="n">
+      <c r="B10" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="8">
@@ -2650,16 +2916,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
         </is>
       </c>
-      <c r="B11" s="28">
+      <c r="B11" s="32">
         <f>Данные!$D$21*Данные!$B$8</f>
         <v>1920</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2669,16 +2935,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
         </is>
       </c>
-      <c r="B12" s="28">
+      <c r="B12" s="32">
         <f>Данные!$D$21*2*Данные!$B$8</f>
         <v>3840</v>
       </c>
-      <c r="C12" s="28">
+      <c r="C12" s="32">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
@@ -2688,16 +2954,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Зерноцид, 2-й контур</t>
         </is>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="32">
         <f>Данные!$G$21*Данные!$B$6</f>
         <v>740</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2707,16 +2973,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B14" s="28">
+      <c r="B14" s="32">
         <f>Данные!$F$21*Данные!$B$7</f>
         <v>3642.5</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2726,7 +2992,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2770,16 +3036,16 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · частичная замена оборудования</t>
         </is>
       </c>
-      <c r="B19" s="28">
+      <c r="B19" s="32">
         <f>Данные!$B$45</f>
         <v>106800</v>
       </c>
-      <c r="C19" s="28" t="n">
+      <c r="C19" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D19" s="7">
@@ -2788,7 +3054,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C20" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2832,16 +3098,16 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="inlineStr">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B24" s="28">
+      <c r="B24" s="32">
         <f>Данные!$B$21*Данные!$B$9</f>
         <v>38880</v>
       </c>
-      <c r="C24" s="28" t="n">
+      <c r="C24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="7">
@@ -2850,16 +3116,16 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B25" s="28">
+      <c r="B25" s="32">
         <f>Данные!$C$21*Данные!$B$9</f>
         <v>73440</v>
       </c>
-      <c r="C25" s="28" t="n">
+      <c r="C25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="7">
@@ -2868,7 +3134,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="29" t="inlineStr">
+      <c r="C26" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2912,16 +3178,16 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="inlineStr">
+      <c r="A30" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · дезинсекция</t>
         </is>
       </c>
-      <c r="B30" s="28">
+      <c r="B30" s="32">
         <f>Данные!$B$51</f>
         <v>100800</v>
       </c>
-      <c r="C30" s="28" t="n">
+      <c r="C30" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D30" s="7">
@@ -2930,7 +3196,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="C31" s="29" t="inlineStr">
+      <c r="C31" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2942,7 +3208,7 @@
     </row>
     <row r="32"/>
     <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="23" t="inlineStr">
+      <c r="A33" s="24" t="inlineStr">
         <is>
           <t>Нормы штата по инкубаторию: 18 точек 1-го контура, 34 второго, 12 клеевых третьего; 1 кг брикетов Pest Killer и 1 кг Зерноцида на обработку.</t>
         </is>
@@ -2980,7 +3246,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Завод по переработке птицы, 8 309 м². У Pest Hunters — подписанный договор №88, цена включает дезинсекцию. У Indigo — предложение из КП от 19.08.2026.</t>
         </is>
@@ -2988,37 +3254,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="26">
+      <c r="B5" s="30">
         <f>D9</f>
         <v>1514400</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="30">
         <f>D10</f>
         <v>2160000</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="30">
         <f>D11</f>
         <v>0</v>
       </c>
@@ -3057,16 +3323,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · полная замена оборудования</t>
         </is>
       </c>
-      <c r="B9" s="28">
+      <c r="B9" s="32">
         <f>Данные!$B$46</f>
         <v>126200</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="8">
@@ -3075,16 +3341,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters · договор №88 от 01.01.2026: дератизация и дезинсекция вместе</t>
         </is>
       </c>
-      <c r="B10" s="28">
+      <c r="B10" s="32">
         <f>Данные!$B$59</f>
         <v>180000</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="8">
@@ -3093,15 +3359,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · нормы расхода по ЗПП не заданы</t>
         </is>
       </c>
-      <c r="B11" s="28" t="n">
+      <c r="B11" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="8">
@@ -3110,7 +3376,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="C12" s="29" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3154,16 +3420,16 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · частичная замена оборудования</t>
         </is>
       </c>
-      <c r="B16" s="28">
+      <c r="B16" s="32">
         <f>Данные!$B$47</f>
         <v>106800</v>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D16" s="7">
@@ -3172,7 +3438,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="29" t="inlineStr">
+      <c r="C17" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3216,16 +3482,16 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions · дезинсекция</t>
         </is>
       </c>
-      <c r="B21" s="28">
+      <c r="B21" s="32">
         <f>Данные!$B$52</f>
         <v>160800</v>
       </c>
-      <c r="C21" s="28" t="n">
+      <c r="C21" s="32" t="n">
         <v>12</v>
       </c>
       <c r="D21" s="7">
@@ -3234,7 +3500,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="29" t="inlineStr">
+      <c r="C22" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3246,14 +3512,14 @@
     </row>
     <row r="23"/>
     <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="23" t="inlineStr">
+      <c r="A24" s="24" t="inlineStr">
         <is>
           <t>Строки не полностью сопоставимы: у Pest Hunters 180 000 ₸ включают и дератизацию, и дезинсекцию, у Indigo эти услуги разделены — 126 200 ₸ дератизация и 160 800 ₸ дезинсекция.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="23" t="inlineStr">
+      <c r="A25" s="24" t="inlineStr">
         <is>
           <t>По штату УКПФ нормы расхода на ЗПП не заданы, поэтому в расчёте ноль.</t>
         </is>
@@ -3292,7 +3558,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Договор №921 от 01.04.2026, действует с апреля по декабрь. Предложений от Indigo по этому объекту нет.</t>
         </is>
@@ -3300,37 +3566,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="26">
+      <c r="B5" s="30">
         <f>D9</f>
         <v>0</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="30">
         <f>D10</f>
         <v>720000</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="30">
         <f>D11</f>
         <v>0</v>
       </c>
@@ -3369,15 +3635,15 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n">
+      <c r="B9" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="8">
@@ -3386,16 +3652,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters · договор №921: дератизация и дезинсекция, выезд по рекламации за 2 рабочих дня</t>
         </is>
       </c>
-      <c r="B10" s="28">
+      <c r="B10" s="32">
         <f>Данные!$B$60</f>
         <v>80000</v>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="32">
         <f>Данные!$B$63</f>
         <v>9</v>
       </c>
@@ -3405,15 +3671,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · нормы расхода по складу не заданы</t>
         </is>
       </c>
-      <c r="B11" s="28" t="n">
+      <c r="B11" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="8">
@@ -3422,7 +3688,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="C12" s="29" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3434,7 +3700,7 @@
     </row>
     <row r="13"/>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>С января по март договор не действует, поэтому в году девять оплачиваемых месяцев.</t>
         </is>
@@ -3472,7 +3738,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Административно-бытовые корпуса на одиннадцати площадках. Ни у Indigo, ни у Pest Hunters отдельной строки по АБК нет.</t>
         </is>
@@ -3480,37 +3746,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="26">
+      <c r="B5" s="30">
         <f>D9</f>
         <v>0</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="30">
         <f>D10</f>
         <v>0</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="30">
         <f>D11+D12+D13+D14</f>
         <v>204506.75</v>
       </c>
@@ -3549,15 +3815,15 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n">
+      <c r="B9" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="8">
@@ -3566,15 +3832,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B10" s="28" t="n">
+      <c r="B10" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="32" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="8">
@@ -3583,16 +3849,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
         </is>
       </c>
-      <c r="B11" s="28">
+      <c r="B11" s="32">
         <f>Данные!$D$22*Данные!$B$8</f>
         <v>10080</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -3602,16 +3868,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
         </is>
       </c>
-      <c r="B12" s="28">
+      <c r="B12" s="32">
         <f>Данные!$D$22*2*Данные!$B$8</f>
         <v>20160</v>
       </c>
-      <c r="C12" s="28">
+      <c r="C12" s="32">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
@@ -3621,16 +3887,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Зерноцид, 2-й контур</t>
         </is>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="32">
         <f>Данные!$G$22*Данные!$B$6</f>
         <v>0</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -3640,16 +3906,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B14" s="28">
+      <c r="B14" s="32">
         <f>Данные!$F$22*Данные!$B$7</f>
         <v>4735.25</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="32">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -3659,7 +3925,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3703,16 +3969,16 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B19" s="28">
+      <c r="B19" s="32">
         <f>Данные!$B$22*Данные!$B$9</f>
         <v>0</v>
       </c>
-      <c r="C19" s="28" t="n">
+      <c r="C19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="7">
@@ -3721,16 +3987,16 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B20" s="28">
+      <c r="B20" s="32">
         <f>Данные!$C$22*Данные!$B$9</f>
         <v>84240</v>
       </c>
-      <c r="C20" s="28" t="n">
+      <c r="C20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="7">
@@ -3739,7 +4005,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="29" t="inlineStr">
+      <c r="C21" s="33" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3751,14 +4017,14 @@
     </row>
     <row r="22"/>
     <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="23" t="inlineStr">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Клеевые станции по корпусам: Б — 11, Ж — 5, Е — 6, В — 6, В (РМ) — 6, Д — 3, Г — 3, БП-12 — 6, БП-13 — 6, БП-14 — 6, А — 5. Приманочные: 4, 2, 3, 3, 3, 4, 3, 5, 5, 5, 2.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="23" t="inlineStr">
+      <c r="A24" s="24" t="inlineStr">
         <is>
           <t>Норма 1,3 кг брикетов Pest Killer по АБК — приблизительная оценка, требует подтверждения. Зерноцид по АБК не заявлен.</t>
         </is>
@@ -3821,17 +4087,17 @@
       <c r="E4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Показатель, ₸</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Оклад 258 488 ₸</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Оклад 350 000 ₸</t>
         </is>
@@ -3883,7 +4149,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="34" t="inlineStr">
         <is>
           <t>Зарплата за год</t>
         </is>
@@ -3914,47 +4180,47 @@
       <c r="I11" s="16" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B12" s="32" t="inlineStr">
+      <c r="B12" s="36" t="inlineStr">
         <is>
           <t>Клеевых 3-го к., шт/мес лето</t>
         </is>
       </c>
-      <c r="C12" s="32" t="inlineStr">
+      <c r="C12" s="36" t="inlineStr">
         <is>
           <t>Клеевых 3-го к., шт/мес зима</t>
         </is>
       </c>
-      <c r="D12" s="32" t="inlineStr">
+      <c r="D12" s="36" t="inlineStr">
         <is>
           <t>Клеевые за год, ₸</t>
         </is>
       </c>
-      <c r="E12" s="32" t="inlineStr">
+      <c r="E12" s="36" t="inlineStr">
         <is>
           <t>Зерноцид, кг/мес</t>
         </is>
       </c>
-      <c r="F12" s="32" t="inlineStr">
+      <c r="F12" s="36" t="inlineStr">
         <is>
           <t>Зерноцид за год, ₸</t>
         </is>
       </c>
-      <c r="G12" s="32" t="inlineStr">
+      <c r="G12" s="36" t="inlineStr">
         <is>
           <t>Pest Killer, кг/мес</t>
         </is>
       </c>
-      <c r="H12" s="32" t="inlineStr">
+      <c r="H12" s="36" t="inlineStr">
         <is>
           <t>Pest Killer за год, ₸</t>
         </is>
       </c>
-      <c r="I12" s="32" t="inlineStr">
+      <c r="I12" s="36" t="inlineStr">
         <is>
           <t>Материалы за год, ₸</t>
         </is>
@@ -3966,11 +4232,11 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B13" s="33">
+      <c r="B13" s="37">
         <f>Данные!$D$20</f>
         <v>0</v>
       </c>
-      <c r="C13" s="33">
+      <c r="C13" s="37">
         <f>Данные!$D$20*2</f>
         <v>0</v>
       </c>
@@ -3978,7 +4244,7 @@
         <f>B13*Данные!$B$8*Данные!$B$15+C13*Данные!$B$8*Данные!$B$16</f>
         <v>0</v>
       </c>
-      <c r="E13" s="48">
+      <c r="E13" s="49">
         <f>Данные!$G$20</f>
         <v>0</v>
       </c>
@@ -3986,7 +4252,7 @@
         <f>E13*Данные!$B$6*Данные!$B$15</f>
         <v>0</v>
       </c>
-      <c r="G13" s="48">
+      <c r="G13" s="49">
         <f>Данные!$F$20</f>
         <v>1</v>
       </c>
@@ -4005,11 +4271,11 @@
           <t>Бройлерные площадки · 8 шт</t>
         </is>
       </c>
-      <c r="B14" s="33">
+      <c r="B14" s="37">
         <f>SUM(Данные!$D$23:$D$30)</f>
         <v>268</v>
       </c>
-      <c r="C14" s="33">
+      <c r="C14" s="37">
         <f>SUM(Данные!$D$23:$D$30)*2</f>
         <v>536</v>
       </c>
@@ -4017,7 +4283,7 @@
         <f>B14*Данные!$B$8*Данные!$B$15+C14*Данные!$B$8*Данные!$B$16</f>
         <v>728960</v>
       </c>
-      <c r="E14" s="48">
+      <c r="E14" s="49">
         <f>SUM(Данные!$G$23:$G$30)</f>
         <v>15</v>
       </c>
@@ -4025,7 +4291,7 @@
         <f>E14*Данные!$B$6*Данные!$B$15</f>
         <v>77700</v>
       </c>
-      <c r="G14" s="48">
+      <c r="G14" s="49">
         <f>SUM(Данные!$F$23:$F$30)</f>
         <v>17</v>
       </c>
@@ -4044,11 +4310,11 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B15" s="33">
+      <c r="B15" s="37">
         <f>Данные!$D$21</f>
         <v>12</v>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="37">
         <f>Данные!$D$21*2</f>
         <v>24</v>
       </c>
@@ -4056,7 +4322,7 @@
         <f>B15*Данные!$B$8*Данные!$B$15+C15*Данные!$B$8*Данные!$B$16</f>
         <v>32640</v>
       </c>
-      <c r="E15" s="48">
+      <c r="E15" s="49">
         <f>Данные!$G$21</f>
         <v>1</v>
       </c>
@@ -4064,7 +4330,7 @@
         <f>E15*Данные!$B$6*Данные!$B$15</f>
         <v>5180</v>
       </c>
-      <c r="G15" s="48">
+      <c r="G15" s="49">
         <f>Данные!$F$21</f>
         <v>1</v>
       </c>
@@ -4083,11 +4349,11 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B16" s="33">
+      <c r="B16" s="37">
         <f>Данные!$D$22</f>
         <v>63</v>
       </c>
-      <c r="C16" s="33">
+      <c r="C16" s="37">
         <f>Данные!$D$22*2</f>
         <v>126</v>
       </c>
@@ -4095,7 +4361,7 @@
         <f>B16*Данные!$B$8*Данные!$B$15+C16*Данные!$B$8*Данные!$B$16</f>
         <v>171360</v>
       </c>
-      <c r="E16" s="48">
+      <c r="E16" s="49">
         <f>Данные!$G$22</f>
         <v>0</v>
       </c>
@@ -4103,7 +4369,7 @@
         <f>E16*Данные!$B$6*Данные!$B$15</f>
         <v>0</v>
       </c>
-      <c r="G16" s="48">
+      <c r="G16" s="49">
         <f>Данные!$F$22</f>
         <v>1.3</v>
       </c>
@@ -4140,13 +4406,13 @@
           <t>МАТЕРИАЛЫ ЗА ГОД, ИТОГО</t>
         </is>
       </c>
-      <c r="B18" s="35" t="n"/>
-      <c r="C18" s="35" t="n"/>
+      <c r="B18" s="22" t="n"/>
+      <c r="C18" s="22" t="n"/>
       <c r="D18" s="12">
         <f>SUM(D13:D17)</f>
         <v>932960</v>
       </c>
-      <c r="E18" s="49">
+      <c r="E18" s="50">
         <f>SUM(E13:E17)</f>
         <v>16</v>
       </c>
@@ -4154,7 +4420,7 @@
         <f>SUM(F13:F17)</f>
         <v>82880</v>
       </c>
-      <c r="G18" s="49">
+      <c r="G18" s="50">
         <f>SUM(G13:G17)</f>
         <v>20.3</v>
       </c>
@@ -4181,32 +4447,32 @@
       <c r="F20" s="16" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="37" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B21" s="38" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>1-й контур, шт</t>
         </is>
       </c>
-      <c r="C21" s="38" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>2-й контур, шт</t>
         </is>
       </c>
-      <c r="D21" s="38" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>Всего, шт</t>
         </is>
       </c>
-      <c r="E21" s="38" t="inlineStr">
+      <c r="E21" s="20" t="inlineStr">
         <is>
           <t>Цена, ₸/шт</t>
         </is>
       </c>
-      <c r="F21" s="38" t="inlineStr">
+      <c r="F21" s="20" t="inlineStr">
         <is>
           <t>Разово, ₸</t>
         </is>
@@ -4218,19 +4484,19 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B22" s="33">
+      <c r="B22" s="37">
         <f>Данные!$B$20</f>
         <v>0</v>
       </c>
-      <c r="C22" s="33">
+      <c r="C22" s="37">
         <f>Данные!$C$20</f>
         <v>29</v>
       </c>
-      <c r="D22" s="33">
+      <c r="D22" s="37">
         <f>B22+C22</f>
         <v>29</v>
       </c>
-      <c r="E22" s="28">
+      <c r="E22" s="32">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4245,19 +4511,19 @@
           <t>Бройлерные площадки · 8 шт</t>
         </is>
       </c>
-      <c r="B23" s="33">
+      <c r="B23" s="37">
         <f>SUM(Данные!$B$23:$B$30)</f>
         <v>161</v>
       </c>
-      <c r="C23" s="33">
+      <c r="C23" s="37">
         <f>SUM(Данные!$C$23:$C$30)</f>
         <v>1096</v>
       </c>
-      <c r="D23" s="33">
+      <c r="D23" s="37">
         <f>B23+C23</f>
         <v>1257</v>
       </c>
-      <c r="E23" s="28">
+      <c r="E23" s="32">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4272,19 +4538,19 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B24" s="33">
+      <c r="B24" s="37">
         <f>Данные!$B$21</f>
         <v>18</v>
       </c>
-      <c r="C24" s="33">
+      <c r="C24" s="37">
         <f>Данные!$C$21</f>
         <v>34</v>
       </c>
-      <c r="D24" s="33">
+      <c r="D24" s="37">
         <f>B24+C24</f>
         <v>52</v>
       </c>
-      <c r="E24" s="28">
+      <c r="E24" s="32">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4299,19 +4565,19 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B25" s="33">
+      <c r="B25" s="37">
         <f>Данные!$B$22</f>
         <v>0</v>
       </c>
-      <c r="C25" s="33">
+      <c r="C25" s="37">
         <f>Данные!$C$22</f>
         <v>39</v>
       </c>
-      <c r="D25" s="33">
+      <c r="D25" s="37">
         <f>B25+C25</f>
         <v>39</v>
       </c>
-      <c r="E25" s="28">
+      <c r="E25" s="32">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4326,19 +4592,19 @@
           <t>ИТОГО РАЗОВО</t>
         </is>
       </c>
-      <c r="B26" s="39">
+      <c r="B26" s="40">
         <f>SUM(B22:B25)</f>
         <v>179</v>
       </c>
-      <c r="C26" s="39">
+      <c r="C26" s="40">
         <f>SUM(C22:C25)</f>
         <v>1198</v>
       </c>
-      <c r="D26" s="39">
+      <c r="D26" s="40">
         <f>SUM(D22:D25)</f>
         <v>1377</v>
       </c>
-      <c r="E26" s="35" t="n"/>
+      <c r="E26" s="22" t="n"/>
       <c r="F26" s="12">
         <f>SUM(F22:F25)</f>
         <v>2974320</v>
@@ -4358,32 +4624,32 @@
       <c r="F28" s="16" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="31" t="inlineStr">
+      <c r="A29" s="35" t="inlineStr">
         <is>
           <t>Численность, чел.</t>
         </is>
       </c>
-      <c r="B29" s="32" t="inlineStr">
+      <c r="B29" s="36" t="inlineStr">
         <is>
           <t>ЗП в месяц, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="C29" s="32" t="inlineStr">
+      <c r="C29" s="36" t="inlineStr">
         <is>
           <t>ЗП за год, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="D29" s="32" t="inlineStr">
+      <c r="D29" s="36" t="inlineStr">
         <is>
           <t>Материалы за год, ₸</t>
         </is>
       </c>
-      <c r="E29" s="32" t="inlineStr">
+      <c r="E29" s="36" t="inlineStr">
         <is>
           <t>Итого за год, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="F29" s="32" t="inlineStr">
+      <c r="F29" s="36" t="inlineStr">
         <is>
           <t>Итого за год, ₸ · оклад 350 000</t>
         </is>
@@ -4616,7 +4882,7 @@
     </row>
     <row r="39"/>
     <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="23" t="inlineStr">
+      <c r="A40" s="24" t="inlineStr">
         <is>
           <t>Материалы от численности не зависят — норма ядов и станций привязана к точкам, а не к людям. Каждый дополнительный дератизатор добавляет только фонд оплаты труда.</t>
         </is>
@@ -4680,26 +4946,26 @@
       <c r="H4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>Ед. изм.</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr"/>
-      <c r="E5" s="20" t="inlineStr"/>
-      <c r="F5" s="20" t="inlineStr"/>
-      <c r="G5" s="20" t="inlineStr"/>
-      <c r="H5" s="20" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr"/>
+      <c r="E5" s="26" t="inlineStr"/>
+      <c r="F5" s="26" t="inlineStr"/>
+      <c r="G5" s="26" t="inlineStr"/>
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Источник / примечание</t>
         </is>
@@ -4711,7 +4977,7 @@
           <t>Зерноцид</t>
         </is>
       </c>
-      <c r="B6" s="40" t="n">
+      <c r="B6" s="41" t="n">
         <v>740</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -4719,7 +4985,7 @@
           <t>₸/кг</t>
         </is>
       </c>
-      <c r="H6" s="41" t="inlineStr">
+      <c r="H6" s="42" t="inlineStr">
         <is>
           <t>внутренние данные УКПФ</t>
         </is>
@@ -4731,7 +4997,7 @@
           <t>Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B7" s="40" t="n">
+      <c r="B7" s="41" t="n">
         <v>3642.5</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -4739,7 +5005,7 @@
           <t>₸/кг</t>
         </is>
       </c>
-      <c r="H7" s="41" t="inlineStr">
+      <c r="H7" s="42" t="inlineStr">
         <is>
           <t>перенесено из прежнего расчёта по ККЗ; в исходных нормах цены не было</t>
         </is>
@@ -4751,7 +5017,7 @@
           <t>Клеевая станция 3-го контура</t>
         </is>
       </c>
-      <c r="B8" s="40" t="n">
+      <c r="B8" s="41" t="n">
         <v>160</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -4759,7 +5025,7 @@
           <t>₸/шт</t>
         </is>
       </c>
-      <c r="H8" s="41" t="inlineStr">
+      <c r="H8" s="42" t="inlineStr">
         <is>
           <t>внутренние данные УКПФ, расходуется ежемесячно</t>
         </is>
@@ -4771,7 +5037,7 @@
           <t>Приманочная станция 1–2 контура</t>
         </is>
       </c>
-      <c r="B9" s="40" t="n">
+      <c r="B9" s="41" t="n">
         <v>2160</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -4779,7 +5045,7 @@
           <t>₸/шт</t>
         </is>
       </c>
-      <c r="H9" s="41" t="inlineStr">
+      <c r="H9" s="42" t="inlineStr">
         <is>
           <t>разовая закупка; цена из прежнего расчёта по ККЗ (29 шт = 62 640 ₸)</t>
         </is>
@@ -4791,7 +5057,7 @@
           <t>Бутылка</t>
         </is>
       </c>
-      <c r="B10" s="40" t="n">
+      <c r="B10" s="41" t="n">
         <v>68</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -4799,7 +5065,7 @@
           <t>₸/шт</t>
         </is>
       </c>
-      <c r="H10" s="41" t="inlineStr">
+      <c r="H10" s="42" t="inlineStr">
         <is>
           <t>внутренние данные УКПФ</t>
         </is>
@@ -4811,7 +5077,7 @@
           <t>Бутылки, расход</t>
         </is>
       </c>
-      <c r="B11" s="40" t="n">
+      <c r="B11" s="41" t="n">
         <v>40</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -4819,7 +5085,7 @@
           <t>шт/мес</t>
         </is>
       </c>
-      <c r="H11" s="41" t="inlineStr">
+      <c r="H11" s="42" t="inlineStr">
         <is>
           <t>тёплый сезон, зимой ноль; оценка, по объектам не разносится</t>
         </is>
@@ -4831,7 +5097,7 @@
           <t>Оклад дератизатора · вариант 1</t>
         </is>
       </c>
-      <c r="B12" s="40" t="n">
+      <c r="B12" s="41" t="n">
         <v>258488</v>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -4839,7 +5105,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H12" s="41" t="inlineStr">
+      <c r="H12" s="42" t="inlineStr">
         <is>
           <t>действующий оклад</t>
         </is>
@@ -4851,7 +5117,7 @@
           <t>Оклад дератизатора · вариант 2</t>
         </is>
       </c>
-      <c r="B13" s="40" t="n">
+      <c r="B13" s="41" t="n">
         <v>350000</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -4859,7 +5125,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H13" s="41" t="inlineStr">
+      <c r="H13" s="42" t="inlineStr">
         <is>
           <t>альтернативный уровень для сравнения</t>
         </is>
@@ -4871,7 +5137,7 @@
           <t>Численность штата</t>
         </is>
       </c>
-      <c r="B14" s="40" t="n">
+      <c r="B14" s="41" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -4879,7 +5145,7 @@
           <t>чел.</t>
         </is>
       </c>
-      <c r="H14" s="41" t="inlineStr">
+      <c r="H14" s="42" t="inlineStr">
         <is>
           <t>измените — пересчитаются все листы</t>
         </is>
@@ -4891,7 +5157,7 @@
           <t>Тёплых месяцев (апрель — октябрь)</t>
         </is>
       </c>
-      <c r="B15" s="40" t="n">
+      <c r="B15" s="41" t="n">
         <v>7</v>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -4899,7 +5165,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H15" s="41" t="inlineStr">
+      <c r="H15" s="42" t="inlineStr">
         <is>
           <t>заряжаются все три контура</t>
         </is>
@@ -4911,7 +5177,7 @@
           <t>Зимних месяцев (ноябрь — март)</t>
         </is>
       </c>
-      <c r="B16" s="40" t="n">
+      <c r="B16" s="41" t="n">
         <v>5</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -4919,7 +5185,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H16" s="41" t="inlineStr">
+      <c r="H16" s="42" t="inlineStr">
         <is>
           <t>1-й и 2-й контуры не заряжаются, 3-й обслуживается вдвое</t>
         </is>
@@ -4941,42 +5207,42 @@
       <c r="H18" s="16" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="35" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B19" s="32" t="inlineStr">
+      <c r="B19" s="36" t="inlineStr">
         <is>
           <t>1-й контур, шт</t>
         </is>
       </c>
-      <c r="C19" s="32" t="inlineStr">
+      <c r="C19" s="36" t="inlineStr">
         <is>
           <t>2-й контур, шт</t>
         </is>
       </c>
-      <c r="D19" s="32" t="inlineStr">
+      <c r="D19" s="36" t="inlineStr">
         <is>
           <t>3-й контур, шт</t>
         </is>
       </c>
-      <c r="E19" s="32" t="inlineStr">
+      <c r="E19" s="36" t="inlineStr">
         <is>
           <t>Всего точек, шт</t>
         </is>
       </c>
-      <c r="F19" s="32" t="inlineStr">
+      <c r="F19" s="36" t="inlineStr">
         <is>
           <t>Pest Killer, кг</t>
         </is>
       </c>
-      <c r="G19" s="32" t="inlineStr">
+      <c r="G19" s="36" t="inlineStr">
         <is>
           <t>Зерноцид, кг</t>
         </is>
       </c>
-      <c r="H19" s="32" t="inlineStr">
+      <c r="H19" s="36" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
@@ -4988,26 +5254,26 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B20" s="40" t="n">
+      <c r="B20" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="40" t="n">
+      <c r="C20" s="41" t="n">
         <v>29</v>
       </c>
-      <c r="D20" s="40" t="n">
+      <c r="D20" s="41" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="7">
         <f>SUM(B20:D20)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="50" t="n">
+      <c r="F20" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="50" t="n">
+      <c r="G20" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="41" t="inlineStr">
+      <c r="H20" s="42" t="inlineStr">
         <is>
           <t>29 приманочных станций 2-го контура</t>
         </is>
@@ -5019,26 +5285,26 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B21" s="40" t="n">
+      <c r="B21" s="41" t="n">
         <v>18</v>
       </c>
-      <c r="C21" s="40" t="n">
+      <c r="C21" s="41" t="n">
         <v>34</v>
       </c>
-      <c r="D21" s="40" t="n">
+      <c r="D21" s="41" t="n">
         <v>12</v>
       </c>
       <c r="E21" s="7">
         <f>SUM(B21:D21)</f>
         <v>18</v>
       </c>
-      <c r="F21" s="50" t="n">
+      <c r="F21" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="50" t="n">
+      <c r="G21" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="41" t="inlineStr"/>
+      <c r="H21" s="42" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -5046,26 +5312,26 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B22" s="40" t="n">
+      <c r="B22" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="40" t="n">
+      <c r="C22" s="41" t="n">
         <v>39</v>
       </c>
-      <c r="D22" s="40" t="n">
+      <c r="D22" s="41" t="n">
         <v>63</v>
       </c>
       <c r="E22" s="7">
         <f>SUM(B22:D22)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="50" t="n">
+      <c r="F22" s="51" t="n">
         <v>1.3</v>
       </c>
-      <c r="G22" s="50" t="n">
+      <c r="G22" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="41" t="inlineStr">
+      <c r="H22" s="42" t="inlineStr">
         <is>
           <t>1,3 кг — приблизительная оценка, требует подтверждения</t>
         </is>
@@ -5077,26 +5343,26 @@
           <t>Площадка А</t>
         </is>
       </c>
-      <c r="B23" s="40" t="n">
+      <c r="B23" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="C23" s="40" t="n">
+      <c r="C23" s="41" t="n">
         <v>147</v>
       </c>
-      <c r="D23" s="40" t="n">
+      <c r="D23" s="41" t="n">
         <v>20</v>
       </c>
       <c r="E23" s="7">
         <f>SUM(B23:D23)</f>
         <v>13</v>
       </c>
-      <c r="F23" s="50" t="n">
+      <c r="F23" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="50" t="n">
+      <c r="G23" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="41" t="inlineStr"/>
+      <c r="H23" s="42" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -5104,26 +5370,26 @@
           <t>Площадка Б</t>
         </is>
       </c>
-      <c r="B24" s="40" t="n">
+      <c r="B24" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C24" s="40" t="n">
+      <c r="C24" s="41" t="n">
         <v>146</v>
       </c>
-      <c r="D24" s="40" t="n">
+      <c r="D24" s="41" t="n">
         <v>20</v>
       </c>
       <c r="E24" s="7">
         <f>SUM(B24:D24)</f>
         <v>17</v>
       </c>
-      <c r="F24" s="50" t="n">
+      <c r="F24" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="50" t="n">
+      <c r="G24" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="H24" s="41" t="inlineStr"/>
+      <c r="H24" s="42" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -5131,26 +5397,26 @@
           <t>В / Восточка</t>
         </is>
       </c>
-      <c r="B25" s="40" t="n">
+      <c r="B25" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="C25" s="40" t="n">
+      <c r="C25" s="41" t="n">
         <v>239</v>
       </c>
-      <c r="D25" s="40" t="n">
+      <c r="D25" s="41" t="n">
         <v>30</v>
       </c>
       <c r="E25" s="7">
         <f>SUM(B25:D25)</f>
         <v>50</v>
       </c>
-      <c r="F25" s="50" t="n">
+      <c r="F25" s="51" t="n">
         <v>3.5</v>
       </c>
-      <c r="G25" s="50" t="n">
+      <c r="G25" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="41" t="inlineStr"/>
+      <c r="H25" s="42" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -5158,26 +5424,26 @@
           <t>Площадка Г</t>
         </is>
       </c>
-      <c r="B26" s="40" t="n">
+      <c r="B26" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C26" s="40" t="n">
+      <c r="C26" s="41" t="n">
         <v>88</v>
       </c>
-      <c r="D26" s="40" t="n">
+      <c r="D26" s="41" t="n">
         <v>80</v>
       </c>
       <c r="E26" s="7">
         <f>SUM(B26:D26)</f>
         <v>17</v>
       </c>
-      <c r="F26" s="50" t="n">
+      <c r="F26" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="50" t="n">
+      <c r="G26" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="H26" s="41" t="inlineStr"/>
+      <c r="H26" s="42" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -5185,26 +5451,26 @@
           <t>Площадка Д</t>
         </is>
       </c>
-      <c r="B27" s="40" t="n">
+      <c r="B27" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="C27" s="40" t="n">
+      <c r="C27" s="41" t="n">
         <v>69</v>
       </c>
-      <c r="D27" s="40" t="n">
+      <c r="D27" s="41" t="n">
         <v>64</v>
       </c>
       <c r="E27" s="7">
         <f>SUM(B27:D27)</f>
         <v>15</v>
       </c>
-      <c r="F27" s="50" t="n">
+      <c r="F27" s="51" t="n">
         <v>1.5</v>
       </c>
-      <c r="G27" s="50" t="n">
+      <c r="G27" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="41" t="inlineStr"/>
+      <c r="H27" s="42" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -5212,26 +5478,26 @@
           <t>Площадка Е</t>
         </is>
       </c>
-      <c r="B28" s="40" t="n">
+      <c r="B28" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="C28" s="40" t="n">
+      <c r="C28" s="41" t="n">
         <v>147</v>
       </c>
-      <c r="D28" s="40" t="n">
+      <c r="D28" s="41" t="n">
         <v>20</v>
       </c>
       <c r="E28" s="7">
         <f>SUM(B28:D28)</f>
         <v>13</v>
       </c>
-      <c r="F28" s="50" t="n">
+      <c r="F28" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="50" t="n">
+      <c r="G28" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="H28" s="41" t="inlineStr"/>
+      <c r="H28" s="42" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -5239,26 +5505,26 @@
           <t>Площадка Ж</t>
         </is>
       </c>
-      <c r="B29" s="40" t="n">
+      <c r="B29" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C29" s="40" t="n">
+      <c r="C29" s="41" t="n">
         <v>73</v>
       </c>
-      <c r="D29" s="40" t="n">
+      <c r="D29" s="41" t="n">
         <v>10</v>
       </c>
       <c r="E29" s="7">
         <f>SUM(B29:D29)</f>
         <v>17</v>
       </c>
-      <c r="F29" s="50" t="n">
+      <c r="F29" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="50" t="n">
+      <c r="G29" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="H29" s="41" t="inlineStr"/>
+      <c r="H29" s="42" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -5266,26 +5532,26 @@
           <t>Айыртау (БП)</t>
         </is>
       </c>
-      <c r="B30" s="40" t="n">
+      <c r="B30" s="41" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="40" t="n">
+      <c r="C30" s="41" t="n">
         <v>187</v>
       </c>
-      <c r="D30" s="40" t="n">
+      <c r="D30" s="41" t="n">
         <v>24</v>
       </c>
       <c r="E30" s="7">
         <f>SUM(B30:D30)</f>
         <v>19</v>
       </c>
-      <c r="F30" s="50" t="n">
+      <c r="F30" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="G30" s="50" t="n">
+      <c r="G30" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="H30" s="41" t="inlineStr"/>
+      <c r="H30" s="42" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -5297,9 +5563,9 @@
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
-      <c r="F31" s="48" t="n"/>
-      <c r="G31" s="48" t="n"/>
-      <c r="H31" s="41" t="inlineStr">
+      <c r="F31" s="49" t="n"/>
+      <c r="G31" s="49" t="n"/>
+      <c r="H31" s="42" t="inlineStr">
         <is>
           <t>нормы расхода не заданы</t>
         </is>
@@ -5315,9 +5581,9 @@
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
-      <c r="F32" s="48" t="n"/>
-      <c r="G32" s="48" t="n"/>
-      <c r="H32" s="41" t="inlineStr">
+      <c r="F32" s="49" t="n"/>
+      <c r="G32" s="49" t="n"/>
+      <c r="H32" s="42" t="inlineStr">
         <is>
           <t>нормы расхода не заданы</t>
         </is>
@@ -5345,15 +5611,15 @@
         <f>SUM(E20:E32)</f>
         <v>179</v>
       </c>
-      <c r="F33" s="49">
+      <c r="F33" s="50">
         <f>SUM(F20:F32)</f>
         <v>20.3</v>
       </c>
-      <c r="G33" s="49">
+      <c r="G33" s="50">
         <f>SUM(G20:G32)</f>
         <v>16</v>
       </c>
-      <c r="H33" s="35" t="n"/>
+      <c r="H33" s="22" t="n"/>
     </row>
     <row r="34"/>
     <row r="35">
@@ -5371,26 +5637,26 @@
       <c r="H35" s="16" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="A36" s="26" t="inlineStr">
         <is>
           <t>Позиция</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="C36" s="20" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
         <is>
           <t>Ед. изм.</t>
         </is>
       </c>
-      <c r="D36" s="20" t="inlineStr"/>
-      <c r="E36" s="20" t="inlineStr"/>
-      <c r="F36" s="20" t="inlineStr"/>
-      <c r="G36" s="20" t="inlineStr"/>
-      <c r="H36" s="20" t="inlineStr">
+      <c r="D36" s="26" t="inlineStr"/>
+      <c r="E36" s="26" t="inlineStr"/>
+      <c r="F36" s="26" t="inlineStr"/>
+      <c r="G36" s="26" t="inlineStr"/>
+      <c r="H36" s="26" t="inlineStr">
         <is>
           <t>Источник</t>
         </is>
@@ -5402,7 +5668,7 @@
           <t>Indigo · ККЗ, дератизация</t>
         </is>
       </c>
-      <c r="B37" s="40" t="n">
+      <c r="B37" s="41" t="n">
         <v>96600</v>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -5410,7 +5676,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H37" s="41" t="inlineStr">
+      <c r="H37" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); барьер вокруг периметра кормоцеха и грязный барьер</t>
         </is>
@@ -5422,7 +5688,7 @@
           <t>Indigo · Айыртау БП, полная замена</t>
         </is>
       </c>
-      <c r="B38" s="40" t="n">
+      <c r="B38" s="41" t="n">
         <v>618400</v>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -5430,7 +5696,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H38" s="41" t="inlineStr">
+      <c r="H38" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 180 ед. оборудования</t>
         </is>
@@ -5442,7 +5708,7 @@
           <t>Indigo · Айыртау БП, частичная замена</t>
         </is>
       </c>
-      <c r="B39" s="40" t="n">
+      <c r="B39" s="41" t="n">
         <v>478400</v>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -5450,7 +5716,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H39" s="41" t="inlineStr">
+      <c r="H39" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5462,7 +5728,7 @@
           <t>Indigo · Многоэтажки Д и Г, полная замена</t>
         </is>
       </c>
-      <c r="B40" s="40" t="n">
+      <c r="B40" s="41" t="n">
         <v>569800</v>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -5470,7 +5736,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H40" s="41" t="inlineStr">
+      <c r="H40" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 166 ед. оборудования</t>
         </is>
@@ -5482,7 +5748,7 @@
           <t>Indigo · Многоэтажки Д и Г, частичная замена</t>
         </is>
       </c>
-      <c r="B41" s="40" t="n">
+      <c r="B41" s="41" t="n">
         <v>440700</v>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -5490,7 +5756,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H41" s="41" t="inlineStr">
+      <c r="H41" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5502,7 +5768,7 @@
           <t>Indigo · Площадки А,Б,Е,Ж,В,В(РМ), полная</t>
         </is>
       </c>
-      <c r="B42" s="40" t="n">
+      <c r="B42" s="41" t="n">
         <v>2599100</v>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -5510,7 +5776,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H42" s="41" t="inlineStr">
+      <c r="H42" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 793 ед. оборудования</t>
         </is>
@@ -5522,7 +5788,7 @@
           <t>Indigo · Площадки А,Б,Е,Ж,В,В(РМ), частичная</t>
         </is>
       </c>
-      <c r="B43" s="40" t="n">
+      <c r="B43" s="41" t="n">
         <v>2010300</v>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -5530,7 +5796,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H43" s="41" t="inlineStr">
+      <c r="H43" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5542,7 +5808,7 @@
           <t>Indigo · Инкубаторий, полная замена</t>
         </is>
       </c>
-      <c r="B44" s="40" t="n">
+      <c r="B44" s="41" t="n">
         <v>126200</v>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -5550,7 +5816,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H44" s="41" t="inlineStr">
+      <c r="H44" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 48 ед. оборудования</t>
         </is>
@@ -5562,7 +5828,7 @@
           <t>Indigo · Инкубаторий, частичная замена</t>
         </is>
       </c>
-      <c r="B45" s="40" t="n">
+      <c r="B45" s="41" t="n">
         <v>106800</v>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -5570,7 +5836,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H45" s="41" t="inlineStr">
+      <c r="H45" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5582,7 +5848,7 @@
           <t>Indigo · ЗПП, полная замена</t>
         </is>
       </c>
-      <c r="B46" s="40" t="n">
+      <c r="B46" s="41" t="n">
         <v>126200</v>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -5590,7 +5856,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H46" s="41" t="inlineStr">
+      <c r="H46" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5602,7 +5868,7 @@
           <t>Indigo · ЗПП, частичная замена</t>
         </is>
       </c>
-      <c r="B47" s="40" t="n">
+      <c r="B47" s="41" t="n">
         <v>106800</v>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -5610,7 +5876,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H47" s="41" t="inlineStr">
+      <c r="H47" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5622,7 +5888,7 @@
           <t>Indigo · дезинсекция, Айыртау БП</t>
         </is>
       </c>
-      <c r="B48" s="40" t="n">
+      <c r="B48" s="41" t="n">
         <v>720000</v>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -5630,7 +5896,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H48" s="41" t="inlineStr">
+      <c r="H48" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5642,7 +5908,7 @@
           <t>Indigo · дезинсекция, Многоэтажки</t>
         </is>
       </c>
-      <c r="B49" s="40" t="n">
+      <c r="B49" s="41" t="n">
         <v>1080000</v>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -5650,7 +5916,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H49" s="41" t="inlineStr">
+      <c r="H49" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5662,7 +5928,7 @@
           <t>Indigo · дезинсекция, Площадки</t>
         </is>
       </c>
-      <c r="B50" s="40" t="n">
+      <c r="B50" s="41" t="n">
         <v>3000000</v>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -5670,7 +5936,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H50" s="41" t="inlineStr">
+      <c r="H50" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5682,7 +5948,7 @@
           <t>Indigo · дезинсекция, Инкубаторий</t>
         </is>
       </c>
-      <c r="B51" s="40" t="n">
+      <c r="B51" s="41" t="n">
         <v>100800</v>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -5690,7 +5956,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H51" s="41" t="inlineStr">
+      <c r="H51" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5702,7 +5968,7 @@
           <t>Indigo · дезинсекция, ЗПП</t>
         </is>
       </c>
-      <c r="B52" s="40" t="n">
+      <c r="B52" s="41" t="n">
         <v>160800</v>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -5710,7 +5976,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H52" s="41" t="inlineStr">
+      <c r="H52" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5722,7 +5988,7 @@
           <t>Pest Hunters · ККЗ, дератизация</t>
         </is>
       </c>
-      <c r="B53" s="40" t="n">
+      <c r="B53" s="41" t="n">
         <v>75000</v>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -5730,7 +5996,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H53" s="41" t="inlineStr">
+      <c r="H53" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -5742,7 +6008,7 @@
           <t>Pest Hunters · ККЗ, дезинсекция</t>
         </is>
       </c>
-      <c r="B54" s="40" t="n">
+      <c r="B54" s="41" t="n">
         <v>70000</v>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -5750,7 +6016,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H54" s="41" t="inlineStr">
+      <c r="H54" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -5762,7 +6028,7 @@
           <t>Pest Hunters · площадки, март — ноябрь</t>
         </is>
       </c>
-      <c r="B55" s="40" t="n">
+      <c r="B55" s="41" t="n">
         <v>3172000</v>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -5770,7 +6036,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H55" s="41" t="inlineStr">
+      <c r="H55" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); 122 объекта, оборудование подрядчика</t>
         </is>
@@ -5782,7 +6048,7 @@
           <t>Pest Hunters · площадки, декабрь — февраль</t>
         </is>
       </c>
-      <c r="B56" s="40" t="n">
+      <c r="B56" s="41" t="n">
         <v>2074000</v>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -5790,7 +6056,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H56" s="41" t="inlineStr">
+      <c r="H56" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); 122 объекта, оборудование подрядчика</t>
         </is>
@@ -5802,7 +6068,7 @@
           <t>Pest Hunters · площадки альт., март — ноябрь</t>
         </is>
       </c>
-      <c r="B57" s="40" t="n">
+      <c r="B57" s="41" t="n">
         <v>2806000</v>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -5810,7 +6076,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H57" s="41" t="inlineStr">
+      <c r="H57" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); оборудование заказчика</t>
         </is>
@@ -5822,7 +6088,7 @@
           <t>Pest Hunters · площадки альт., дек. — февраль</t>
         </is>
       </c>
-      <c r="B58" s="40" t="n">
+      <c r="B58" s="41" t="n">
         <v>1830000</v>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -5830,7 +6096,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H58" s="41" t="inlineStr">
+      <c r="H58" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); оборудование заказчика</t>
         </is>
@@ -5842,7 +6108,7 @@
           <t>Pest Hunters · ЗПП</t>
         </is>
       </c>
-      <c r="B59" s="40" t="n">
+      <c r="B59" s="41" t="n">
         <v>180000</v>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -5850,7 +6116,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H59" s="41" t="inlineStr">
+      <c r="H59" s="42" t="inlineStr">
         <is>
           <t>договор №88 от 01.01.2026; дератизация + дезинсекция, 8 309 м², 3 обхода в месяц</t>
         </is>
@@ -5862,7 +6128,7 @@
           <t>Pest Hunters · склад ТМЦ</t>
         </is>
       </c>
-      <c r="B60" s="40" t="n">
+      <c r="B60" s="41" t="n">
         <v>80000</v>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -5870,7 +6136,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H60" s="41" t="inlineStr">
+      <c r="H60" s="42" t="inlineStr">
         <is>
           <t>договор №921 от 01.04.2026; дератизация + дезинсекция, 1 обход в месяц</t>
         </is>
@@ -5882,7 +6148,7 @@
           <t>Месяцев высокого тарифа площадок (мар — ноя)</t>
         </is>
       </c>
-      <c r="B61" s="40" t="n">
+      <c r="B61" s="41" t="n">
         <v>9</v>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -5890,7 +6156,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H61" s="41" t="inlineStr">
+      <c r="H61" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -5902,7 +6168,7 @@
           <t>Месяцев низкого тарифа площадок (дек — фев)</t>
         </is>
       </c>
-      <c r="B62" s="40" t="n">
+      <c r="B62" s="41" t="n">
         <v>3</v>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -5910,7 +6176,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H62" s="41" t="inlineStr">
+      <c r="H62" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -5922,7 +6188,7 @@
           <t>Месяцев действия договора по складу ТМЦ</t>
         </is>
       </c>
-      <c r="B63" s="40" t="n">
+      <c r="B63" s="41" t="n">
         <v>9</v>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -5930,7 +6196,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H63" s="41" t="inlineStr">
+      <c r="H63" s="42" t="inlineStr">
         <is>
           <t>апрель — декабрь 2026</t>
         </is>
@@ -5942,7 +6208,7 @@
           <t>Скидка Indigo за всю территорию фабрики</t>
         </is>
       </c>
-      <c r="B64" s="43" t="n">
+      <c r="B64" s="44" t="n">
         <v>0.15</v>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -5950,7 +6216,7 @@
           <t>доля</t>
         </is>
       </c>
-      <c r="H64" s="41" t="inlineStr">
+      <c r="H64" s="42" t="inlineStr">
         <is>
           <t>КП от 19.08.2026, условия предоставления скидок</t>
         </is>
@@ -5962,7 +6228,7 @@
           <t>Скидка Indigo за 100 % предоплату за год</t>
         </is>
       </c>
-      <c r="B65" s="43" t="n">
+      <c r="B65" s="44" t="n">
         <v>0.15</v>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -5970,7 +6236,7 @@
           <t>доля</t>
         </is>
       </c>
-      <c r="H65" s="41" t="inlineStr">
+      <c r="H65" s="42" t="inlineStr">
         <is>
           <t>КП от 19.08.2026, дополнительно к предыдущей</t>
         </is>
@@ -5982,7 +6248,7 @@
           <t>Скидка Indigo неплательщику НДС</t>
         </is>
       </c>
-      <c r="B66" s="43" t="n">
+      <c r="B66" s="44" t="n">
         <v>0.16</v>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -5990,7 +6256,7 @@
           <t>доля</t>
         </is>
       </c>
-      <c r="H66" s="41" t="inlineStr">
+      <c r="H66" s="42" t="inlineStr">
         <is>
           <t>КП от 19.08.2026; цены КП уже включают НДС</t>
         </is>

</xml_diff>

<commit_message>
Show that briquettes are charged into contour 2 stations
The Pest Killer line now names the stations it fills and carries two
derived rows: the 1 198 contour-2 stations being charged and the resulting
0.017 kg per station per month, so the link between station count and
poison consumption is visible rather than implied.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLozcDkCvYTXvP2yAkyMFB
</commit_message>
<xml_diff>
--- a/reports/УКПФ_дератизация_сравнение_КП.xlsx
+++ b/reports/УКПФ_дератизация_сравнение_КП.xlsx
@@ -24,12 +24,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;—&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;×&quot;"/>
-    <numFmt numFmtId="166" formatCode="0 %"/>
-    <numFmt numFmtId="167" formatCode="#,##0;;&quot;—&quot;"/>
-    <numFmt numFmtId="168" formatCode="#,##0.0;;&quot;—&quot;"/>
+    <numFmt numFmtId="166" formatCode="#,##0.000;;&quot;—&quot;"/>
+    <numFmt numFmtId="167" formatCode="0 %"/>
+    <numFmt numFmtId="168" formatCode="#,##0;;&quot;—&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0;;&quot;—&quot;"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -213,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -254,6 +255,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -261,7 +263,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -287,25 +289,32 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -671,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -721,7 +730,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="45" t="n"/>
+      <c r="A5" s="46" t="n"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
           <t>в месяц</t>
@@ -834,7 +843,7 @@
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="E8" s="46" t="n"/>
+      <c r="E8" s="47" t="n"/>
       <c r="F8" s="7">
         <f>G8/12</f>
         <v>5276.458333</v>
@@ -871,7 +880,7 @@
           <t>нормы не заданы</t>
         </is>
       </c>
-      <c r="G9" s="46" t="n"/>
+      <c r="G9" s="47" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -884,7 +893,7 @@
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="C10" s="46" t="n"/>
+      <c r="C10" s="47" t="n"/>
       <c r="D10" s="7">
         <f>E10/12</f>
         <v>60000</v>
@@ -898,7 +907,7 @@
           <t>нормы не заданы</t>
         </is>
       </c>
-      <c r="G10" s="46" t="n"/>
+      <c r="G10" s="47" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -911,13 +920,13 @@
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="C11" s="46" t="n"/>
+      <c r="C11" s="47" t="n"/>
       <c r="D11" s="9" t="inlineStr">
         <is>
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="E11" s="46" t="n"/>
+      <c r="E11" s="47" t="n"/>
       <c r="F11" s="7">
         <f>G11/12</f>
         <v>17042.22917</v>
@@ -1077,7 +1086,7 @@
         <f>C15-G15</f>
         <v>35675696.75</v>
       </c>
-      <c r="D19" s="47">
+      <c r="D19" s="48">
         <f>IF(G15=0,0,C15/G15)</f>
         <v>3.555583381</v>
       </c>
@@ -1096,7 +1105,7 @@
         <f>E15-G15</f>
         <v>24590096.75</v>
       </c>
-      <c r="D20" s="47">
+      <c r="D20" s="48">
         <f>IF(G15=0,0,E15/G15)</f>
         <v>2.761480457</v>
       </c>
@@ -1300,7 +1309,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Pest Killer, брикеты · тёплый сезон</t>
+          <t>Pest Killer, брикеты · заряжаются в станции 2-го контура</t>
         </is>
       </c>
       <c r="B30" s="7">
@@ -1328,358 +1337,350 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">   в том числе станций 2-го контура, которые заряжаются</t>
+        </is>
+      </c>
+      <c r="B31" s="7">
+        <f>Данные!$C$33</f>
+        <v>1198</v>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   расход брикетов на одну станцию 2-го контура</t>
+        </is>
+      </c>
+      <c r="B32" s="49">
+        <f>Данные!$F$33/Данные!$C$33</f>
+        <v>0.01694490818</v>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>кг/мес</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
           <t>Бутылки · тёплый сезон</t>
         </is>
       </c>
-      <c r="B31" s="7">
+      <c r="B33" s="7">
         <f>Данные!$B$11</f>
         <v>40</v>
       </c>
-      <c r="C31" s="21" t="inlineStr">
+      <c r="C33" s="21" t="inlineStr">
         <is>
           <t>шт/мес</t>
         </is>
       </c>
-      <c r="D31" s="7">
+      <c r="D33" s="7">
         <f>Данные!$B$10</f>
         <v>68</v>
       </c>
-      <c r="E31" s="7">
+      <c r="E33" s="7">
         <f>Данные!$B$11*Данные!$B$10</f>
         <v>2720</v>
       </c>
-      <c r="F31" s="8">
+      <c r="F33" s="8">
         <f>Данные!$B$11*Данные!$B$10*Данные!$B$15</f>
         <v>19040</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>ИТОГО ТЕКУЩИЕ РАСХОДЫ ШТАТА</t>
         </is>
       </c>
-      <c r="B32" s="22" t="n"/>
-      <c r="C32" s="22" t="n"/>
-      <c r="D32" s="22" t="n"/>
-      <c r="E32" s="14">
-        <f>F32/12</f>
+      <c r="B34" s="23" t="n"/>
+      <c r="C34" s="23" t="n"/>
+      <c r="D34" s="23" t="n"/>
+      <c r="E34" s="14">
+        <f>F34/12</f>
         <v>1163325.271</v>
       </c>
-      <c r="F32" s="14">
-        <f>F26+F27+F28+F29+F30+F31</f>
+      <c r="F34" s="14">
+        <f>F26+F27+F28+F29+F30+F33</f>
         <v>13959903.25</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Приманочные станции 1-го контура · разовая закупка</t>
         </is>
       </c>
-      <c r="B33" s="7">
+      <c r="B35" s="7">
         <f>Данные!$B$33</f>
         <v>179</v>
       </c>
-      <c r="C33" s="21" t="inlineStr">
+      <c r="C35" s="21" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="D33" s="7">
+      <c r="D35" s="7">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
-      <c r="E33" s="10" t="n"/>
-      <c r="F33" s="8">
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="8">
         <f>Данные!$B$33*Данные!$B$9</f>
         <v>386640</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Приманочные станции 2-го контура · разовая закупка</t>
         </is>
       </c>
-      <c r="B34" s="7">
+      <c r="B36" s="7">
         <f>Данные!$C$33</f>
         <v>1198</v>
       </c>
-      <c r="C34" s="21" t="inlineStr">
+      <c r="C36" s="21" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="D34" s="7">
+      <c r="D36" s="7">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="8">
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="8">
         <f>Данные!$C$33*Данные!$B$9</f>
         <v>2587680</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>ИТОГО РАЗОВАЯ ЗАКУПКА ОБОРУДОВАНИЯ</t>
         </is>
       </c>
-      <c r="B35" s="12">
+      <c r="B37" s="12">
         <f>Данные!$B$33+Данные!$C$33</f>
         <v>1377</v>
       </c>
-      <c r="C35" s="23" t="inlineStr">
+      <c r="C37" s="24" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="D35" s="22" t="n"/>
-      <c r="E35" s="22" t="n"/>
-      <c r="F35" s="12">
-        <f>F33+F34</f>
+      <c r="D37" s="23" t="n"/>
+      <c r="E37" s="23" t="n"/>
+      <c r="F37" s="12">
+        <f>F35+F36</f>
         <v>2974320</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>ИТОГО ПЕРВЫЙ ГОД · с разовой закупкой</t>
         </is>
       </c>
-      <c r="B36" s="22" t="n"/>
-      <c r="C36" s="22" t="n"/>
-      <c r="D36" s="22" t="n"/>
-      <c r="E36" s="22" t="n"/>
-      <c r="F36" s="14">
-        <f>F32+F35</f>
+      <c r="B38" s="23" t="n"/>
+      <c r="C38" s="23" t="n"/>
+      <c r="D38" s="23" t="n"/>
+      <c r="E38" s="23" t="n"/>
+      <c r="F38" s="14">
+        <f>F34+F37</f>
         <v>16934223.25</v>
       </c>
     </row>
-    <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="24" t="inlineStr">
+    <row r="39" ht="26" customHeight="1">
+      <c r="A39" s="25" t="inlineStr">
         <is>
           <t>Материалы от численности не зависят: норма ядов и станций привязана к точкам, а не к людям. Каждый дополнительный дератизатор добавляет только фонд оплаты труда.</t>
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39">
-      <c r="A39" s="15" t="inlineStr">
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>СКИДКИ INDIGO ИЗ КП ОТ 19.08.2026</t>
         </is>
       </c>
-      <c r="B39" s="16" t="n"/>
-      <c r="C39" s="16" t="n"/>
-      <c r="D39" s="16" t="n"/>
-      <c r="E39" s="16" t="n"/>
-      <c r="F39" s="16" t="n"/>
-      <c r="G39" s="16" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+      <c r="B41" s="16" t="n"/>
+      <c r="C41" s="16" t="n"/>
+      <c r="D41" s="16" t="n"/>
+      <c r="E41" s="16" t="n"/>
+      <c r="F41" s="16" t="n"/>
+      <c r="G41" s="16" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>Условие</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>в месяц</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>за год</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>Ставка</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Цена КП без скидок</t>
         </is>
       </c>
-      <c r="B41" s="7">
-        <f>C41/12</f>
+      <c r="B43" s="7">
+        <f>C43/12</f>
         <v>4136300</v>
       </c>
-      <c r="C41" s="8">
+      <c r="C43" s="8">
         <f>C15</f>
         <v>49635600</v>
       </c>
-      <c r="D41" s="10" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="D43" s="10" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>Вся территория фабрики</t>
         </is>
       </c>
-      <c r="B42" s="7">
-        <f>C42/12</f>
+      <c r="B44" s="7">
+        <f>C44/12</f>
         <v>3515855</v>
       </c>
-      <c r="C42" s="8">
+      <c r="C44" s="8">
         <f>C15*(1-Данные!$B$64)</f>
         <v>42190260</v>
       </c>
-      <c r="D42" s="25">
+      <c r="D44" s="50">
         <f>Данные!$B$64</f>
         <v>0.15</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>Вся территория + 100 % предоплата</t>
         </is>
       </c>
-      <c r="B43" s="7">
-        <f>C43/12</f>
+      <c r="B45" s="7">
+        <f>C45/12</f>
         <v>2988476.75</v>
       </c>
-      <c r="C43" s="8">
+      <c r="C45" s="8">
         <f>C15*(1-Данные!$B$64)*(1-Данные!$B$65)</f>
         <v>35861721</v>
       </c>
-      <c r="D43" s="25">
+      <c r="D45" s="50">
         <f>Данные!$B$65</f>
         <v>0.15</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>Вся территория + предоплата + неплательщик НДС</t>
         </is>
       </c>
-      <c r="B44" s="7">
-        <f>C44/12</f>
+      <c r="B46" s="7">
+        <f>C46/12</f>
         <v>2510320.47</v>
       </c>
-      <c r="C44" s="8">
+      <c r="C46" s="8">
         <f>C15*(1-Данные!$B$64)*(1-Данные!$B$65)*(1-Данные!$B$66)</f>
         <v>30123845.64</v>
       </c>
-      <c r="D44" s="25">
+      <c r="D46" s="50">
         <f>Данные!$B$66</f>
         <v>0.16</v>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46">
-      <c r="A46" s="15" t="inlineStr">
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>ПЕРИОДИЧНОСТЬ ОБХОДОВ</t>
         </is>
       </c>
-      <c r="B46" s="16" t="n"/>
-      <c r="C46" s="16" t="n"/>
-      <c r="D46" s="16" t="n"/>
-      <c r="E46" s="16" t="n"/>
-      <c r="F46" s="16" t="n"/>
-      <c r="G46" s="16" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="26" t="inlineStr">
+      <c r="B48" s="16" t="n"/>
+      <c r="C48" s="16" t="n"/>
+      <c r="D48" s="16" t="n"/>
+      <c r="E48" s="16" t="n"/>
+      <c r="F48" s="16" t="n"/>
+      <c r="G48" s="16" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
         <is>
           <t>Вариант</t>
         </is>
       </c>
-      <c r="B47" s="26" t="inlineStr">
+      <c r="B49" s="27" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="C47" s="26" t="inlineStr">
+      <c r="C49" s="27" t="inlineStr">
         <is>
           <t>Обходов в месяц</t>
         </is>
       </c>
-      <c r="D47" s="26" t="inlineStr">
+      <c r="D49" s="27" t="inlineStr">
         <is>
           <t>Что зафиксировано в документах</t>
         </is>
       </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>Indigo Solutions</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>все объекты</t>
-        </is>
-      </c>
-      <c r="C48" s="21" t="inlineStr">
-        <is>
-          <t>в КП не указана</t>
-        </is>
-      </c>
-      <c r="D48" s="27" t="inlineStr">
-        <is>
-          <t>ответ по заявке ≤ 2 ч, выезд ≤ 24 ч, вызовы без ограничений</t>
-        </is>
-      </c>
-      <c r="E48" s="48" t="n"/>
-      <c r="F48" s="48" t="n"/>
-      <c r="G48" s="46" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>Pest Hunters</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>ККЗ</t>
-        </is>
-      </c>
-      <c r="C49" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="27" t="inlineStr">
-        <is>
-          <t>выезд по запросу</t>
-        </is>
-      </c>
-      <c r="E49" s="48" t="n"/>
-      <c r="F49" s="48" t="n"/>
-      <c r="G49" s="46" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Pest Hunters</t>
+          <t>Indigo Solutions</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>бройлерные площадки</t>
-        </is>
-      </c>
-      <c r="C50" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="27" t="inlineStr">
-        <is>
-          <t>дополнительные визиты по вызову</t>
-        </is>
-      </c>
-      <c r="E50" s="48" t="n"/>
-      <c r="F50" s="48" t="n"/>
-      <c r="G50" s="46" t="n"/>
+          <t>все объекты</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>в КП не указана</t>
+        </is>
+      </c>
+      <c r="D50" s="28" t="inlineStr">
+        <is>
+          <t>ответ по заявке ≤ 2 ч, выезд ≤ 24 ч, вызовы без ограничений</t>
+        </is>
+      </c>
+      <c r="E50" s="51" t="n"/>
+      <c r="F50" s="51" t="n"/>
+      <c r="G50" s="47" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -1689,20 +1690,20 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>ЗПП</t>
+          <t>ККЗ</t>
         </is>
       </c>
       <c r="C51" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="D51" s="27" t="inlineStr">
-        <is>
-          <t>по графику на 2026 год, бригада из трёх человек</t>
-        </is>
-      </c>
-      <c r="E51" s="48" t="n"/>
-      <c r="F51" s="48" t="n"/>
-      <c r="G51" s="46" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D51" s="28" t="inlineStr">
+        <is>
+          <t>выезд по запросу</t>
+        </is>
+      </c>
+      <c r="E51" s="51" t="n"/>
+      <c r="F51" s="51" t="n"/>
+      <c r="G51" s="47" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -1712,64 +1713,110 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>склад ТМЦ</t>
+          <t>бройлерные площадки</t>
         </is>
       </c>
       <c r="C52" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="D52" s="27" t="inlineStr">
-        <is>
-          <t>выезд по рекламации за два рабочих дня</t>
-        </is>
-      </c>
-      <c r="E52" s="48" t="n"/>
-      <c r="F52" s="48" t="n"/>
-      <c r="G52" s="46" t="n"/>
+      <c r="D52" s="28" t="inlineStr">
+        <is>
+          <t>дополнительные визиты по вызову</t>
+        </is>
+      </c>
+      <c r="E52" s="51" t="n"/>
+      <c r="F52" s="51" t="n"/>
+      <c r="G52" s="47" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
+          <t>Pest Hunters</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>ЗПП</t>
+        </is>
+      </c>
+      <c r="C53" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" s="28" t="inlineStr">
+        <is>
+          <t>по графику на 2026 год, бригада из трёх человек</t>
+        </is>
+      </c>
+      <c r="E53" s="51" t="n"/>
+      <c r="F53" s="51" t="n"/>
+      <c r="G53" s="47" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Pest Hunters</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>склад ТМЦ</t>
+        </is>
+      </c>
+      <c r="C54" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="28" t="inlineStr">
+        <is>
+          <t>выезд по рекламации за два рабочих дня</t>
+        </is>
+      </c>
+      <c r="E54" s="51" t="n"/>
+      <c r="F54" s="51" t="n"/>
+      <c r="G54" s="47" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>все объекты</t>
         </is>
       </c>
-      <c r="C53" s="21" t="n">
+      <c r="C55" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="D53" s="27" t="inlineStr">
+      <c r="D55" s="28" t="inlineStr">
         <is>
           <t>присутствие 5/2, реакция в тот же день</t>
         </is>
       </c>
-      <c r="E53" s="48" t="n"/>
-      <c r="F53" s="48" t="n"/>
-      <c r="G53" s="46" t="n"/>
+      <c r="E55" s="51" t="n"/>
+      <c r="F55" s="51" t="n"/>
+      <c r="G55" s="47" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="D48:G48"/>
+    <mergeCell ref="D54:G54"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="D11:E11"/>
+    <mergeCell ref="A39:G39"/>
     <mergeCell ref="D50:G50"/>
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="D53:G53"/>
-    <mergeCell ref="B10:C10"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D49:G49"/>
+    <mergeCell ref="D55:G55"/>
     <mergeCell ref="D51:G51"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1798,7 +1845,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>Кормоцех. Indigo — КП от 19.08.2026, цены с НДС. Pest Hunters — КП №26/12, без НДС. Штат УКПФ — 29 приманочных станций 2-го контура, 1 кг брикетов Pest Killer на обработку.</t>
         </is>
@@ -1806,37 +1853,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="30">
+      <c r="B5" s="31">
         <f>D9</f>
         <v>1159200</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="31">
         <f>D10</f>
         <v>900000</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="31">
         <f>D11+D12+D13+D14</f>
         <v>25497.5</v>
       </c>
@@ -1875,16 +1922,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · барьер вокруг периметра кормоцеха и грязный барьер</t>
         </is>
       </c>
-      <c r="B9" s="32">
+      <c r="B9" s="33">
         <f>Данные!$B$37</f>
         <v>96600</v>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="8">
@@ -1893,16 +1940,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters · дератизация</t>
         </is>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="33">
         <f>Данные!$B$53</f>
         <v>75000</v>
       </c>
-      <c r="C10" s="32" t="n">
+      <c r="C10" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="8">
@@ -1911,16 +1958,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
         </is>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="33">
         <f>Данные!$D$20*Данные!$B$8</f>
         <v>0</v>
       </c>
-      <c r="C11" s="32">
+      <c r="C11" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -1930,16 +1977,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
         </is>
       </c>
-      <c r="B12" s="32">
+      <c r="B12" s="33">
         <f>Данные!$D$20*2*Данные!$B$8</f>
         <v>0</v>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="33">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
@@ -1949,16 +1996,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Зерноцид, 2-й контур</t>
         </is>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="33">
         <f>Данные!$G$20*Данные!$B$6</f>
         <v>0</v>
       </c>
-      <c r="C13" s="32">
+      <c r="C13" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -1968,16 +2015,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B14" s="32">
+      <c r="B14" s="33">
         <f>Данные!$F$20*Данные!$B$7</f>
         <v>3642.5</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -1987,7 +2034,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C15" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2031,16 +2078,16 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B19" s="32">
+      <c r="B19" s="33">
         <f>Данные!$B$20*Данные!$B$9</f>
         <v>0</v>
       </c>
-      <c r="C19" s="32" t="n">
+      <c r="C19" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="7">
@@ -2049,16 +2096,16 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="33">
         <f>Данные!$C$20*Данные!$B$9</f>
         <v>62640</v>
       </c>
-      <c r="C20" s="32" t="n">
+      <c r="C20" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="7">
@@ -2067,7 +2114,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="33" t="inlineStr">
+      <c r="C21" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2111,16 +2158,16 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="A25" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters · дезинсекция</t>
         </is>
       </c>
-      <c r="B25" s="32">
+      <c r="B25" s="33">
         <f>Данные!$B$54</f>
         <v>70000</v>
       </c>
-      <c r="C25" s="32" t="n">
+      <c r="C25" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D25" s="7">
@@ -2129,7 +2176,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="33" t="inlineStr">
+      <c r="C26" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2141,14 +2188,14 @@
     </row>
     <row r="27"/>
     <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="24" t="inlineStr">
+      <c r="A28" s="25" t="inlineStr">
         <is>
           <t>Зерноцид по ККЗ в нормах не заявлен, поэтому строка Зерноцида даёт ноль.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="24" t="inlineStr">
+      <c r="A29" s="25" t="inlineStr">
         <is>
           <t>Зарплата дератизаторов по объектам не делится — она на листе «Штат УКПФ».</t>
         </is>
@@ -2187,7 +2234,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>Восемь площадок: А, Б, В (Восточка), Г, Д, Е, Ж, Айыртау. У Indigo они разбиты на три группы, у Pest Hunters — 122 объекта с сезонным тарифом.</t>
         </is>
@@ -2195,37 +2242,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="30">
+      <c r="B5" s="31">
         <f>D9+D10+D11</f>
         <v>45447600</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="31">
         <f>D12+D13</f>
         <v>34770000</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="31">
         <f>D14+D15+D16+D17</f>
         <v>1240117.5</v>
       </c>
@@ -2264,16 +2311,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Айыртау БП (БП-12, БП-13, БП-14) — полная замена, 180 ед.</t>
         </is>
       </c>
-      <c r="B9" s="32">
+      <c r="B9" s="33">
         <f>Данные!$B$38</f>
         <v>618400</v>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="8">
@@ -2282,16 +2329,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Многоэтажки, площадки Д и Г — полная замена, 166 ед.</t>
         </is>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="33">
         <f>Данные!$B$40</f>
         <v>569800</v>
       </c>
-      <c r="C10" s="32" t="n">
+      <c r="C10" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="8">
@@ -2300,16 +2347,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (рем. молод), В — полная замена, 793 ед.</t>
         </is>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="33">
         <f>Данные!$B$42</f>
         <v>2599100</v>
       </c>
-      <c r="C11" s="32" t="n">
+      <c r="C11" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D11" s="8">
@@ -2318,16 +2365,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters · 122 объекта, март — ноябрь, оборудование подрядчика</t>
         </is>
       </c>
-      <c r="B12" s="32">
+      <c r="B12" s="33">
         <f>Данные!$B$55</f>
         <v>3172000</v>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="33">
         <f>Данные!$B$61</f>
         <v>9</v>
       </c>
@@ -2337,16 +2384,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters · 122 объекта, декабрь — февраль, оборудование подрядчика</t>
         </is>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="33">
         <f>Данные!$B$56</f>
         <v>2074000</v>
       </c>
-      <c r="C13" s="32">
+      <c r="C13" s="33">
         <f>Данные!$B$62</f>
         <v>3</v>
       </c>
@@ -2356,16 +2403,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
         </is>
       </c>
-      <c r="B14" s="32">
+      <c r="B14" s="33">
         <f>SUM(Данные!$D$23:$D$30)*Данные!$B$8</f>
         <v>42880</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2375,16 +2422,16 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
         </is>
       </c>
-      <c r="B15" s="32">
+      <c r="B15" s="33">
         <f>SUM(Данные!$D$23:$D$30)*2*Данные!$B$8</f>
         <v>85760</v>
       </c>
-      <c r="C15" s="32">
+      <c r="C15" s="33">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
@@ -2394,16 +2441,16 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Зерноцид, 2-й контур</t>
         </is>
       </c>
-      <c r="B16" s="32">
+      <c r="B16" s="33">
         <f>SUM(Данные!$G$23:$G$30)*Данные!$B$6</f>
         <v>11100</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2413,16 +2460,16 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B17" s="32">
+      <c r="B17" s="33">
         <f>SUM(Данные!$F$23:$F$30)*Данные!$B$7</f>
         <v>61922.5</v>
       </c>
-      <c r="C17" s="32">
+      <c r="C17" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2432,7 +2479,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="33" t="inlineStr">
+      <c r="C18" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2476,16 +2523,16 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="31" t="inlineStr">
+      <c r="A22" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Айыртау БП — частичная замена</t>
         </is>
       </c>
-      <c r="B22" s="32">
+      <c r="B22" s="33">
         <f>Данные!$B$39</f>
         <v>478400</v>
       </c>
-      <c r="C22" s="32" t="n">
+      <c r="C22" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D22" s="7">
@@ -2494,16 +2541,16 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Многоэтажки Д и Г — частичная замена</t>
         </is>
       </c>
-      <c r="B23" s="32">
+      <c r="B23" s="33">
         <f>Данные!$B$41</f>
         <v>440700</v>
       </c>
-      <c r="C23" s="32" t="n">
+      <c r="C23" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D23" s="7">
@@ -2512,16 +2559,16 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (РМ), В — частичная замена</t>
         </is>
       </c>
-      <c r="B24" s="32">
+      <c r="B24" s="33">
         <f>Данные!$B$43</f>
         <v>2010300</v>
       </c>
-      <c r="C24" s="32" t="n">
+      <c r="C24" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D24" s="7">
@@ -2530,16 +2577,16 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="A25" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters · 122 объекта, март — ноябрь, оборудование заказчика</t>
         </is>
       </c>
-      <c r="B25" s="32">
+      <c r="B25" s="33">
         <f>Данные!$B$57</f>
         <v>2806000</v>
       </c>
-      <c r="C25" s="32">
+      <c r="C25" s="33">
         <f>Данные!$B$61</f>
         <v>9</v>
       </c>
@@ -2549,16 +2596,16 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="31" t="inlineStr">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters · 122 объекта, декабрь — февраль, оборудование заказчика</t>
         </is>
       </c>
-      <c r="B26" s="32">
+      <c r="B26" s="33">
         <f>Данные!$B$58</f>
         <v>1830000</v>
       </c>
-      <c r="C26" s="32">
+      <c r="C26" s="33">
         <f>Данные!$B$62</f>
         <v>3</v>
       </c>
@@ -2568,7 +2615,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="C27" s="33" t="inlineStr">
+      <c r="C27" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2612,16 +2659,16 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="31" t="inlineStr">
+      <c r="A31" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B31" s="32">
+      <c r="B31" s="33">
         <f>SUM(Данные!$B$23:$B$30)*Данные!$B$9</f>
         <v>347760</v>
       </c>
-      <c r="C31" s="32" t="n">
+      <c r="C31" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="7">
@@ -2630,16 +2677,16 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="31" t="inlineStr">
+      <c r="A32" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B32" s="32">
+      <c r="B32" s="33">
         <f>SUM(Данные!$C$23:$C$30)*Данные!$B$9</f>
         <v>2367360</v>
       </c>
-      <c r="C32" s="32" t="n">
+      <c r="C32" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="7">
@@ -2648,7 +2695,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="C33" s="33" t="inlineStr">
+      <c r="C33" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2692,16 +2739,16 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="31" t="inlineStr">
+      <c r="A37" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Айыртау БП</t>
         </is>
       </c>
-      <c r="B37" s="32">
+      <c r="B37" s="33">
         <f>Данные!$B$48</f>
         <v>720000</v>
       </c>
-      <c r="C37" s="32" t="n">
+      <c r="C37" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D37" s="7">
@@ -2710,16 +2757,16 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="31" t="inlineStr">
+      <c r="A38" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Многоэтажки Д и Г</t>
         </is>
       </c>
-      <c r="B38" s="32">
+      <c r="B38" s="33">
         <f>Данные!$B$49</f>
         <v>1080000</v>
       </c>
-      <c r="C38" s="32" t="n">
+      <c r="C38" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D38" s="7">
@@ -2728,16 +2775,16 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="31" t="inlineStr">
+      <c r="A39" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (РМ), В</t>
         </is>
       </c>
-      <c r="B39" s="32">
+      <c r="B39" s="33">
         <f>Данные!$B$50</f>
         <v>3000000</v>
       </c>
-      <c r="C39" s="32" t="n">
+      <c r="C39" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D39" s="7">
@@ -2746,7 +2793,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="33" t="inlineStr">
+      <c r="C40" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -2758,14 +2805,14 @@
     </row>
     <row r="41"/>
     <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="24" t="inlineStr">
+      <c r="A42" s="25" t="inlineStr">
         <is>
           <t>Состав площадок у Indigo и в нашем расчёте описан по-разному: у них шесть напольных площадок плюс «В (рем. молод)», у нас восемь площадок по контурам. Сопоставлять построчно нельзя, только суммарно.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="24" t="inlineStr">
+      <c r="A43" s="25" t="inlineStr">
         <is>
           <t>Разовая закупка приманочных станций 1-го и 2-го контура показана справочно и в годовой итог не входит.</t>
         </is>
@@ -2804,7 +2851,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>У Indigo появился в КП от 19.08.2026: 48 ед. оборудования. У Pest Hunters предложения нет.</t>
         </is>
@@ -2812,37 +2859,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="30">
+      <c r="B5" s="31">
         <f>D9</f>
         <v>1514400</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="31">
         <f>D10</f>
         <v>0</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="31">
         <f>D11+D12+D13+D14</f>
         <v>63317.5</v>
       </c>
@@ -2881,16 +2928,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · полная замена оборудования, 48 ед.</t>
         </is>
       </c>
-      <c r="B9" s="32">
+      <c r="B9" s="33">
         <f>Данные!$B$44</f>
         <v>126200</v>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="8">
@@ -2899,15 +2946,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B10" s="32" t="n">
+      <c r="B10" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="32" t="n">
+      <c r="C10" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="8">
@@ -2916,16 +2963,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
         </is>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="33">
         <f>Данные!$D$21*Данные!$B$8</f>
         <v>1920</v>
       </c>
-      <c r="C11" s="32">
+      <c r="C11" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2935,16 +2982,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
         </is>
       </c>
-      <c r="B12" s="32">
+      <c r="B12" s="33">
         <f>Данные!$D$21*2*Данные!$B$8</f>
         <v>3840</v>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="33">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
@@ -2954,16 +3001,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Зерноцид, 2-й контур</t>
         </is>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="33">
         <f>Данные!$G$21*Данные!$B$6</f>
         <v>740</v>
       </c>
-      <c r="C13" s="32">
+      <c r="C13" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2973,16 +3020,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B14" s="32">
+      <c r="B14" s="33">
         <f>Данные!$F$21*Данные!$B$7</f>
         <v>3642.5</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -2992,7 +3039,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C15" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3036,16 +3083,16 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · частичная замена оборудования</t>
         </is>
       </c>
-      <c r="B19" s="32">
+      <c r="B19" s="33">
         <f>Данные!$B$45</f>
         <v>106800</v>
       </c>
-      <c r="C19" s="32" t="n">
+      <c r="C19" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D19" s="7">
@@ -3054,7 +3101,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="C20" s="33" t="inlineStr">
+      <c r="C20" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3098,16 +3145,16 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B24" s="32">
+      <c r="B24" s="33">
         <f>Данные!$B$21*Данные!$B$9</f>
         <v>38880</v>
       </c>
-      <c r="C24" s="32" t="n">
+      <c r="C24" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="7">
@@ -3116,16 +3163,16 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="A25" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B25" s="32">
+      <c r="B25" s="33">
         <f>Данные!$C$21*Данные!$B$9</f>
         <v>73440</v>
       </c>
-      <c r="C25" s="32" t="n">
+      <c r="C25" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="7">
@@ -3134,7 +3181,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="33" t="inlineStr">
+      <c r="C26" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3178,16 +3225,16 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="31" t="inlineStr">
+      <c r="A30" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · дезинсекция</t>
         </is>
       </c>
-      <c r="B30" s="32">
+      <c r="B30" s="33">
         <f>Данные!$B$51</f>
         <v>100800</v>
       </c>
-      <c r="C30" s="32" t="n">
+      <c r="C30" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D30" s="7">
@@ -3196,7 +3243,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="C31" s="33" t="inlineStr">
+      <c r="C31" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3208,7 +3255,7 @@
     </row>
     <row r="32"/>
     <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="24" t="inlineStr">
+      <c r="A33" s="25" t="inlineStr">
         <is>
           <t>Нормы штата по инкубаторию: 18 точек 1-го контура, 34 второго, 12 клеевых третьего; 1 кг брикетов Pest Killer и 1 кг Зерноцида на обработку.</t>
         </is>
@@ -3246,7 +3293,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>Завод по переработке птицы, 8 309 м². У Pest Hunters — подписанный договор №88, цена включает дезинсекцию. У Indigo — предложение из КП от 19.08.2026.</t>
         </is>
@@ -3254,37 +3301,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="30">
+      <c r="B5" s="31">
         <f>D9</f>
         <v>1514400</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="31">
         <f>D10</f>
         <v>2160000</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="31">
         <f>D11</f>
         <v>0</v>
       </c>
@@ -3323,16 +3370,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · полная замена оборудования</t>
         </is>
       </c>
-      <c r="B9" s="32">
+      <c r="B9" s="33">
         <f>Данные!$B$46</f>
         <v>126200</v>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="8">
@@ -3341,16 +3388,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters · договор №88 от 01.01.2026: дератизация и дезинсекция вместе</t>
         </is>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="33">
         <f>Данные!$B$59</f>
         <v>180000</v>
       </c>
-      <c r="C10" s="32" t="n">
+      <c r="C10" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D10" s="8">
@@ -3359,15 +3406,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · нормы расхода по ЗПП не заданы</t>
         </is>
       </c>
-      <c r="B11" s="32" t="n">
+      <c r="B11" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="32" t="n">
+      <c r="C11" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="8">
@@ -3376,7 +3423,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C12" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3420,16 +3467,16 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · частичная замена оборудования</t>
         </is>
       </c>
-      <c r="B16" s="32">
+      <c r="B16" s="33">
         <f>Данные!$B$47</f>
         <v>106800</v>
       </c>
-      <c r="C16" s="32" t="n">
+      <c r="C16" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D16" s="7">
@@ -3438,7 +3485,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="33" t="inlineStr">
+      <c r="C17" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3482,16 +3529,16 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · дезинсекция</t>
         </is>
       </c>
-      <c r="B21" s="32">
+      <c r="B21" s="33">
         <f>Данные!$B$52</f>
         <v>160800</v>
       </c>
-      <c r="C21" s="32" t="n">
+      <c r="C21" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D21" s="7">
@@ -3500,7 +3547,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="33" t="inlineStr">
+      <c r="C22" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3512,14 +3559,14 @@
     </row>
     <row r="23"/>
     <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>Строки не полностью сопоставимы: у Pest Hunters 180 000 ₸ включают и дератизацию, и дезинсекцию, у Indigo эти услуги разделены — 126 200 ₸ дератизация и 160 800 ₸ дезинсекция.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>По штату УКПФ нормы расхода на ЗПП не заданы, поэтому в расчёте ноль.</t>
         </is>
@@ -3558,7 +3605,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>Договор №921 от 01.04.2026, действует с апреля по декабрь. Предложений от Indigo по этому объекту нет.</t>
         </is>
@@ -3566,37 +3613,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="30">
+      <c r="B5" s="31">
         <f>D9</f>
         <v>0</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="31">
         <f>D10</f>
         <v>720000</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="31">
         <f>D11</f>
         <v>0</v>
       </c>
@@ -3635,15 +3682,15 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="B9" s="32" t="n">
+      <c r="B9" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="8">
@@ -3652,16 +3699,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters · договор №921: дератизация и дезинсекция, выезд по рекламации за 2 рабочих дня</t>
         </is>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="33">
         <f>Данные!$B$60</f>
         <v>80000</v>
       </c>
-      <c r="C10" s="32">
+      <c r="C10" s="33">
         <f>Данные!$B$63</f>
         <v>9</v>
       </c>
@@ -3671,15 +3718,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · нормы расхода по складу не заданы</t>
         </is>
       </c>
-      <c r="B11" s="32" t="n">
+      <c r="B11" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="32" t="n">
+      <c r="C11" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="8">
@@ -3688,7 +3735,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C12" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3700,7 +3747,7 @@
     </row>
     <row r="13"/>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>С января по март договор не действует, поэтому в году девять оплачиваемых месяцев.</t>
         </is>
@@ -3738,7 +3785,7 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>Административно-бытовые корпуса на одиннадцати площадках. Ни у Indigo, ни у Pest Hunters отдельной строки по АБК нет.</t>
         </is>
@@ -3746,37 +3793,37 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>ЗА ГОД, ₸</t>
         </is>
       </c>
-      <c r="B4" s="29" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Штат УКПФ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="30">
+      <c r="B5" s="31">
         <f>D9</f>
         <v>0</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="31">
         <f>D10</f>
         <v>0</v>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="31">
         <f>D11+D12+D13+D14</f>
         <v>204506.75</v>
       </c>
@@ -3815,15 +3862,15 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions</t>
         </is>
       </c>
-      <c r="B9" s="32" t="n">
+      <c r="B9" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="8">
@@ -3832,15 +3879,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters</t>
         </is>
       </c>
-      <c r="B10" s="32" t="n">
+      <c r="B10" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="32" t="n">
+      <c r="C10" s="33" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="8">
@@ -3849,16 +3896,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, тёплый сезон</t>
         </is>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="33">
         <f>Данные!$D$22*Данные!$B$8</f>
         <v>10080</v>
       </c>
-      <c r="C11" s="32">
+      <c r="C11" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -3868,16 +3915,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Клеевые станции 3-го контура, зимний сезон — объём вдвое</t>
         </is>
       </c>
-      <c r="B12" s="32">
+      <c r="B12" s="33">
         <f>Данные!$D$22*2*Данные!$B$8</f>
         <v>20160</v>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="33">
         <f>Данные!$B$16</f>
         <v>5</v>
       </c>
@@ -3887,16 +3934,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Зерноцид, 2-й контур</t>
         </is>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="33">
         <f>Данные!$G$22*Данные!$B$6</f>
         <v>0</v>
       </c>
-      <c r="C13" s="32">
+      <c r="C13" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -3906,16 +3953,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B14" s="32">
+      <c r="B14" s="33">
         <f>Данные!$F$22*Данные!$B$7</f>
         <v>4735.25</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="33">
         <f>Данные!$B$15</f>
         <v>7</v>
       </c>
@@ -3925,7 +3972,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C15" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -3969,16 +4016,16 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B19" s="32">
+      <c r="B19" s="33">
         <f>Данные!$B$22*Данные!$B$9</f>
         <v>0</v>
       </c>
-      <c r="C19" s="32" t="n">
+      <c r="C19" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="7">
@@ -3987,16 +4034,16 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="33">
         <f>Данные!$C$22*Данные!$B$9</f>
         <v>84240</v>
       </c>
-      <c r="C20" s="32" t="n">
+      <c r="C20" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="7">
@@ -4005,7 +4052,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="33" t="inlineStr">
+      <c r="C21" s="34" t="inlineStr">
         <is>
           <t>Итого</t>
         </is>
@@ -4017,14 +4064,14 @@
     </row>
     <row r="22"/>
     <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="25" t="inlineStr">
         <is>
           <t>Клеевые станции по корпусам: Б — 11, Ж — 5, Е — 6, В — 6, В (РМ) — 6, Д — 3, Г — 3, БП-12 — 6, БП-13 — 6, БП-14 — 6, А — 5. Приманочные: 4, 2, 3, 3, 3, 4, 3, 5, 5, 5, 2.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>Норма 1,3 кг брикетов Pest Killer по АБК — приблизительная оценка, требует подтверждения. Зерноцид по АБК не заявлен.</t>
         </is>
@@ -4087,17 +4134,17 @@
       <c r="E4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Показатель, ₸</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>Оклад 258 488 ₸</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Оклад 350 000 ₸</t>
         </is>
@@ -4149,7 +4196,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="34" t="inlineStr">
+      <c r="A9" s="35" t="inlineStr">
         <is>
           <t>Зарплата за год</t>
         </is>
@@ -4180,47 +4227,47 @@
       <c r="I11" s="16" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="35" t="inlineStr">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B12" s="36" t="inlineStr">
+      <c r="B12" s="37" t="inlineStr">
         <is>
           <t>Клеевых 3-го к., шт/мес лето</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
+      <c r="C12" s="37" t="inlineStr">
         <is>
           <t>Клеевых 3-го к., шт/мес зима</t>
         </is>
       </c>
-      <c r="D12" s="36" t="inlineStr">
+      <c r="D12" s="37" t="inlineStr">
         <is>
           <t>Клеевые за год, ₸</t>
         </is>
       </c>
-      <c r="E12" s="36" t="inlineStr">
+      <c r="E12" s="37" t="inlineStr">
         <is>
           <t>Зерноцид, кг/мес</t>
         </is>
       </c>
-      <c r="F12" s="36" t="inlineStr">
+      <c r="F12" s="37" t="inlineStr">
         <is>
           <t>Зерноцид за год, ₸</t>
         </is>
       </c>
-      <c r="G12" s="36" t="inlineStr">
+      <c r="G12" s="37" t="inlineStr">
         <is>
           <t>Pest Killer, кг/мес</t>
         </is>
       </c>
-      <c r="H12" s="36" t="inlineStr">
+      <c r="H12" s="37" t="inlineStr">
         <is>
           <t>Pest Killer за год, ₸</t>
         </is>
       </c>
-      <c r="I12" s="36" t="inlineStr">
+      <c r="I12" s="37" t="inlineStr">
         <is>
           <t>Материалы за год, ₸</t>
         </is>
@@ -4232,11 +4279,11 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B13" s="37">
+      <c r="B13" s="52">
         <f>Данные!$D$20</f>
         <v>0</v>
       </c>
-      <c r="C13" s="37">
+      <c r="C13" s="52">
         <f>Данные!$D$20*2</f>
         <v>0</v>
       </c>
@@ -4244,7 +4291,7 @@
         <f>B13*Данные!$B$8*Данные!$B$15+C13*Данные!$B$8*Данные!$B$16</f>
         <v>0</v>
       </c>
-      <c r="E13" s="49">
+      <c r="E13" s="53">
         <f>Данные!$G$20</f>
         <v>0</v>
       </c>
@@ -4252,7 +4299,7 @@
         <f>E13*Данные!$B$6*Данные!$B$15</f>
         <v>0</v>
       </c>
-      <c r="G13" s="49">
+      <c r="G13" s="53">
         <f>Данные!$F$20</f>
         <v>1</v>
       </c>
@@ -4271,11 +4318,11 @@
           <t>Бройлерные площадки · 8 шт</t>
         </is>
       </c>
-      <c r="B14" s="37">
+      <c r="B14" s="52">
         <f>SUM(Данные!$D$23:$D$30)</f>
         <v>268</v>
       </c>
-      <c r="C14" s="37">
+      <c r="C14" s="52">
         <f>SUM(Данные!$D$23:$D$30)*2</f>
         <v>536</v>
       </c>
@@ -4283,7 +4330,7 @@
         <f>B14*Данные!$B$8*Данные!$B$15+C14*Данные!$B$8*Данные!$B$16</f>
         <v>728960</v>
       </c>
-      <c r="E14" s="49">
+      <c r="E14" s="53">
         <f>SUM(Данные!$G$23:$G$30)</f>
         <v>15</v>
       </c>
@@ -4291,7 +4338,7 @@
         <f>E14*Данные!$B$6*Данные!$B$15</f>
         <v>77700</v>
       </c>
-      <c r="G14" s="49">
+      <c r="G14" s="53">
         <f>SUM(Данные!$F$23:$F$30)</f>
         <v>17</v>
       </c>
@@ -4310,11 +4357,11 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B15" s="37">
+      <c r="B15" s="52">
         <f>Данные!$D$21</f>
         <v>12</v>
       </c>
-      <c r="C15" s="37">
+      <c r="C15" s="52">
         <f>Данные!$D$21*2</f>
         <v>24</v>
       </c>
@@ -4322,7 +4369,7 @@
         <f>B15*Данные!$B$8*Данные!$B$15+C15*Данные!$B$8*Данные!$B$16</f>
         <v>32640</v>
       </c>
-      <c r="E15" s="49">
+      <c r="E15" s="53">
         <f>Данные!$G$21</f>
         <v>1</v>
       </c>
@@ -4330,7 +4377,7 @@
         <f>E15*Данные!$B$6*Данные!$B$15</f>
         <v>5180</v>
       </c>
-      <c r="G15" s="49">
+      <c r="G15" s="53">
         <f>Данные!$F$21</f>
         <v>1</v>
       </c>
@@ -4349,11 +4396,11 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B16" s="37">
+      <c r="B16" s="52">
         <f>Данные!$D$22</f>
         <v>63</v>
       </c>
-      <c r="C16" s="37">
+      <c r="C16" s="52">
         <f>Данные!$D$22*2</f>
         <v>126</v>
       </c>
@@ -4361,7 +4408,7 @@
         <f>B16*Данные!$B$8*Данные!$B$15+C16*Данные!$B$8*Данные!$B$16</f>
         <v>171360</v>
       </c>
-      <c r="E16" s="49">
+      <c r="E16" s="53">
         <f>Данные!$G$22</f>
         <v>0</v>
       </c>
@@ -4369,7 +4416,7 @@
         <f>E16*Данные!$B$6*Данные!$B$15</f>
         <v>0</v>
       </c>
-      <c r="G16" s="49">
+      <c r="G16" s="53">
         <f>Данные!$F$22</f>
         <v>1.3</v>
       </c>
@@ -4406,13 +4453,13 @@
           <t>МАТЕРИАЛЫ ЗА ГОД, ИТОГО</t>
         </is>
       </c>
-      <c r="B18" s="22" t="n"/>
-      <c r="C18" s="22" t="n"/>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="23" t="n"/>
       <c r="D18" s="12">
         <f>SUM(D13:D17)</f>
         <v>932960</v>
       </c>
-      <c r="E18" s="50">
+      <c r="E18" s="54">
         <f>SUM(E13:E17)</f>
         <v>16</v>
       </c>
@@ -4420,7 +4467,7 @@
         <f>SUM(F13:F17)</f>
         <v>82880</v>
       </c>
-      <c r="G18" s="50">
+      <c r="G18" s="54">
         <f>SUM(G13:G17)</f>
         <v>20.3</v>
       </c>
@@ -4484,19 +4531,19 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B22" s="37">
+      <c r="B22" s="52">
         <f>Данные!$B$20</f>
         <v>0</v>
       </c>
-      <c r="C22" s="37">
+      <c r="C22" s="52">
         <f>Данные!$C$20</f>
         <v>29</v>
       </c>
-      <c r="D22" s="37">
+      <c r="D22" s="52">
         <f>B22+C22</f>
         <v>29</v>
       </c>
-      <c r="E22" s="32">
+      <c r="E22" s="33">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4511,19 +4558,19 @@
           <t>Бройлерные площадки · 8 шт</t>
         </is>
       </c>
-      <c r="B23" s="37">
+      <c r="B23" s="52">
         <f>SUM(Данные!$B$23:$B$30)</f>
         <v>161</v>
       </c>
-      <c r="C23" s="37">
+      <c r="C23" s="52">
         <f>SUM(Данные!$C$23:$C$30)</f>
         <v>1096</v>
       </c>
-      <c r="D23" s="37">
+      <c r="D23" s="52">
         <f>B23+C23</f>
         <v>1257</v>
       </c>
-      <c r="E23" s="32">
+      <c r="E23" s="33">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4538,19 +4585,19 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B24" s="37">
+      <c r="B24" s="52">
         <f>Данные!$B$21</f>
         <v>18</v>
       </c>
-      <c r="C24" s="37">
+      <c r="C24" s="52">
         <f>Данные!$C$21</f>
         <v>34</v>
       </c>
-      <c r="D24" s="37">
+      <c r="D24" s="52">
         <f>B24+C24</f>
         <v>52</v>
       </c>
-      <c r="E24" s="32">
+      <c r="E24" s="33">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4565,19 +4612,19 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B25" s="37">
+      <c r="B25" s="52">
         <f>Данные!$B$22</f>
         <v>0</v>
       </c>
-      <c r="C25" s="37">
+      <c r="C25" s="52">
         <f>Данные!$C$22</f>
         <v>39</v>
       </c>
-      <c r="D25" s="37">
+      <c r="D25" s="52">
         <f>B25+C25</f>
         <v>39</v>
       </c>
-      <c r="E25" s="32">
+      <c r="E25" s="33">
         <f>Данные!$B$9</f>
         <v>2160</v>
       </c>
@@ -4592,19 +4639,19 @@
           <t>ИТОГО РАЗОВО</t>
         </is>
       </c>
-      <c r="B26" s="40">
+      <c r="B26" s="55">
         <f>SUM(B22:B25)</f>
         <v>179</v>
       </c>
-      <c r="C26" s="40">
+      <c r="C26" s="55">
         <f>SUM(C22:C25)</f>
         <v>1198</v>
       </c>
-      <c r="D26" s="40">
+      <c r="D26" s="55">
         <f>SUM(D22:D25)</f>
         <v>1377</v>
       </c>
-      <c r="E26" s="22" t="n"/>
+      <c r="E26" s="23" t="n"/>
       <c r="F26" s="12">
         <f>SUM(F22:F25)</f>
         <v>2974320</v>
@@ -4624,32 +4671,32 @@
       <c r="F28" s="16" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="35" t="inlineStr">
+      <c r="A29" s="36" t="inlineStr">
         <is>
           <t>Численность, чел.</t>
         </is>
       </c>
-      <c r="B29" s="36" t="inlineStr">
+      <c r="B29" s="37" t="inlineStr">
         <is>
           <t>ЗП в месяц, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="C29" s="36" t="inlineStr">
+      <c r="C29" s="37" t="inlineStr">
         <is>
           <t>ЗП за год, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="D29" s="36" t="inlineStr">
+      <c r="D29" s="37" t="inlineStr">
         <is>
           <t>Материалы за год, ₸</t>
         </is>
       </c>
-      <c r="E29" s="36" t="inlineStr">
+      <c r="E29" s="37" t="inlineStr">
         <is>
           <t>Итого за год, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="F29" s="36" t="inlineStr">
+      <c r="F29" s="37" t="inlineStr">
         <is>
           <t>Итого за год, ₸ · оклад 350 000</t>
         </is>
@@ -4882,7 +4929,7 @@
     </row>
     <row r="39"/>
     <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="24" t="inlineStr">
+      <c r="A40" s="25" t="inlineStr">
         <is>
           <t>Материалы от численности не зависят — норма ядов и станций привязана к точкам, а не к людям. Каждый дополнительный дератизатор добавляет только фонд оплаты труда.</t>
         </is>
@@ -4946,26 +4993,26 @@
       <c r="H4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Ед. изм.</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr"/>
-      <c r="E5" s="26" t="inlineStr"/>
-      <c r="F5" s="26" t="inlineStr"/>
-      <c r="G5" s="26" t="inlineStr"/>
-      <c r="H5" s="26" t="inlineStr">
+      <c r="D5" s="27" t="inlineStr"/>
+      <c r="E5" s="27" t="inlineStr"/>
+      <c r="F5" s="27" t="inlineStr"/>
+      <c r="G5" s="27" t="inlineStr"/>
+      <c r="H5" s="27" t="inlineStr">
         <is>
           <t>Источник / примечание</t>
         </is>
@@ -4977,7 +5024,7 @@
           <t>Зерноцид</t>
         </is>
       </c>
-      <c r="B6" s="41" t="n">
+      <c r="B6" s="42" t="n">
         <v>740</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -4985,7 +5032,7 @@
           <t>₸/кг</t>
         </is>
       </c>
-      <c r="H6" s="42" t="inlineStr">
+      <c r="H6" s="43" t="inlineStr">
         <is>
           <t>внутренние данные УКПФ</t>
         </is>
@@ -4997,7 +5044,7 @@
           <t>Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B7" s="41" t="n">
+      <c r="B7" s="42" t="n">
         <v>3642.5</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -5005,7 +5052,7 @@
           <t>₸/кг</t>
         </is>
       </c>
-      <c r="H7" s="42" t="inlineStr">
+      <c r="H7" s="43" t="inlineStr">
         <is>
           <t>перенесено из прежнего расчёта по ККЗ; в исходных нормах цены не было</t>
         </is>
@@ -5017,7 +5064,7 @@
           <t>Клеевая станция 3-го контура</t>
         </is>
       </c>
-      <c r="B8" s="41" t="n">
+      <c r="B8" s="42" t="n">
         <v>160</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -5025,7 +5072,7 @@
           <t>₸/шт</t>
         </is>
       </c>
-      <c r="H8" s="42" t="inlineStr">
+      <c r="H8" s="43" t="inlineStr">
         <is>
           <t>внутренние данные УКПФ, расходуется ежемесячно</t>
         </is>
@@ -5037,7 +5084,7 @@
           <t>Приманочная станция 1–2 контура</t>
         </is>
       </c>
-      <c r="B9" s="41" t="n">
+      <c r="B9" s="42" t="n">
         <v>2160</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -5045,7 +5092,7 @@
           <t>₸/шт</t>
         </is>
       </c>
-      <c r="H9" s="42" t="inlineStr">
+      <c r="H9" s="43" t="inlineStr">
         <is>
           <t>разовая закупка; цена из прежнего расчёта по ККЗ (29 шт = 62 640 ₸)</t>
         </is>
@@ -5057,7 +5104,7 @@
           <t>Бутылка</t>
         </is>
       </c>
-      <c r="B10" s="41" t="n">
+      <c r="B10" s="42" t="n">
         <v>68</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -5065,7 +5112,7 @@
           <t>₸/шт</t>
         </is>
       </c>
-      <c r="H10" s="42" t="inlineStr">
+      <c r="H10" s="43" t="inlineStr">
         <is>
           <t>внутренние данные УКПФ</t>
         </is>
@@ -5077,7 +5124,7 @@
           <t>Бутылки, расход</t>
         </is>
       </c>
-      <c r="B11" s="41" t="n">
+      <c r="B11" s="42" t="n">
         <v>40</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -5085,7 +5132,7 @@
           <t>шт/мес</t>
         </is>
       </c>
-      <c r="H11" s="42" t="inlineStr">
+      <c r="H11" s="43" t="inlineStr">
         <is>
           <t>тёплый сезон, зимой ноль; оценка, по объектам не разносится</t>
         </is>
@@ -5097,7 +5144,7 @@
           <t>Оклад дератизатора · вариант 1</t>
         </is>
       </c>
-      <c r="B12" s="41" t="n">
+      <c r="B12" s="42" t="n">
         <v>258488</v>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -5105,7 +5152,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H12" s="42" t="inlineStr">
+      <c r="H12" s="43" t="inlineStr">
         <is>
           <t>действующий оклад</t>
         </is>
@@ -5117,7 +5164,7 @@
           <t>Оклад дератизатора · вариант 2</t>
         </is>
       </c>
-      <c r="B13" s="41" t="n">
+      <c r="B13" s="42" t="n">
         <v>350000</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -5125,7 +5172,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H13" s="42" t="inlineStr">
+      <c r="H13" s="43" t="inlineStr">
         <is>
           <t>альтернативный уровень для сравнения</t>
         </is>
@@ -5137,7 +5184,7 @@
           <t>Численность штата</t>
         </is>
       </c>
-      <c r="B14" s="41" t="n">
+      <c r="B14" s="42" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -5145,7 +5192,7 @@
           <t>чел.</t>
         </is>
       </c>
-      <c r="H14" s="42" t="inlineStr">
+      <c r="H14" s="43" t="inlineStr">
         <is>
           <t>измените — пересчитаются все листы</t>
         </is>
@@ -5157,7 +5204,7 @@
           <t>Тёплых месяцев (апрель — октябрь)</t>
         </is>
       </c>
-      <c r="B15" s="41" t="n">
+      <c r="B15" s="42" t="n">
         <v>7</v>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -5165,7 +5212,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H15" s="42" t="inlineStr">
+      <c r="H15" s="43" t="inlineStr">
         <is>
           <t>заряжаются все три контура</t>
         </is>
@@ -5177,7 +5224,7 @@
           <t>Зимних месяцев (ноябрь — март)</t>
         </is>
       </c>
-      <c r="B16" s="41" t="n">
+      <c r="B16" s="42" t="n">
         <v>5</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -5185,7 +5232,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H16" s="42" t="inlineStr">
+      <c r="H16" s="43" t="inlineStr">
         <is>
           <t>1-й и 2-й контуры не заряжаются, 3-й обслуживается вдвое</t>
         </is>
@@ -5207,42 +5254,42 @@
       <c r="H18" s="16" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="35" t="inlineStr">
+      <c r="A19" s="36" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B19" s="36" t="inlineStr">
+      <c r="B19" s="37" t="inlineStr">
         <is>
           <t>1-й контур, шт</t>
         </is>
       </c>
-      <c r="C19" s="36" t="inlineStr">
+      <c r="C19" s="37" t="inlineStr">
         <is>
           <t>2-й контур, шт</t>
         </is>
       </c>
-      <c r="D19" s="36" t="inlineStr">
+      <c r="D19" s="37" t="inlineStr">
         <is>
           <t>3-й контур, шт</t>
         </is>
       </c>
-      <c r="E19" s="36" t="inlineStr">
+      <c r="E19" s="37" t="inlineStr">
         <is>
           <t>Всего точек, шт</t>
         </is>
       </c>
-      <c r="F19" s="36" t="inlineStr">
+      <c r="F19" s="37" t="inlineStr">
         <is>
           <t>Pest Killer, кг</t>
         </is>
       </c>
-      <c r="G19" s="36" t="inlineStr">
+      <c r="G19" s="37" t="inlineStr">
         <is>
           <t>Зерноцид, кг</t>
         </is>
       </c>
-      <c r="H19" s="36" t="inlineStr">
+      <c r="H19" s="37" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
@@ -5254,26 +5301,26 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B20" s="41" t="n">
+      <c r="B20" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="41" t="n">
+      <c r="C20" s="42" t="n">
         <v>29</v>
       </c>
-      <c r="D20" s="41" t="n">
+      <c r="D20" s="42" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="7">
         <f>SUM(B20:D20)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="51" t="n">
+      <c r="F20" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="51" t="n">
+      <c r="G20" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="42" t="inlineStr">
+      <c r="H20" s="43" t="inlineStr">
         <is>
           <t>29 приманочных станций 2-го контура</t>
         </is>
@@ -5285,26 +5332,26 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B21" s="41" t="n">
+      <c r="B21" s="42" t="n">
         <v>18</v>
       </c>
-      <c r="C21" s="41" t="n">
+      <c r="C21" s="42" t="n">
         <v>34</v>
       </c>
-      <c r="D21" s="41" t="n">
+      <c r="D21" s="42" t="n">
         <v>12</v>
       </c>
       <c r="E21" s="7">
         <f>SUM(B21:D21)</f>
         <v>18</v>
       </c>
-      <c r="F21" s="51" t="n">
+      <c r="F21" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="51" t="n">
+      <c r="G21" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="42" t="inlineStr"/>
+      <c r="H21" s="43" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -5312,26 +5359,26 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B22" s="41" t="n">
+      <c r="B22" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="41" t="n">
+      <c r="C22" s="42" t="n">
         <v>39</v>
       </c>
-      <c r="D22" s="41" t="n">
+      <c r="D22" s="42" t="n">
         <v>63</v>
       </c>
       <c r="E22" s="7">
         <f>SUM(B22:D22)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="51" t="n">
+      <c r="F22" s="56" t="n">
         <v>1.3</v>
       </c>
-      <c r="G22" s="51" t="n">
+      <c r="G22" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="42" t="inlineStr">
+      <c r="H22" s="43" t="inlineStr">
         <is>
           <t>1,3 кг — приблизительная оценка, требует подтверждения</t>
         </is>
@@ -5343,26 +5390,26 @@
           <t>Площадка А</t>
         </is>
       </c>
-      <c r="B23" s="41" t="n">
+      <c r="B23" s="42" t="n">
         <v>13</v>
       </c>
-      <c r="C23" s="41" t="n">
+      <c r="C23" s="42" t="n">
         <v>147</v>
       </c>
-      <c r="D23" s="41" t="n">
+      <c r="D23" s="42" t="n">
         <v>20</v>
       </c>
       <c r="E23" s="7">
         <f>SUM(B23:D23)</f>
         <v>13</v>
       </c>
-      <c r="F23" s="51" t="n">
+      <c r="F23" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="51" t="n">
+      <c r="G23" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="42" t="inlineStr"/>
+      <c r="H23" s="43" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -5370,26 +5417,26 @@
           <t>Площадка Б</t>
         </is>
       </c>
-      <c r="B24" s="41" t="n">
+      <c r="B24" s="42" t="n">
         <v>17</v>
       </c>
-      <c r="C24" s="41" t="n">
+      <c r="C24" s="42" t="n">
         <v>146</v>
       </c>
-      <c r="D24" s="41" t="n">
+      <c r="D24" s="42" t="n">
         <v>20</v>
       </c>
       <c r="E24" s="7">
         <f>SUM(B24:D24)</f>
         <v>17</v>
       </c>
-      <c r="F24" s="51" t="n">
+      <c r="F24" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="51" t="n">
+      <c r="G24" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="H24" s="42" t="inlineStr"/>
+      <c r="H24" s="43" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -5397,26 +5444,26 @@
           <t>В / Восточка</t>
         </is>
       </c>
-      <c r="B25" s="41" t="n">
+      <c r="B25" s="42" t="n">
         <v>50</v>
       </c>
-      <c r="C25" s="41" t="n">
+      <c r="C25" s="42" t="n">
         <v>239</v>
       </c>
-      <c r="D25" s="41" t="n">
+      <c r="D25" s="42" t="n">
         <v>30</v>
       </c>
       <c r="E25" s="7">
         <f>SUM(B25:D25)</f>
         <v>50</v>
       </c>
-      <c r="F25" s="51" t="n">
+      <c r="F25" s="56" t="n">
         <v>3.5</v>
       </c>
-      <c r="G25" s="51" t="n">
+      <c r="G25" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="42" t="inlineStr"/>
+      <c r="H25" s="43" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -5424,26 +5471,26 @@
           <t>Площадка Г</t>
         </is>
       </c>
-      <c r="B26" s="41" t="n">
+      <c r="B26" s="42" t="n">
         <v>17</v>
       </c>
-      <c r="C26" s="41" t="n">
+      <c r="C26" s="42" t="n">
         <v>88</v>
       </c>
-      <c r="D26" s="41" t="n">
+      <c r="D26" s="42" t="n">
         <v>80</v>
       </c>
       <c r="E26" s="7">
         <f>SUM(B26:D26)</f>
         <v>17</v>
       </c>
-      <c r="F26" s="51" t="n">
+      <c r="F26" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="51" t="n">
+      <c r="G26" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="H26" s="42" t="inlineStr"/>
+      <c r="H26" s="43" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -5451,26 +5498,26 @@
           <t>Площадка Д</t>
         </is>
       </c>
-      <c r="B27" s="41" t="n">
+      <c r="B27" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="C27" s="41" t="n">
+      <c r="C27" s="42" t="n">
         <v>69</v>
       </c>
-      <c r="D27" s="41" t="n">
+      <c r="D27" s="42" t="n">
         <v>64</v>
       </c>
       <c r="E27" s="7">
         <f>SUM(B27:D27)</f>
         <v>15</v>
       </c>
-      <c r="F27" s="51" t="n">
+      <c r="F27" s="56" t="n">
         <v>1.5</v>
       </c>
-      <c r="G27" s="51" t="n">
+      <c r="G27" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="42" t="inlineStr"/>
+      <c r="H27" s="43" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -5478,26 +5525,26 @@
           <t>Площадка Е</t>
         </is>
       </c>
-      <c r="B28" s="41" t="n">
+      <c r="B28" s="42" t="n">
         <v>13</v>
       </c>
-      <c r="C28" s="41" t="n">
+      <c r="C28" s="42" t="n">
         <v>147</v>
       </c>
-      <c r="D28" s="41" t="n">
+      <c r="D28" s="42" t="n">
         <v>20</v>
       </c>
       <c r="E28" s="7">
         <f>SUM(B28:D28)</f>
         <v>13</v>
       </c>
-      <c r="F28" s="51" t="n">
+      <c r="F28" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="51" t="n">
+      <c r="G28" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="H28" s="42" t="inlineStr"/>
+      <c r="H28" s="43" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -5505,26 +5552,26 @@
           <t>Площадка Ж</t>
         </is>
       </c>
-      <c r="B29" s="41" t="n">
+      <c r="B29" s="42" t="n">
         <v>17</v>
       </c>
-      <c r="C29" s="41" t="n">
+      <c r="C29" s="42" t="n">
         <v>73</v>
       </c>
-      <c r="D29" s="41" t="n">
+      <c r="D29" s="42" t="n">
         <v>10</v>
       </c>
       <c r="E29" s="7">
         <f>SUM(B29:D29)</f>
         <v>17</v>
       </c>
-      <c r="F29" s="51" t="n">
+      <c r="F29" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="51" t="n">
+      <c r="G29" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="H29" s="42" t="inlineStr"/>
+      <c r="H29" s="43" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -5532,26 +5579,26 @@
           <t>Айыртау (БП)</t>
         </is>
       </c>
-      <c r="B30" s="41" t="n">
+      <c r="B30" s="42" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="41" t="n">
+      <c r="C30" s="42" t="n">
         <v>187</v>
       </c>
-      <c r="D30" s="41" t="n">
+      <c r="D30" s="42" t="n">
         <v>24</v>
       </c>
       <c r="E30" s="7">
         <f>SUM(B30:D30)</f>
         <v>19</v>
       </c>
-      <c r="F30" s="51" t="n">
+      <c r="F30" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="G30" s="51" t="n">
+      <c r="G30" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="H30" s="42" t="inlineStr"/>
+      <c r="H30" s="43" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -5563,9 +5610,9 @@
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
-      <c r="F31" s="49" t="n"/>
-      <c r="G31" s="49" t="n"/>
-      <c r="H31" s="42" t="inlineStr">
+      <c r="F31" s="53" t="n"/>
+      <c r="G31" s="53" t="n"/>
+      <c r="H31" s="43" t="inlineStr">
         <is>
           <t>нормы расхода не заданы</t>
         </is>
@@ -5581,9 +5628,9 @@
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
-      <c r="F32" s="49" t="n"/>
-      <c r="G32" s="49" t="n"/>
-      <c r="H32" s="42" t="inlineStr">
+      <c r="F32" s="53" t="n"/>
+      <c r="G32" s="53" t="n"/>
+      <c r="H32" s="43" t="inlineStr">
         <is>
           <t>нормы расхода не заданы</t>
         </is>
@@ -5611,15 +5658,15 @@
         <f>SUM(E20:E32)</f>
         <v>179</v>
       </c>
-      <c r="F33" s="50">
+      <c r="F33" s="54">
         <f>SUM(F20:F32)</f>
         <v>20.3</v>
       </c>
-      <c r="G33" s="50">
+      <c r="G33" s="54">
         <f>SUM(G20:G32)</f>
         <v>16</v>
       </c>
-      <c r="H33" s="22" t="n"/>
+      <c r="H33" s="23" t="n"/>
     </row>
     <row r="34"/>
     <row r="35">
@@ -5637,26 +5684,26 @@
       <c r="H35" s="16" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="26" t="inlineStr">
+      <c r="A36" s="27" t="inlineStr">
         <is>
           <t>Позиция</t>
         </is>
       </c>
-      <c r="B36" s="26" t="inlineStr">
+      <c r="B36" s="27" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="C36" s="26" t="inlineStr">
+      <c r="C36" s="27" t="inlineStr">
         <is>
           <t>Ед. изм.</t>
         </is>
       </c>
-      <c r="D36" s="26" t="inlineStr"/>
-      <c r="E36" s="26" t="inlineStr"/>
-      <c r="F36" s="26" t="inlineStr"/>
-      <c r="G36" s="26" t="inlineStr"/>
-      <c r="H36" s="26" t="inlineStr">
+      <c r="D36" s="27" t="inlineStr"/>
+      <c r="E36" s="27" t="inlineStr"/>
+      <c r="F36" s="27" t="inlineStr"/>
+      <c r="G36" s="27" t="inlineStr"/>
+      <c r="H36" s="27" t="inlineStr">
         <is>
           <t>Источник</t>
         </is>
@@ -5668,7 +5715,7 @@
           <t>Indigo · ККЗ, дератизация</t>
         </is>
       </c>
-      <c r="B37" s="41" t="n">
+      <c r="B37" s="42" t="n">
         <v>96600</v>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -5676,7 +5723,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H37" s="42" t="inlineStr">
+      <c r="H37" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); барьер вокруг периметра кормоцеха и грязный барьер</t>
         </is>
@@ -5688,7 +5735,7 @@
           <t>Indigo · Айыртау БП, полная замена</t>
         </is>
       </c>
-      <c r="B38" s="41" t="n">
+      <c r="B38" s="42" t="n">
         <v>618400</v>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -5696,7 +5743,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H38" s="42" t="inlineStr">
+      <c r="H38" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 180 ед. оборудования</t>
         </is>
@@ -5708,7 +5755,7 @@
           <t>Indigo · Айыртау БП, частичная замена</t>
         </is>
       </c>
-      <c r="B39" s="41" t="n">
+      <c r="B39" s="42" t="n">
         <v>478400</v>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -5716,7 +5763,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H39" s="42" t="inlineStr">
+      <c r="H39" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5728,7 +5775,7 @@
           <t>Indigo · Многоэтажки Д и Г, полная замена</t>
         </is>
       </c>
-      <c r="B40" s="41" t="n">
+      <c r="B40" s="42" t="n">
         <v>569800</v>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -5736,7 +5783,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H40" s="42" t="inlineStr">
+      <c r="H40" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 166 ед. оборудования</t>
         </is>
@@ -5748,7 +5795,7 @@
           <t>Indigo · Многоэтажки Д и Г, частичная замена</t>
         </is>
       </c>
-      <c r="B41" s="41" t="n">
+      <c r="B41" s="42" t="n">
         <v>440700</v>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -5756,7 +5803,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H41" s="42" t="inlineStr">
+      <c r="H41" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5768,7 +5815,7 @@
           <t>Indigo · Площадки А,Б,Е,Ж,В,В(РМ), полная</t>
         </is>
       </c>
-      <c r="B42" s="41" t="n">
+      <c r="B42" s="42" t="n">
         <v>2599100</v>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -5776,7 +5823,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H42" s="42" t="inlineStr">
+      <c r="H42" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 793 ед. оборудования</t>
         </is>
@@ -5788,7 +5835,7 @@
           <t>Indigo · Площадки А,Б,Е,Ж,В,В(РМ), частичная</t>
         </is>
       </c>
-      <c r="B43" s="41" t="n">
+      <c r="B43" s="42" t="n">
         <v>2010300</v>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -5796,7 +5843,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H43" s="42" t="inlineStr">
+      <c r="H43" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5808,7 +5855,7 @@
           <t>Indigo · Инкубаторий, полная замена</t>
         </is>
       </c>
-      <c r="B44" s="41" t="n">
+      <c r="B44" s="42" t="n">
         <v>126200</v>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -5816,7 +5863,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H44" s="42" t="inlineStr">
+      <c r="H44" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 48 ед. оборудования</t>
         </is>
@@ -5828,7 +5875,7 @@
           <t>Indigo · Инкубаторий, частичная замена</t>
         </is>
       </c>
-      <c r="B45" s="41" t="n">
+      <c r="B45" s="42" t="n">
         <v>106800</v>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -5836,7 +5883,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H45" s="42" t="inlineStr">
+      <c r="H45" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5848,7 +5895,7 @@
           <t>Indigo · ЗПП, полная замена</t>
         </is>
       </c>
-      <c r="B46" s="41" t="n">
+      <c r="B46" s="42" t="n">
         <v>126200</v>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -5856,7 +5903,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H46" s="42" t="inlineStr">
+      <c r="H46" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5868,7 +5915,7 @@
           <t>Indigo · ЗПП, частичная замена</t>
         </is>
       </c>
-      <c r="B47" s="41" t="n">
+      <c r="B47" s="42" t="n">
         <v>106800</v>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -5876,7 +5923,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H47" s="42" t="inlineStr">
+      <c r="H47" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5888,7 +5935,7 @@
           <t>Indigo · дезинсекция, Айыртау БП</t>
         </is>
       </c>
-      <c r="B48" s="41" t="n">
+      <c r="B48" s="42" t="n">
         <v>720000</v>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -5896,7 +5943,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H48" s="42" t="inlineStr">
+      <c r="H48" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5908,7 +5955,7 @@
           <t>Indigo · дезинсекция, Многоэтажки</t>
         </is>
       </c>
-      <c r="B49" s="41" t="n">
+      <c r="B49" s="42" t="n">
         <v>1080000</v>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -5916,7 +5963,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H49" s="42" t="inlineStr">
+      <c r="H49" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5928,7 +5975,7 @@
           <t>Indigo · дезинсекция, Площадки</t>
         </is>
       </c>
-      <c r="B50" s="41" t="n">
+      <c r="B50" s="42" t="n">
         <v>3000000</v>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -5936,7 +5983,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H50" s="42" t="inlineStr">
+      <c r="H50" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5948,7 +5995,7 @@
           <t>Indigo · дезинсекция, Инкубаторий</t>
         </is>
       </c>
-      <c r="B51" s="41" t="n">
+      <c r="B51" s="42" t="n">
         <v>100800</v>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -5956,7 +6003,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H51" s="42" t="inlineStr">
+      <c r="H51" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5968,7 +6015,7 @@
           <t>Indigo · дезинсекция, ЗПП</t>
         </is>
       </c>
-      <c r="B52" s="41" t="n">
+      <c r="B52" s="42" t="n">
         <v>160800</v>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -5976,7 +6023,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H52" s="42" t="inlineStr">
+      <c r="H52" s="43" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5988,7 +6035,7 @@
           <t>Pest Hunters · ККЗ, дератизация</t>
         </is>
       </c>
-      <c r="B53" s="41" t="n">
+      <c r="B53" s="42" t="n">
         <v>75000</v>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -5996,7 +6043,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H53" s="42" t="inlineStr">
+      <c r="H53" s="43" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -6008,7 +6055,7 @@
           <t>Pest Hunters · ККЗ, дезинсекция</t>
         </is>
       </c>
-      <c r="B54" s="41" t="n">
+      <c r="B54" s="42" t="n">
         <v>70000</v>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -6016,7 +6063,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H54" s="42" t="inlineStr">
+      <c r="H54" s="43" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -6028,7 +6075,7 @@
           <t>Pest Hunters · площадки, март — ноябрь</t>
         </is>
       </c>
-      <c r="B55" s="41" t="n">
+      <c r="B55" s="42" t="n">
         <v>3172000</v>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -6036,7 +6083,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H55" s="42" t="inlineStr">
+      <c r="H55" s="43" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); 122 объекта, оборудование подрядчика</t>
         </is>
@@ -6048,7 +6095,7 @@
           <t>Pest Hunters · площадки, декабрь — февраль</t>
         </is>
       </c>
-      <c r="B56" s="41" t="n">
+      <c r="B56" s="42" t="n">
         <v>2074000</v>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -6056,7 +6103,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H56" s="42" t="inlineStr">
+      <c r="H56" s="43" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); 122 объекта, оборудование подрядчика</t>
         </is>
@@ -6068,7 +6115,7 @@
           <t>Pest Hunters · площадки альт., март — ноябрь</t>
         </is>
       </c>
-      <c r="B57" s="41" t="n">
+      <c r="B57" s="42" t="n">
         <v>2806000</v>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -6076,7 +6123,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H57" s="42" t="inlineStr">
+      <c r="H57" s="43" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); оборудование заказчика</t>
         </is>
@@ -6088,7 +6135,7 @@
           <t>Pest Hunters · площадки альт., дек. — февраль</t>
         </is>
       </c>
-      <c r="B58" s="41" t="n">
+      <c r="B58" s="42" t="n">
         <v>1830000</v>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -6096,7 +6143,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H58" s="42" t="inlineStr">
+      <c r="H58" s="43" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); оборудование заказчика</t>
         </is>
@@ -6108,7 +6155,7 @@
           <t>Pest Hunters · ЗПП</t>
         </is>
       </c>
-      <c r="B59" s="41" t="n">
+      <c r="B59" s="42" t="n">
         <v>180000</v>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -6116,7 +6163,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H59" s="42" t="inlineStr">
+      <c r="H59" s="43" t="inlineStr">
         <is>
           <t>договор №88 от 01.01.2026; дератизация + дезинсекция, 8 309 м², 3 обхода в месяц</t>
         </is>
@@ -6128,7 +6175,7 @@
           <t>Pest Hunters · склад ТМЦ</t>
         </is>
       </c>
-      <c r="B60" s="41" t="n">
+      <c r="B60" s="42" t="n">
         <v>80000</v>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -6136,7 +6183,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H60" s="42" t="inlineStr">
+      <c r="H60" s="43" t="inlineStr">
         <is>
           <t>договор №921 от 01.04.2026; дератизация + дезинсекция, 1 обход в месяц</t>
         </is>
@@ -6148,7 +6195,7 @@
           <t>Месяцев высокого тарифа площадок (мар — ноя)</t>
         </is>
       </c>
-      <c r="B61" s="41" t="n">
+      <c r="B61" s="42" t="n">
         <v>9</v>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -6156,7 +6203,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H61" s="42" t="inlineStr">
+      <c r="H61" s="43" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -6168,7 +6215,7 @@
           <t>Месяцев низкого тарифа площадок (дек — фев)</t>
         </is>
       </c>
-      <c r="B62" s="41" t="n">
+      <c r="B62" s="42" t="n">
         <v>3</v>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -6176,7 +6223,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H62" s="42" t="inlineStr">
+      <c r="H62" s="43" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -6188,7 +6235,7 @@
           <t>Месяцев действия договора по складу ТМЦ</t>
         </is>
       </c>
-      <c r="B63" s="41" t="n">
+      <c r="B63" s="42" t="n">
         <v>9</v>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -6196,7 +6243,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H63" s="42" t="inlineStr">
+      <c r="H63" s="43" t="inlineStr">
         <is>
           <t>апрель — декабрь 2026</t>
         </is>
@@ -6208,7 +6255,7 @@
           <t>Скидка Indigo за всю территорию фабрики</t>
         </is>
       </c>
-      <c r="B64" s="44" t="n">
+      <c r="B64" s="57" t="n">
         <v>0.15</v>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -6216,7 +6263,7 @@
           <t>доля</t>
         </is>
       </c>
-      <c r="H64" s="42" t="inlineStr">
+      <c r="H64" s="43" t="inlineStr">
         <is>
           <t>КП от 19.08.2026, условия предоставления скидок</t>
         </is>
@@ -6228,7 +6275,7 @@
           <t>Скидка Indigo за 100 % предоплату за год</t>
         </is>
       </c>
-      <c r="B65" s="44" t="n">
+      <c r="B65" s="57" t="n">
         <v>0.15</v>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -6236,7 +6283,7 @@
           <t>доля</t>
         </is>
       </c>
-      <c r="H65" s="42" t="inlineStr">
+      <c r="H65" s="43" t="inlineStr">
         <is>
           <t>КП от 19.08.2026, дополнительно к предыдущей</t>
         </is>
@@ -6248,7 +6295,7 @@
           <t>Скидка Indigo неплательщику НДС</t>
         </is>
       </c>
-      <c r="B66" s="44" t="n">
+      <c r="B66" s="57" t="n">
         <v>0.16</v>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -6256,7 +6303,7 @@
           <t>доля</t>
         </is>
       </c>
-      <c r="H66" s="42" t="inlineStr">
+      <c r="H66" s="43" t="inlineStr">
         <is>
           <t>КП от 19.08.2026; цены КП уже включают НДС</t>
         </is>

</xml_diff>

<commit_message>
Remove the bogus per-block "Итого" row on object sheets
Each block on an object sheet lists Indigo, Pest Hunters and the in-house
crew as three alternatives, not three parts of a bill - summing all three
rows into one total (SUM(D_start:D_last)) mixed unrelated providers into
a meaningless number, e.g. 2 084 698 on ККЗ. The correct per-provider
totals at the top of each sheet were already right and are untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLozcDkCvYTXvP2yAkyMFB
</commit_message>
<xml_diff>
--- a/reports/УКПФ_дератизация_сравнение_КП.xlsx
+++ b/reports/УКПФ_дератизация_сравнение_КП.xlsx
@@ -214,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -279,9 +279,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -730,7 +727,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="46" t="n"/>
+      <c r="A5" s="45" t="n"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
           <t>в месяц</t>
@@ -843,7 +840,7 @@
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="E8" s="47" t="n"/>
+      <c r="E8" s="46" t="n"/>
       <c r="F8" s="7">
         <f>G8/12</f>
         <v>5276.458333</v>
@@ -880,7 +877,7 @@
           <t>нормы не заданы</t>
         </is>
       </c>
-      <c r="G9" s="47" t="n"/>
+      <c r="G9" s="46" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -893,7 +890,7 @@
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="C10" s="47" t="n"/>
+      <c r="C10" s="46" t="n"/>
       <c r="D10" s="7">
         <f>E10/12</f>
         <v>60000</v>
@@ -907,7 +904,7 @@
           <t>нормы не заданы</t>
         </is>
       </c>
-      <c r="G10" s="47" t="n"/>
+      <c r="G10" s="46" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -920,13 +917,13 @@
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="C11" s="47" t="n"/>
+      <c r="C11" s="46" t="n"/>
       <c r="D11" s="9" t="inlineStr">
         <is>
           <t>нет в КП</t>
         </is>
       </c>
-      <c r="E11" s="47" t="n"/>
+      <c r="E11" s="46" t="n"/>
       <c r="F11" s="7">
         <f>G11/12</f>
         <v>17042.22917</v>
@@ -1086,7 +1083,7 @@
         <f>C15-G15</f>
         <v>35675696.75</v>
       </c>
-      <c r="D19" s="48">
+      <c r="D19" s="47">
         <f>IF(G15=0,0,C15/G15)</f>
         <v>3.555583381</v>
       </c>
@@ -1105,7 +1102,7 @@
         <f>E15-G15</f>
         <v>24590096.75</v>
       </c>
-      <c r="D20" s="48">
+      <c r="D20" s="47">
         <f>IF(G15=0,0,E15/G15)</f>
         <v>2.761480457</v>
       </c>
@@ -1359,7 +1356,7 @@
           <t xml:space="preserve">   расход брикетов на одну станцию 2-го контура</t>
         </is>
       </c>
-      <c r="B32" s="49">
+      <c r="B32" s="48">
         <f>Данные!$F$33/Данные!$C$33</f>
         <v>0.01694490818</v>
       </c>
@@ -1578,7 +1575,7 @@
         <f>C15*(1-Данные!$B$64)</f>
         <v>42190260</v>
       </c>
-      <c r="D44" s="50">
+      <c r="D44" s="49">
         <f>Данные!$B$64</f>
         <v>0.15</v>
       </c>
@@ -1597,7 +1594,7 @@
         <f>C15*(1-Данные!$B$64)*(1-Данные!$B$65)</f>
         <v>35861721</v>
       </c>
-      <c r="D45" s="50">
+      <c r="D45" s="49">
         <f>Данные!$B$65</f>
         <v>0.15</v>
       </c>
@@ -1616,7 +1613,7 @@
         <f>C15*(1-Данные!$B$64)*(1-Данные!$B$65)*(1-Данные!$B$66)</f>
         <v>30123845.64</v>
       </c>
-      <c r="D46" s="50">
+      <c r="D46" s="49">
         <f>Данные!$B$66</f>
         <v>0.16</v>
       </c>
@@ -1678,9 +1675,9 @@
           <t>ответ по заявке ≤ 2 ч, выезд ≤ 24 ч, вызовы без ограничений</t>
         </is>
       </c>
-      <c r="E50" s="51" t="n"/>
-      <c r="F50" s="51" t="n"/>
-      <c r="G50" s="47" t="n"/>
+      <c r="E50" s="50" t="n"/>
+      <c r="F50" s="50" t="n"/>
+      <c r="G50" s="46" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -1701,9 +1698,9 @@
           <t>выезд по запросу</t>
         </is>
       </c>
-      <c r="E51" s="51" t="n"/>
-      <c r="F51" s="51" t="n"/>
-      <c r="G51" s="47" t="n"/>
+      <c r="E51" s="50" t="n"/>
+      <c r="F51" s="50" t="n"/>
+      <c r="G51" s="46" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -1724,9 +1721,9 @@
           <t>дополнительные визиты по вызову</t>
         </is>
       </c>
-      <c r="E52" s="51" t="n"/>
-      <c r="F52" s="51" t="n"/>
-      <c r="G52" s="47" t="n"/>
+      <c r="E52" s="50" t="n"/>
+      <c r="F52" s="50" t="n"/>
+      <c r="G52" s="46" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -1747,9 +1744,9 @@
           <t>по графику на 2026 год, бригада из трёх человек</t>
         </is>
       </c>
-      <c r="E53" s="51" t="n"/>
-      <c r="F53" s="51" t="n"/>
-      <c r="G53" s="47" t="n"/>
+      <c r="E53" s="50" t="n"/>
+      <c r="F53" s="50" t="n"/>
+      <c r="G53" s="46" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
@@ -1770,9 +1767,9 @@
           <t>выезд по рекламации за два рабочих дня</t>
         </is>
       </c>
-      <c r="E54" s="51" t="n"/>
-      <c r="F54" s="51" t="n"/>
-      <c r="G54" s="47" t="n"/>
+      <c r="E54" s="50" t="n"/>
+      <c r="F54" s="50" t="n"/>
+      <c r="G54" s="46" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -1793,9 +1790,9 @@
           <t>присутствие 5/2, реакция в тот же день</t>
         </is>
       </c>
-      <c r="E55" s="51" t="n"/>
-      <c r="F55" s="51" t="n"/>
-      <c r="G55" s="47" t="n"/>
+      <c r="E55" s="50" t="n"/>
+      <c r="F55" s="50" t="n"/>
+      <c r="G55" s="46" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -1828,7 +1825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2033,169 +2030,136 @@
         <v>25497.5</v>
       </c>
     </row>
-    <row r="15">
-      <c r="C15" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D15" s="12">
-        <f>SUM(D9:D14)</f>
-        <v>2084697.5</v>
-      </c>
-    </row>
-    <row r="16"/>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>РАЗОВЫЕ ЗАТРАТЫ ШТАТА (СПРАВОЧНО)</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+    </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>РАЗОВЫЕ ЗАТРАТЫ ШТАТА (СПРАВОЧНО)</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="n"/>
-      <c r="C17" s="16" t="n"/>
-      <c r="D17" s="16" t="n"/>
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Цена в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Месяцев</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>За год, ₸</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Цена в месяц, ₸</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Месяцев</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>За год, ₸</t>
-        </is>
+      <c r="A18" s="32" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B18" s="33">
+        <f>Данные!$B$20*Данные!$B$9</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="7">
+        <f>B18*C18</f>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="32" t="inlineStr">
         <is>
-          <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
+          <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
       <c r="B19" s="33">
-        <f>Данные!$B$20*Данные!$B$9</f>
-        <v>0</v>
+        <f>Данные!$C$20*Данные!$B$9</f>
+        <v>62640</v>
       </c>
       <c r="C19" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="7">
         <f>B19*C19</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="32" t="inlineStr">
-        <is>
-          <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="B20" s="33">
-        <f>Данные!$C$20*Данные!$B$9</f>
         <v>62640</v>
       </c>
-      <c r="C20" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="7">
-        <f>B20*C20</f>
-        <v>62640</v>
-      </c>
-    </row>
+    </row>
+    <row r="20"/>
     <row r="21">
-      <c r="C21" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D21" s="12">
-        <f>SUM(D19:D20)</f>
-        <v>62640</v>
-      </c>
-    </row>
-    <row r="22"/>
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="16" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Цена в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Месяцев</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>За год, ₸</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
-        </is>
-      </c>
-      <c r="B23" s="16" t="n"/>
-      <c r="C23" s="16" t="n"/>
-      <c r="D23" s="16" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Цена в месяц, ₸</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Месяцев</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>За год, ₸</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="32" t="inlineStr">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>Pest Hunters · дезинсекция</t>
         </is>
       </c>
-      <c r="B25" s="33">
+      <c r="B23" s="33">
         <f>Данные!$B$54</f>
         <v>70000</v>
       </c>
-      <c r="C25" s="33" t="n">
+      <c r="C23" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="D25" s="7">
-        <f>B25*C25</f>
+      <c r="D23" s="7">
+        <f>B23*C23</f>
         <v>840000</v>
       </c>
     </row>
-    <row r="26">
-      <c r="C26" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D26" s="12">
-        <f>SUM(D25:D25)</f>
-        <v>840000</v>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="25" t="inlineStr">
+    <row r="24"/>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>Зерноцид по ККЗ в нормах не заявлен, поэтому строка Зерноцида даёт ноль.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="25" t="inlineStr">
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="25" t="inlineStr">
         <is>
           <t>Зарплата дератизаторов по объектам не делится — она на листе «Штат УКПФ».</t>
         </is>
@@ -2203,8 +2167,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A26:D26"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2217,7 +2181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2478,341 +2442,297 @@
         <v>433457.5</v>
       </c>
     </row>
-    <row r="18">
-      <c r="C18" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D18" s="12">
-        <f>SUM(D9:D17)</f>
-        <v>81457717.5</v>
-      </c>
-    </row>
-    <row r="19"/>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>АЛЬТЕРНАТИВНЫЕ ВАРИАНТЫ ИЗ ТЕХ ЖЕ КП</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="16" t="n"/>
+    </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>АЛЬТЕРНАТИВНЫЕ ВАРИАНТЫ ИЗ ТЕХ ЖЕ КП</t>
-        </is>
-      </c>
-      <c r="B20" s="16" t="n"/>
-      <c r="C20" s="16" t="n"/>
-      <c r="D20" s="16" t="n"/>
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Цена в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Месяцев</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>За год, ₸</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Цена в месяц, ₸</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Месяцев</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>За год, ₸</t>
-        </is>
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t>Indigo Solutions · Айыртау БП — частичная замена</t>
+        </is>
+      </c>
+      <c r="B21" s="33">
+        <f>Данные!$B$39</f>
+        <v>478400</v>
+      </c>
+      <c r="C21" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" s="7">
+        <f>B21*C21</f>
+        <v>5740800</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="32" t="inlineStr">
         <is>
-          <t>Indigo Solutions · Айыртау БП — частичная замена</t>
+          <t>Indigo Solutions · Многоэтажки Д и Г — частичная замена</t>
         </is>
       </c>
       <c r="B22" s="33">
-        <f>Данные!$B$39</f>
-        <v>478400</v>
+        <f>Данные!$B$41</f>
+        <v>440700</v>
       </c>
       <c r="C22" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D22" s="7">
         <f>B22*C22</f>
-        <v>5740800</v>
+        <v>5288400</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="32" t="inlineStr">
         <is>
-          <t>Indigo Solutions · Многоэтажки Д и Г — частичная замена</t>
+          <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (РМ), В — частичная замена</t>
         </is>
       </c>
       <c r="B23" s="33">
-        <f>Данные!$B$41</f>
-        <v>440700</v>
+        <f>Данные!$B$43</f>
+        <v>2010300</v>
       </c>
       <c r="C23" s="33" t="n">
         <v>12</v>
       </c>
       <c r="D23" s="7">
         <f>B23*C23</f>
-        <v>5288400</v>
+        <v>24123600</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="32" t="inlineStr">
         <is>
-          <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (РМ), В — частичная замена</t>
+          <t>Pest Hunters · 122 объекта, март — ноябрь, оборудование заказчика</t>
         </is>
       </c>
       <c r="B24" s="33">
-        <f>Данные!$B$43</f>
-        <v>2010300</v>
-      </c>
-      <c r="C24" s="33" t="n">
-        <v>12</v>
+        <f>Данные!$B$57</f>
+        <v>2806000</v>
+      </c>
+      <c r="C24" s="33">
+        <f>Данные!$B$61</f>
+        <v>9</v>
       </c>
       <c r="D24" s="7">
         <f>B24*C24</f>
-        <v>24123600</v>
+        <v>25254000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="32" t="inlineStr">
         <is>
-          <t>Pest Hunters · 122 объекта, март — ноябрь, оборудование заказчика</t>
+          <t>Pest Hunters · 122 объекта, декабрь — февраль, оборудование заказчика</t>
         </is>
       </c>
       <c r="B25" s="33">
-        <f>Данные!$B$57</f>
-        <v>2806000</v>
+        <f>Данные!$B$58</f>
+        <v>1830000</v>
       </c>
       <c r="C25" s="33">
-        <f>Данные!$B$61</f>
-        <v>9</v>
+        <f>Данные!$B$62</f>
+        <v>3</v>
       </c>
       <c r="D25" s="7">
         <f>B25*C25</f>
-        <v>25254000</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="32" t="inlineStr">
-        <is>
-          <t>Pest Hunters · 122 объекта, декабрь — февраль, оборудование заказчика</t>
-        </is>
-      </c>
-      <c r="B26" s="33">
-        <f>Данные!$B$58</f>
-        <v>1830000</v>
-      </c>
-      <c r="C26" s="33">
-        <f>Данные!$B$62</f>
-        <v>3</v>
-      </c>
-      <c r="D26" s="7">
-        <f>B26*C26</f>
         <v>5490000</v>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
-      <c r="C27" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D27" s="12">
-        <f>SUM(D22:D26)</f>
-        <v>65896800</v>
-      </c>
-    </row>
-    <row r="28"/>
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>РАЗОВЫЕ ЗАТРАТЫ ШТАТА (СПРАВОЧНО)</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="16" t="n"/>
+      <c r="D27" s="16" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Цена в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Месяцев</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>За год, ₸</t>
+        </is>
+      </c>
+    </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>РАЗОВЫЕ ЗАТРАТЫ ШТАТА (СПРАВОЧНО)</t>
-        </is>
-      </c>
-      <c r="B29" s="16" t="n"/>
-      <c r="C29" s="16" t="n"/>
-      <c r="D29" s="16" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="17" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Цена в месяц, ₸</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Месяцев</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>За год, ₸</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="32" t="inlineStr">
+      <c r="A29" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B31" s="33">
+      <c r="B29" s="33">
         <f>SUM(Данные!$B$23:$B$30)*Данные!$B$9</f>
         <v>347760</v>
       </c>
-      <c r="C31" s="33" t="n">
+      <c r="C29" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="7">
-        <f>B31*C31</f>
+      <c r="D29" s="7">
+        <f>B29*C29</f>
         <v>347760</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="32" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B32" s="33">
+      <c r="B30" s="33">
         <f>SUM(Данные!$C$23:$C$30)*Данные!$B$9</f>
         <v>2367360</v>
       </c>
-      <c r="C32" s="33" t="n">
+      <c r="C30" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="D32" s="7">
-        <f>B32*C32</f>
+      <c r="D30" s="7">
+        <f>B30*C30</f>
         <v>2367360</v>
       </c>
     </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="n"/>
+      <c r="C32" s="16" t="n"/>
+      <c r="D32" s="16" t="n"/>
+    </row>
     <row r="33">
-      <c r="C33" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D33" s="12">
-        <f>SUM(D31:D32)</f>
-        <v>2715120</v>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
-        <is>
-          <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="n"/>
-      <c r="C35" s="16" t="n"/>
-      <c r="D35" s="16" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Статья</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="32" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Айыртау БП</t>
         </is>
       </c>
-      <c r="B37" s="33">
+      <c r="B34" s="33">
         <f>Данные!$B$48</f>
         <v>720000</v>
       </c>
-      <c r="C37" s="33" t="n">
+      <c r="C34" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="D37" s="7">
-        <f>B37*C37</f>
+      <c r="D34" s="7">
+        <f>B34*C34</f>
         <v>8640000</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="32" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Многоэтажки Д и Г</t>
         </is>
       </c>
-      <c r="B38" s="33">
+      <c r="B35" s="33">
         <f>Данные!$B$49</f>
         <v>1080000</v>
       </c>
-      <c r="C38" s="33" t="n">
+      <c r="C35" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="D38" s="7">
-        <f>B38*C38</f>
+      <c r="D35" s="7">
+        <f>B35*C35</f>
         <v>12960000</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="32" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · Площадки А, Б, Е, Ж, В (РМ), В</t>
         </is>
       </c>
-      <c r="B39" s="33">
+      <c r="B36" s="33">
         <f>Данные!$B$50</f>
         <v>3000000</v>
       </c>
-      <c r="C39" s="33" t="n">
+      <c r="C36" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="D39" s="7">
-        <f>B39*C39</f>
+      <c r="D36" s="7">
+        <f>B36*C36</f>
         <v>36000000</v>
       </c>
     </row>
-    <row r="40">
-      <c r="C40" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D40" s="12">
-        <f>SUM(D37:D39)</f>
-        <v>57600000</v>
-      </c>
-    </row>
-    <row r="41"/>
-    <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="25" t="inlineStr">
+    <row r="37"/>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="25" t="inlineStr">
         <is>
           <t>Состав площадок у Indigo и в нашем расчёте описан по-разному: у них шесть напольных площадок плюс «В (рем. молод)», у нас восемь площадок по контурам. Сопоставлять построчно нельзя, только суммарно.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="25" t="inlineStr">
+    <row r="39" ht="26" customHeight="1">
+      <c r="A39" s="25" t="inlineStr">
         <is>
           <t>Разовая закупка приманочных станций 1-го и 2-го контура показана справочно и в годовой итог не входит.</t>
         </is>
@@ -2820,9 +2740,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A38:D38"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A39:D39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2834,7 +2754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3038,224 +2958,180 @@
         <v>25497.5</v>
       </c>
     </row>
-    <row r="15">
-      <c r="C15" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D15" s="12">
-        <f>SUM(D9:D14)</f>
-        <v>1577717.5</v>
-      </c>
-    </row>
-    <row r="16"/>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>АЛЬТЕРНАТИВНЫЙ ВАРИАНТ INDIGO</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+    </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>АЛЬТЕРНАТИВНЫЙ ВАРИАНТ INDIGO</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="n"/>
-      <c r="C17" s="16" t="n"/>
-      <c r="D17" s="16" t="n"/>
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Цена в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Месяцев</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>За год, ₸</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Цена в месяц, ₸</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Месяцев</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>За год, ₸</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · частичная замена оборудования</t>
         </is>
       </c>
-      <c r="B19" s="33">
+      <c r="B18" s="33">
         <f>Данные!$B$45</f>
         <v>106800</v>
       </c>
-      <c r="C19" s="33" t="n">
+      <c r="C18" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="D19" s="7">
-        <f>B19*C19</f>
+      <c r="D18" s="7">
+        <f>B18*C18</f>
         <v>1281600</v>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
-      <c r="C20" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D20" s="12">
-        <f>SUM(D19:D19)</f>
-        <v>1281600</v>
-      </c>
-    </row>
-    <row r="21"/>
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>РАЗОВЫЕ ЗАТРАТЫ ШТАТА (СПРАВОЧНО)</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="16" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Цена в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Месяцев</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>За год, ₸</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>РАЗОВЫЕ ЗАТРАТЫ ШТАТА (СПРАВОЧНО)</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="n"/>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="16" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Цена в месяц, ₸</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Месяцев</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>За год, ₸</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="A22" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B24" s="33">
+      <c r="B22" s="33">
         <f>Данные!$B$21*Данные!$B$9</f>
         <v>38880</v>
       </c>
-      <c r="C24" s="33" t="n">
+      <c r="C22" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="7">
-        <f>B24*C24</f>
+      <c r="D22" s="7">
+        <f>B22*C22</f>
         <v>38880</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="32" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
-      <c r="B25" s="33">
+      <c r="B23" s="33">
         <f>Данные!$C$21*Данные!$B$9</f>
         <v>73440</v>
       </c>
-      <c r="C25" s="33" t="n">
+      <c r="C23" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="7">
-        <f>B25*C25</f>
+      <c r="D23" s="7">
+        <f>B23*C23</f>
         <v>73440</v>
       </c>
     </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+    </row>
     <row r="26">
-      <c r="C26" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D26" s="12">
-        <f>SUM(D24:D25)</f>
-        <v>112320</v>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
-        </is>
-      </c>
-      <c r="B28" s="16" t="n"/>
-      <c r="C28" s="16" t="n"/>
-      <c r="D28" s="16" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Статья</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Цена в месяц, ₸</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Месяцев</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>За год, ₸</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="32" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · дезинсекция</t>
         </is>
       </c>
-      <c r="B30" s="33">
+      <c r="B27" s="33">
         <f>Данные!$B$51</f>
         <v>100800</v>
       </c>
-      <c r="C30" s="33" t="n">
+      <c r="C27" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="D30" s="7">
-        <f>B30*C30</f>
+      <c r="D27" s="7">
+        <f>B27*C27</f>
         <v>1209600</v>
       </c>
     </row>
-    <row r="31">
-      <c r="C31" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D31" s="12">
-        <f>SUM(D30:D30)</f>
-        <v>1209600</v>
-      </c>
-    </row>
-    <row r="32"/>
-    <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="25" t="inlineStr">
+    <row r="28"/>
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="25" t="inlineStr">
         <is>
           <t>Нормы штата по инкубаторию: 18 точек 1-го контура, 34 второго, 12 клеевых третьего; 1 кг брикетов Pest Killer и 1 кг Зерноцида на обработку.</t>
         </is>
@@ -3263,7 +3139,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A29:D29"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3276,7 +3152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3422,151 +3298,118 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="C12" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D12" s="12">
-        <f>SUM(D9:D11)</f>
-        <v>3674400</v>
-      </c>
-    </row>
-    <row r="13"/>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>АЛЬТЕРНАТИВНЫЙ ВАРИАНТ INDIGO</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="16" t="n"/>
+      <c r="D13" s="16" t="n"/>
+    </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>АЛЬТЕРНАТИВНЫЙ ВАРИАНТ INDIGO</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="n"/>
-      <c r="C14" s="16" t="n"/>
-      <c r="D14" s="16" t="n"/>
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Цена в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Месяцев</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>За год, ₸</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Цена в месяц, ₸</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Месяцев</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>За год, ₸</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · частичная замена оборудования</t>
         </is>
       </c>
-      <c r="B16" s="33">
+      <c r="B15" s="33">
         <f>Данные!$B$47</f>
         <v>106800</v>
       </c>
-      <c r="C16" s="33" t="n">
+      <c r="C15" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="D16" s="7">
-        <f>B16*C16</f>
+      <c r="D15" s="7">
+        <f>B15*C15</f>
         <v>1281600</v>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
-      <c r="C17" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D17" s="12">
-        <f>SUM(D16:D16)</f>
-        <v>1281600</v>
-      </c>
-    </row>
-    <row r="18"/>
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Цена в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Месяцев</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>За год, ₸</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>СПРАВОЧНО: ДЕЗИНСЕКЦИЯ — В СРАВНЕНИЕ НЕ ВХОДИТ</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="n"/>
-      <c r="C19" s="16" t="n"/>
-      <c r="D19" s="16" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Цена в месяц, ₸</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Месяцев</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>За год, ₸</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>Indigo Solutions · дезинсекция</t>
         </is>
       </c>
-      <c r="B21" s="33">
+      <c r="B19" s="33">
         <f>Данные!$B$52</f>
         <v>160800</v>
       </c>
-      <c r="C21" s="33" t="n">
+      <c r="C19" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="D21" s="7">
-        <f>B21*C21</f>
+      <c r="D19" s="7">
+        <f>B19*C19</f>
         <v>1929600</v>
       </c>
     </row>
-    <row r="22">
-      <c r="C22" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D22" s="12">
-        <f>SUM(D21:D21)</f>
-        <v>1929600</v>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="25" t="inlineStr">
+    <row r="20"/>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>Строки не полностью сопоставимы: у Pest Hunters 180 000 ₸ включают и дератизацию, и дезинсекцию, у Indigo эти услуги разделены — 126 200 ₸ дератизация и 160 800 ₸ дезинсекция.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="25" t="inlineStr">
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>По штату УКПФ нормы расхода на ЗПП не заданы, поэтому в расчёте ноль.</t>
         </is>
@@ -3574,8 +3417,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A21:D21"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3588,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3734,20 +3577,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="C12" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D12" s="12">
-        <f>SUM(D9:D11)</f>
-        <v>720000</v>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="25" t="inlineStr">
+    <row r="12"/>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>С января по март договор не действует, поэтому в году девять оплачиваемых месяцев.</t>
         </is>
@@ -3755,7 +3587,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A13:D13"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3768,7 +3600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3971,107 +3803,85 @@
         <v>33146.75</v>
       </c>
     </row>
-    <row r="15">
-      <c r="C15" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D15" s="12">
-        <f>SUM(D9:D14)</f>
-        <v>204506.75</v>
-      </c>
-    </row>
-    <row r="16"/>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>РАЗОВЫЕ ЗАТРАТЫ ШТАТА (СПРАВОЧНО)</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+    </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>РАЗОВЫЕ ЗАТРАТЫ ШТАТА (СПРАВОЧНО)</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="n"/>
-      <c r="C17" s="16" t="n"/>
-      <c r="D17" s="16" t="n"/>
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Цена в месяц, ₸</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Месяцев</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>За год, ₸</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Статья</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Цена в месяц, ₸</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Месяцев</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>За год, ₸</t>
-        </is>
+      <c r="A18" s="32" t="inlineStr">
+        <is>
+          <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
+        </is>
+      </c>
+      <c r="B18" s="33">
+        <f>Данные!$B$22*Данные!$B$9</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="7">
+        <f>B18*C18</f>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="32" t="inlineStr">
         <is>
-          <t>Штат УКПФ · Приманочные станции 1-го контура — разовая закупка</t>
+          <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
         </is>
       </c>
       <c r="B19" s="33">
-        <f>Данные!$B$22*Данные!$B$9</f>
-        <v>0</v>
+        <f>Данные!$C$22*Данные!$B$9</f>
+        <v>84240</v>
       </c>
       <c r="C19" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="7">
         <f>B19*C19</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="32" t="inlineStr">
-        <is>
-          <t>Штат УКПФ · Приманочные станции 2-го контура — разовая закупка</t>
-        </is>
-      </c>
-      <c r="B20" s="33">
-        <f>Данные!$C$22*Данные!$B$9</f>
         <v>84240</v>
       </c>
-      <c r="C20" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="7">
-        <f>B20*C20</f>
-        <v>84240</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="C21" s="34" t="inlineStr">
-        <is>
-          <t>Итого</t>
-        </is>
-      </c>
-      <c r="D21" s="12">
-        <f>SUM(D19:D20)</f>
-        <v>84240</v>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="25" t="inlineStr">
+    </row>
+    <row r="20"/>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>Клеевые станции по корпусам: Б — 11, Ж — 5, Е — 6, В — 6, В (РМ) — 6, Д — 3, Г — 3, БП-12 — 6, БП-13 — 6, БП-14 — 6, А — 5. Приманочные: 4, 2, 3, 3, 3, 4, 3, 5, 5, 5, 2.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="25" t="inlineStr">
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>Норма 1,3 кг брикетов Pest Killer по АБК — приблизительная оценка, требует подтверждения. Зерноцид по АБК не заявлен.</t>
         </is>
@@ -4079,8 +3889,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A21:D21"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4196,7 +4006,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="35" t="inlineStr">
+      <c r="A9" s="34" t="inlineStr">
         <is>
           <t>Зарплата за год</t>
         </is>
@@ -4227,47 +4037,47 @@
       <c r="I11" s="16" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="inlineStr">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B12" s="37" t="inlineStr">
+      <c r="B12" s="36" t="inlineStr">
         <is>
           <t>Клеевых 3-го к., шт/мес лето</t>
         </is>
       </c>
-      <c r="C12" s="37" t="inlineStr">
+      <c r="C12" s="36" t="inlineStr">
         <is>
           <t>Клеевых 3-го к., шт/мес зима</t>
         </is>
       </c>
-      <c r="D12" s="37" t="inlineStr">
+      <c r="D12" s="36" t="inlineStr">
         <is>
           <t>Клеевые за год, ₸</t>
         </is>
       </c>
-      <c r="E12" s="37" t="inlineStr">
+      <c r="E12" s="36" t="inlineStr">
         <is>
           <t>Зерноцид, кг/мес</t>
         </is>
       </c>
-      <c r="F12" s="37" t="inlineStr">
+      <c r="F12" s="36" t="inlineStr">
         <is>
           <t>Зерноцид за год, ₸</t>
         </is>
       </c>
-      <c r="G12" s="37" t="inlineStr">
+      <c r="G12" s="36" t="inlineStr">
         <is>
           <t>Pest Killer, кг/мес</t>
         </is>
       </c>
-      <c r="H12" s="37" t="inlineStr">
+      <c r="H12" s="36" t="inlineStr">
         <is>
           <t>Pest Killer за год, ₸</t>
         </is>
       </c>
-      <c r="I12" s="37" t="inlineStr">
+      <c r="I12" s="36" t="inlineStr">
         <is>
           <t>Материалы за год, ₸</t>
         </is>
@@ -4279,11 +4089,11 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B13" s="52">
+      <c r="B13" s="51">
         <f>Данные!$D$20</f>
         <v>0</v>
       </c>
-      <c r="C13" s="52">
+      <c r="C13" s="51">
         <f>Данные!$D$20*2</f>
         <v>0</v>
       </c>
@@ -4291,7 +4101,7 @@
         <f>B13*Данные!$B$8*Данные!$B$15+C13*Данные!$B$8*Данные!$B$16</f>
         <v>0</v>
       </c>
-      <c r="E13" s="53">
+      <c r="E13" s="52">
         <f>Данные!$G$20</f>
         <v>0</v>
       </c>
@@ -4299,7 +4109,7 @@
         <f>E13*Данные!$B$6*Данные!$B$15</f>
         <v>0</v>
       </c>
-      <c r="G13" s="53">
+      <c r="G13" s="52">
         <f>Данные!$F$20</f>
         <v>1</v>
       </c>
@@ -4318,11 +4128,11 @@
           <t>Бройлерные площадки · 8 шт</t>
         </is>
       </c>
-      <c r="B14" s="52">
+      <c r="B14" s="51">
         <f>SUM(Данные!$D$23:$D$30)</f>
         <v>268</v>
       </c>
-      <c r="C14" s="52">
+      <c r="C14" s="51">
         <f>SUM(Данные!$D$23:$D$30)*2</f>
         <v>536</v>
       </c>
@@ -4330,7 +4140,7 @@
         <f>B14*Данные!$B$8*Данные!$B$15+C14*Данные!$B$8*Данные!$B$16</f>
         <v>728960</v>
       </c>
-      <c r="E14" s="53">
+      <c r="E14" s="52">
         <f>SUM(Данные!$G$23:$G$30)</f>
         <v>15</v>
       </c>
@@ -4338,7 +4148,7 @@
         <f>E14*Данные!$B$6*Данные!$B$15</f>
         <v>77700</v>
       </c>
-      <c r="G14" s="53">
+      <c r="G14" s="52">
         <f>SUM(Данные!$F$23:$F$30)</f>
         <v>17</v>
       </c>
@@ -4357,11 +4167,11 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B15" s="52">
+      <c r="B15" s="51">
         <f>Данные!$D$21</f>
         <v>12</v>
       </c>
-      <c r="C15" s="52">
+      <c r="C15" s="51">
         <f>Данные!$D$21*2</f>
         <v>24</v>
       </c>
@@ -4369,7 +4179,7 @@
         <f>B15*Данные!$B$8*Данные!$B$15+C15*Данные!$B$8*Данные!$B$16</f>
         <v>32640</v>
       </c>
-      <c r="E15" s="53">
+      <c r="E15" s="52">
         <f>Данные!$G$21</f>
         <v>1</v>
       </c>
@@ -4377,7 +4187,7 @@
         <f>E15*Данные!$B$6*Данные!$B$15</f>
         <v>5180</v>
       </c>
-      <c r="G15" s="53">
+      <c r="G15" s="52">
         <f>Данные!$F$21</f>
         <v>1</v>
       </c>
@@ -4396,11 +4206,11 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B16" s="52">
+      <c r="B16" s="51">
         <f>Данные!$D$22</f>
         <v>63</v>
       </c>
-      <c r="C16" s="52">
+      <c r="C16" s="51">
         <f>Данные!$D$22*2</f>
         <v>126</v>
       </c>
@@ -4408,7 +4218,7 @@
         <f>B16*Данные!$B$8*Данные!$B$15+C16*Данные!$B$8*Данные!$B$16</f>
         <v>171360</v>
       </c>
-      <c r="E16" s="53">
+      <c r="E16" s="52">
         <f>Данные!$G$22</f>
         <v>0</v>
       </c>
@@ -4416,7 +4226,7 @@
         <f>E16*Данные!$B$6*Данные!$B$15</f>
         <v>0</v>
       </c>
-      <c r="G16" s="53">
+      <c r="G16" s="52">
         <f>Данные!$F$22</f>
         <v>1.3</v>
       </c>
@@ -4459,7 +4269,7 @@
         <f>SUM(D13:D17)</f>
         <v>932960</v>
       </c>
-      <c r="E18" s="54">
+      <c r="E18" s="53">
         <f>SUM(E13:E17)</f>
         <v>16</v>
       </c>
@@ -4467,7 +4277,7 @@
         <f>SUM(F13:F17)</f>
         <v>82880</v>
       </c>
-      <c r="G18" s="54">
+      <c r="G18" s="53">
         <f>SUM(G13:G17)</f>
         <v>20.3</v>
       </c>
@@ -4531,15 +4341,15 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B22" s="52">
+      <c r="B22" s="51">
         <f>Данные!$B$20</f>
         <v>0</v>
       </c>
-      <c r="C22" s="52">
+      <c r="C22" s="51">
         <f>Данные!$C$20</f>
         <v>29</v>
       </c>
-      <c r="D22" s="52">
+      <c r="D22" s="51">
         <f>B22+C22</f>
         <v>29</v>
       </c>
@@ -4558,15 +4368,15 @@
           <t>Бройлерные площадки · 8 шт</t>
         </is>
       </c>
-      <c r="B23" s="52">
+      <c r="B23" s="51">
         <f>SUM(Данные!$B$23:$B$30)</f>
         <v>161</v>
       </c>
-      <c r="C23" s="52">
+      <c r="C23" s="51">
         <f>SUM(Данные!$C$23:$C$30)</f>
         <v>1096</v>
       </c>
-      <c r="D23" s="52">
+      <c r="D23" s="51">
         <f>B23+C23</f>
         <v>1257</v>
       </c>
@@ -4585,15 +4395,15 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B24" s="52">
+      <c r="B24" s="51">
         <f>Данные!$B$21</f>
         <v>18</v>
       </c>
-      <c r="C24" s="52">
+      <c r="C24" s="51">
         <f>Данные!$C$21</f>
         <v>34</v>
       </c>
-      <c r="D24" s="52">
+      <c r="D24" s="51">
         <f>B24+C24</f>
         <v>52</v>
       </c>
@@ -4612,15 +4422,15 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B25" s="52">
+      <c r="B25" s="51">
         <f>Данные!$B$22</f>
         <v>0</v>
       </c>
-      <c r="C25" s="52">
+      <c r="C25" s="51">
         <f>Данные!$C$22</f>
         <v>39</v>
       </c>
-      <c r="D25" s="52">
+      <c r="D25" s="51">
         <f>B25+C25</f>
         <v>39</v>
       </c>
@@ -4639,15 +4449,15 @@
           <t>ИТОГО РАЗОВО</t>
         </is>
       </c>
-      <c r="B26" s="55">
+      <c r="B26" s="54">
         <f>SUM(B22:B25)</f>
         <v>179</v>
       </c>
-      <c r="C26" s="55">
+      <c r="C26" s="54">
         <f>SUM(C22:C25)</f>
         <v>1198</v>
       </c>
-      <c r="D26" s="55">
+      <c r="D26" s="54">
         <f>SUM(D22:D25)</f>
         <v>1377</v>
       </c>
@@ -4671,32 +4481,32 @@
       <c r="F28" s="16" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="36" t="inlineStr">
+      <c r="A29" s="35" t="inlineStr">
         <is>
           <t>Численность, чел.</t>
         </is>
       </c>
-      <c r="B29" s="37" t="inlineStr">
+      <c r="B29" s="36" t="inlineStr">
         <is>
           <t>ЗП в месяц, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="C29" s="37" t="inlineStr">
+      <c r="C29" s="36" t="inlineStr">
         <is>
           <t>ЗП за год, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="D29" s="37" t="inlineStr">
+      <c r="D29" s="36" t="inlineStr">
         <is>
           <t>Материалы за год, ₸</t>
         </is>
       </c>
-      <c r="E29" s="37" t="inlineStr">
+      <c r="E29" s="36" t="inlineStr">
         <is>
           <t>Итого за год, ₸ · оклад 258 488</t>
         </is>
       </c>
-      <c r="F29" s="37" t="inlineStr">
+      <c r="F29" s="36" t="inlineStr">
         <is>
           <t>Итого за год, ₸ · оклад 350 000</t>
         </is>
@@ -5024,7 +4834,7 @@
           <t>Зерноцид</t>
         </is>
       </c>
-      <c r="B6" s="42" t="n">
+      <c r="B6" s="41" t="n">
         <v>740</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -5032,7 +4842,7 @@
           <t>₸/кг</t>
         </is>
       </c>
-      <c r="H6" s="43" t="inlineStr">
+      <c r="H6" s="42" t="inlineStr">
         <is>
           <t>внутренние данные УКПФ</t>
         </is>
@@ -5044,7 +4854,7 @@
           <t>Pest Killer, брикеты</t>
         </is>
       </c>
-      <c r="B7" s="42" t="n">
+      <c r="B7" s="41" t="n">
         <v>3642.5</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -5052,7 +4862,7 @@
           <t>₸/кг</t>
         </is>
       </c>
-      <c r="H7" s="43" t="inlineStr">
+      <c r="H7" s="42" t="inlineStr">
         <is>
           <t>перенесено из прежнего расчёта по ККЗ; в исходных нормах цены не было</t>
         </is>
@@ -5064,7 +4874,7 @@
           <t>Клеевая станция 3-го контура</t>
         </is>
       </c>
-      <c r="B8" s="42" t="n">
+      <c r="B8" s="41" t="n">
         <v>160</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -5072,7 +4882,7 @@
           <t>₸/шт</t>
         </is>
       </c>
-      <c r="H8" s="43" t="inlineStr">
+      <c r="H8" s="42" t="inlineStr">
         <is>
           <t>внутренние данные УКПФ, расходуется ежемесячно</t>
         </is>
@@ -5084,7 +4894,7 @@
           <t>Приманочная станция 1–2 контура</t>
         </is>
       </c>
-      <c r="B9" s="42" t="n">
+      <c r="B9" s="41" t="n">
         <v>2160</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -5092,7 +4902,7 @@
           <t>₸/шт</t>
         </is>
       </c>
-      <c r="H9" s="43" t="inlineStr">
+      <c r="H9" s="42" t="inlineStr">
         <is>
           <t>разовая закупка; цена из прежнего расчёта по ККЗ (29 шт = 62 640 ₸)</t>
         </is>
@@ -5104,7 +4914,7 @@
           <t>Бутылка</t>
         </is>
       </c>
-      <c r="B10" s="42" t="n">
+      <c r="B10" s="41" t="n">
         <v>68</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -5112,7 +4922,7 @@
           <t>₸/шт</t>
         </is>
       </c>
-      <c r="H10" s="43" t="inlineStr">
+      <c r="H10" s="42" t="inlineStr">
         <is>
           <t>внутренние данные УКПФ</t>
         </is>
@@ -5124,7 +4934,7 @@
           <t>Бутылки, расход</t>
         </is>
       </c>
-      <c r="B11" s="42" t="n">
+      <c r="B11" s="41" t="n">
         <v>40</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -5132,7 +4942,7 @@
           <t>шт/мес</t>
         </is>
       </c>
-      <c r="H11" s="43" t="inlineStr">
+      <c r="H11" s="42" t="inlineStr">
         <is>
           <t>тёплый сезон, зимой ноль; оценка, по объектам не разносится</t>
         </is>
@@ -5144,7 +4954,7 @@
           <t>Оклад дератизатора · вариант 1</t>
         </is>
       </c>
-      <c r="B12" s="42" t="n">
+      <c r="B12" s="41" t="n">
         <v>258488</v>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -5152,7 +4962,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H12" s="43" t="inlineStr">
+      <c r="H12" s="42" t="inlineStr">
         <is>
           <t>действующий оклад</t>
         </is>
@@ -5164,7 +4974,7 @@
           <t>Оклад дератизатора · вариант 2</t>
         </is>
       </c>
-      <c r="B13" s="42" t="n">
+      <c r="B13" s="41" t="n">
         <v>350000</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -5172,7 +4982,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H13" s="43" t="inlineStr">
+      <c r="H13" s="42" t="inlineStr">
         <is>
           <t>альтернативный уровень для сравнения</t>
         </is>
@@ -5184,7 +4994,7 @@
           <t>Численность штата</t>
         </is>
       </c>
-      <c r="B14" s="42" t="n">
+      <c r="B14" s="41" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -5192,7 +5002,7 @@
           <t>чел.</t>
         </is>
       </c>
-      <c r="H14" s="43" t="inlineStr">
+      <c r="H14" s="42" t="inlineStr">
         <is>
           <t>измените — пересчитаются все листы</t>
         </is>
@@ -5204,7 +5014,7 @@
           <t>Тёплых месяцев (апрель — октябрь)</t>
         </is>
       </c>
-      <c r="B15" s="42" t="n">
+      <c r="B15" s="41" t="n">
         <v>7</v>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -5212,7 +5022,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H15" s="43" t="inlineStr">
+      <c r="H15" s="42" t="inlineStr">
         <is>
           <t>заряжаются все три контура</t>
         </is>
@@ -5224,7 +5034,7 @@
           <t>Зимних месяцев (ноябрь — март)</t>
         </is>
       </c>
-      <c r="B16" s="42" t="n">
+      <c r="B16" s="41" t="n">
         <v>5</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -5232,7 +5042,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H16" s="43" t="inlineStr">
+      <c r="H16" s="42" t="inlineStr">
         <is>
           <t>1-й и 2-й контуры не заряжаются, 3-й обслуживается вдвое</t>
         </is>
@@ -5254,42 +5064,42 @@
       <c r="H18" s="16" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="36" t="inlineStr">
+      <c r="A19" s="35" t="inlineStr">
         <is>
           <t>Объект</t>
         </is>
       </c>
-      <c r="B19" s="37" t="inlineStr">
+      <c r="B19" s="36" t="inlineStr">
         <is>
           <t>1-й контур, шт</t>
         </is>
       </c>
-      <c r="C19" s="37" t="inlineStr">
+      <c r="C19" s="36" t="inlineStr">
         <is>
           <t>2-й контур, шт</t>
         </is>
       </c>
-      <c r="D19" s="37" t="inlineStr">
+      <c r="D19" s="36" t="inlineStr">
         <is>
           <t>3-й контур, шт</t>
         </is>
       </c>
-      <c r="E19" s="37" t="inlineStr">
+      <c r="E19" s="36" t="inlineStr">
         <is>
           <t>Всего точек, шт</t>
         </is>
       </c>
-      <c r="F19" s="37" t="inlineStr">
+      <c r="F19" s="36" t="inlineStr">
         <is>
           <t>Pest Killer, кг</t>
         </is>
       </c>
-      <c r="G19" s="37" t="inlineStr">
+      <c r="G19" s="36" t="inlineStr">
         <is>
           <t>Зерноцид, кг</t>
         </is>
       </c>
-      <c r="H19" s="37" t="inlineStr">
+      <c r="H19" s="36" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
@@ -5301,26 +5111,26 @@
           <t>ККЗ · кормоцех</t>
         </is>
       </c>
-      <c r="B20" s="42" t="n">
+      <c r="B20" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="C20" s="42" t="n">
+      <c r="C20" s="41" t="n">
         <v>29</v>
       </c>
-      <c r="D20" s="42" t="n">
+      <c r="D20" s="41" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="7">
         <f>SUM(B20:D20)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="56" t="n">
+      <c r="F20" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="56" t="n">
+      <c r="G20" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="43" t="inlineStr">
+      <c r="H20" s="42" t="inlineStr">
         <is>
           <t>29 приманочных станций 2-го контура</t>
         </is>
@@ -5332,26 +5142,26 @@
           <t>Инкубаторий</t>
         </is>
       </c>
-      <c r="B21" s="42" t="n">
+      <c r="B21" s="41" t="n">
         <v>18</v>
       </c>
-      <c r="C21" s="42" t="n">
+      <c r="C21" s="41" t="n">
         <v>34</v>
       </c>
-      <c r="D21" s="42" t="n">
+      <c r="D21" s="41" t="n">
         <v>12</v>
       </c>
       <c r="E21" s="7">
         <f>SUM(B21:D21)</f>
         <v>18</v>
       </c>
-      <c r="F21" s="56" t="n">
+      <c r="F21" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="56" t="n">
+      <c r="G21" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="43" t="inlineStr"/>
+      <c r="H21" s="42" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -5359,26 +5169,26 @@
           <t>АБК · 11 корпусов</t>
         </is>
       </c>
-      <c r="B22" s="42" t="n">
+      <c r="B22" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="42" t="n">
+      <c r="C22" s="41" t="n">
         <v>39</v>
       </c>
-      <c r="D22" s="42" t="n">
+      <c r="D22" s="41" t="n">
         <v>63</v>
       </c>
       <c r="E22" s="7">
         <f>SUM(B22:D22)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="56" t="n">
+      <c r="F22" s="55" t="n">
         <v>1.3</v>
       </c>
-      <c r="G22" s="56" t="n">
+      <c r="G22" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="43" t="inlineStr">
+      <c r="H22" s="42" t="inlineStr">
         <is>
           <t>1,3 кг — приблизительная оценка, требует подтверждения</t>
         </is>
@@ -5390,26 +5200,26 @@
           <t>Площадка А</t>
         </is>
       </c>
-      <c r="B23" s="42" t="n">
+      <c r="B23" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="C23" s="42" t="n">
+      <c r="C23" s="41" t="n">
         <v>147</v>
       </c>
-      <c r="D23" s="42" t="n">
+      <c r="D23" s="41" t="n">
         <v>20</v>
       </c>
       <c r="E23" s="7">
         <f>SUM(B23:D23)</f>
         <v>13</v>
       </c>
-      <c r="F23" s="56" t="n">
+      <c r="F23" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="56" t="n">
+      <c r="G23" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="43" t="inlineStr"/>
+      <c r="H23" s="42" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -5417,26 +5227,26 @@
           <t>Площадка Б</t>
         </is>
       </c>
-      <c r="B24" s="42" t="n">
+      <c r="B24" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C24" s="42" t="n">
+      <c r="C24" s="41" t="n">
         <v>146</v>
       </c>
-      <c r="D24" s="42" t="n">
+      <c r="D24" s="41" t="n">
         <v>20</v>
       </c>
       <c r="E24" s="7">
         <f>SUM(B24:D24)</f>
         <v>17</v>
       </c>
-      <c r="F24" s="56" t="n">
+      <c r="F24" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="56" t="n">
+      <c r="G24" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="H24" s="43" t="inlineStr"/>
+      <c r="H24" s="42" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -5444,26 +5254,26 @@
           <t>В / Восточка</t>
         </is>
       </c>
-      <c r="B25" s="42" t="n">
+      <c r="B25" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="C25" s="42" t="n">
+      <c r="C25" s="41" t="n">
         <v>239</v>
       </c>
-      <c r="D25" s="42" t="n">
+      <c r="D25" s="41" t="n">
         <v>30</v>
       </c>
       <c r="E25" s="7">
         <f>SUM(B25:D25)</f>
         <v>50</v>
       </c>
-      <c r="F25" s="56" t="n">
+      <c r="F25" s="55" t="n">
         <v>3.5</v>
       </c>
-      <c r="G25" s="56" t="n">
+      <c r="G25" s="55" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="43" t="inlineStr"/>
+      <c r="H25" s="42" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -5471,26 +5281,26 @@
           <t>Площадка Г</t>
         </is>
       </c>
-      <c r="B26" s="42" t="n">
+      <c r="B26" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C26" s="42" t="n">
+      <c r="C26" s="41" t="n">
         <v>88</v>
       </c>
-      <c r="D26" s="42" t="n">
+      <c r="D26" s="41" t="n">
         <v>80</v>
       </c>
       <c r="E26" s="7">
         <f>SUM(B26:D26)</f>
         <v>17</v>
       </c>
-      <c r="F26" s="56" t="n">
+      <c r="F26" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="56" t="n">
+      <c r="G26" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="H26" s="43" t="inlineStr"/>
+      <c r="H26" s="42" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -5498,26 +5308,26 @@
           <t>Площадка Д</t>
         </is>
       </c>
-      <c r="B27" s="42" t="n">
+      <c r="B27" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="C27" s="42" t="n">
+      <c r="C27" s="41" t="n">
         <v>69</v>
       </c>
-      <c r="D27" s="42" t="n">
+      <c r="D27" s="41" t="n">
         <v>64</v>
       </c>
       <c r="E27" s="7">
         <f>SUM(B27:D27)</f>
         <v>15</v>
       </c>
-      <c r="F27" s="56" t="n">
+      <c r="F27" s="55" t="n">
         <v>1.5</v>
       </c>
-      <c r="G27" s="56" t="n">
+      <c r="G27" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="43" t="inlineStr"/>
+      <c r="H27" s="42" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -5525,26 +5335,26 @@
           <t>Площадка Е</t>
         </is>
       </c>
-      <c r="B28" s="42" t="n">
+      <c r="B28" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="C28" s="42" t="n">
+      <c r="C28" s="41" t="n">
         <v>147</v>
       </c>
-      <c r="D28" s="42" t="n">
+      <c r="D28" s="41" t="n">
         <v>20</v>
       </c>
       <c r="E28" s="7">
         <f>SUM(B28:D28)</f>
         <v>13</v>
       </c>
-      <c r="F28" s="56" t="n">
+      <c r="F28" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="56" t="n">
+      <c r="G28" s="55" t="n">
         <v>2</v>
       </c>
-      <c r="H28" s="43" t="inlineStr"/>
+      <c r="H28" s="42" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -5552,26 +5362,26 @@
           <t>Площадка Ж</t>
         </is>
       </c>
-      <c r="B29" s="42" t="n">
+      <c r="B29" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="C29" s="42" t="n">
+      <c r="C29" s="41" t="n">
         <v>73</v>
       </c>
-      <c r="D29" s="42" t="n">
+      <c r="D29" s="41" t="n">
         <v>10</v>
       </c>
       <c r="E29" s="7">
         <f>SUM(B29:D29)</f>
         <v>17</v>
       </c>
-      <c r="F29" s="56" t="n">
+      <c r="F29" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="56" t="n">
+      <c r="G29" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="H29" s="43" t="inlineStr"/>
+      <c r="H29" s="42" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -5579,26 +5389,26 @@
           <t>Айыртау (БП)</t>
         </is>
       </c>
-      <c r="B30" s="42" t="n">
+      <c r="B30" s="41" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="42" t="n">
+      <c r="C30" s="41" t="n">
         <v>187</v>
       </c>
-      <c r="D30" s="42" t="n">
+      <c r="D30" s="41" t="n">
         <v>24</v>
       </c>
       <c r="E30" s="7">
         <f>SUM(B30:D30)</f>
         <v>19</v>
       </c>
-      <c r="F30" s="56" t="n">
+      <c r="F30" s="55" t="n">
         <v>3</v>
       </c>
-      <c r="G30" s="56" t="n">
+      <c r="G30" s="55" t="n">
         <v>3</v>
       </c>
-      <c r="H30" s="43" t="inlineStr"/>
+      <c r="H30" s="42" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -5610,9 +5420,9 @@
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
-      <c r="F31" s="53" t="n"/>
-      <c r="G31" s="53" t="n"/>
-      <c r="H31" s="43" t="inlineStr">
+      <c r="F31" s="52" t="n"/>
+      <c r="G31" s="52" t="n"/>
+      <c r="H31" s="42" t="inlineStr">
         <is>
           <t>нормы расхода не заданы</t>
         </is>
@@ -5628,9 +5438,9 @@
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
-      <c r="F32" s="53" t="n"/>
-      <c r="G32" s="53" t="n"/>
-      <c r="H32" s="43" t="inlineStr">
+      <c r="F32" s="52" t="n"/>
+      <c r="G32" s="52" t="n"/>
+      <c r="H32" s="42" t="inlineStr">
         <is>
           <t>нормы расхода не заданы</t>
         </is>
@@ -5658,11 +5468,11 @@
         <f>SUM(E20:E32)</f>
         <v>179</v>
       </c>
-      <c r="F33" s="54">
+      <c r="F33" s="53">
         <f>SUM(F20:F32)</f>
         <v>20.3</v>
       </c>
-      <c r="G33" s="54">
+      <c r="G33" s="53">
         <f>SUM(G20:G32)</f>
         <v>16</v>
       </c>
@@ -5715,7 +5525,7 @@
           <t>Indigo · ККЗ, дератизация</t>
         </is>
       </c>
-      <c r="B37" s="42" t="n">
+      <c r="B37" s="41" t="n">
         <v>96600</v>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -5723,7 +5533,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H37" s="43" t="inlineStr">
+      <c r="H37" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); барьер вокруг периметра кормоцеха и грязный барьер</t>
         </is>
@@ -5735,7 +5545,7 @@
           <t>Indigo · Айыртау БП, полная замена</t>
         </is>
       </c>
-      <c r="B38" s="42" t="n">
+      <c r="B38" s="41" t="n">
         <v>618400</v>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -5743,7 +5553,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H38" s="43" t="inlineStr">
+      <c r="H38" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 180 ед. оборудования</t>
         </is>
@@ -5755,7 +5565,7 @@
           <t>Indigo · Айыртау БП, частичная замена</t>
         </is>
       </c>
-      <c r="B39" s="42" t="n">
+      <c r="B39" s="41" t="n">
         <v>478400</v>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -5763,7 +5573,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H39" s="43" t="inlineStr">
+      <c r="H39" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5775,7 +5585,7 @@
           <t>Indigo · Многоэтажки Д и Г, полная замена</t>
         </is>
       </c>
-      <c r="B40" s="42" t="n">
+      <c r="B40" s="41" t="n">
         <v>569800</v>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -5783,7 +5593,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H40" s="43" t="inlineStr">
+      <c r="H40" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 166 ед. оборудования</t>
         </is>
@@ -5795,7 +5605,7 @@
           <t>Indigo · Многоэтажки Д и Г, частичная замена</t>
         </is>
       </c>
-      <c r="B41" s="42" t="n">
+      <c r="B41" s="41" t="n">
         <v>440700</v>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -5803,7 +5613,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H41" s="43" t="inlineStr">
+      <c r="H41" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5815,7 +5625,7 @@
           <t>Indigo · Площадки А,Б,Е,Ж,В,В(РМ), полная</t>
         </is>
       </c>
-      <c r="B42" s="42" t="n">
+      <c r="B42" s="41" t="n">
         <v>2599100</v>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -5823,7 +5633,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H42" s="43" t="inlineStr">
+      <c r="H42" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 793 ед. оборудования</t>
         </is>
@@ -5835,7 +5645,7 @@
           <t>Indigo · Площадки А,Б,Е,Ж,В,В(РМ), частичная</t>
         </is>
       </c>
-      <c r="B43" s="42" t="n">
+      <c r="B43" s="41" t="n">
         <v>2010300</v>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -5843,7 +5653,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H43" s="43" t="inlineStr">
+      <c r="H43" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5855,7 +5665,7 @@
           <t>Indigo · Инкубаторий, полная замена</t>
         </is>
       </c>
-      <c r="B44" s="42" t="n">
+      <c r="B44" s="41" t="n">
         <v>126200</v>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -5863,7 +5673,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H44" s="43" t="inlineStr">
+      <c r="H44" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС); 48 ед. оборудования</t>
         </is>
@@ -5875,7 +5685,7 @@
           <t>Indigo · Инкубаторий, частичная замена</t>
         </is>
       </c>
-      <c r="B45" s="42" t="n">
+      <c r="B45" s="41" t="n">
         <v>106800</v>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -5883,7 +5693,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H45" s="43" t="inlineStr">
+      <c r="H45" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5895,7 +5705,7 @@
           <t>Indigo · ЗПП, полная замена</t>
         </is>
       </c>
-      <c r="B46" s="42" t="n">
+      <c r="B46" s="41" t="n">
         <v>126200</v>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -5903,7 +5713,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H46" s="43" t="inlineStr">
+      <c r="H46" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5915,7 +5725,7 @@
           <t>Indigo · ЗПП, частичная замена</t>
         </is>
       </c>
-      <c r="B47" s="42" t="n">
+      <c r="B47" s="41" t="n">
         <v>106800</v>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -5923,7 +5733,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H47" s="43" t="inlineStr">
+      <c r="H47" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5935,7 +5745,7 @@
           <t>Indigo · дезинсекция, Айыртау БП</t>
         </is>
       </c>
-      <c r="B48" s="42" t="n">
+      <c r="B48" s="41" t="n">
         <v>720000</v>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -5943,7 +5753,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H48" s="43" t="inlineStr">
+      <c r="H48" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5955,7 +5765,7 @@
           <t>Indigo · дезинсекция, Многоэтажки</t>
         </is>
       </c>
-      <c r="B49" s="42" t="n">
+      <c r="B49" s="41" t="n">
         <v>1080000</v>
       </c>
       <c r="C49" s="6" t="inlineStr">
@@ -5963,7 +5773,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H49" s="43" t="inlineStr">
+      <c r="H49" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5975,7 +5785,7 @@
           <t>Indigo · дезинсекция, Площадки</t>
         </is>
       </c>
-      <c r="B50" s="42" t="n">
+      <c r="B50" s="41" t="n">
         <v>3000000</v>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -5983,7 +5793,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H50" s="43" t="inlineStr">
+      <c r="H50" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -5995,7 +5805,7 @@
           <t>Indigo · дезинсекция, Инкубаторий</t>
         </is>
       </c>
-      <c r="B51" s="42" t="n">
+      <c r="B51" s="41" t="n">
         <v>100800</v>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -6003,7 +5813,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H51" s="43" t="inlineStr">
+      <c r="H51" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -6015,7 +5825,7 @@
           <t>Indigo · дезинсекция, ЗПП</t>
         </is>
       </c>
-      <c r="B52" s="42" t="n">
+      <c r="B52" s="41" t="n">
         <v>160800</v>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -6023,7 +5833,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H52" s="43" t="inlineStr">
+      <c r="H52" s="42" t="inlineStr">
         <is>
           <t>Indigo Solutions, КП от 19.08.2026 (цены включают НДС)</t>
         </is>
@@ -6035,7 +5845,7 @@
           <t>Pest Hunters · ККЗ, дератизация</t>
         </is>
       </c>
-      <c r="B53" s="42" t="n">
+      <c r="B53" s="41" t="n">
         <v>75000</v>
       </c>
       <c r="C53" s="6" t="inlineStr">
@@ -6043,7 +5853,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H53" s="43" t="inlineStr">
+      <c r="H53" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -6055,7 +5865,7 @@
           <t>Pest Hunters · ККЗ, дезинсекция</t>
         </is>
       </c>
-      <c r="B54" s="42" t="n">
+      <c r="B54" s="41" t="n">
         <v>70000</v>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -6063,7 +5873,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H54" s="43" t="inlineStr">
+      <c r="H54" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -6075,7 +5885,7 @@
           <t>Pest Hunters · площадки, март — ноябрь</t>
         </is>
       </c>
-      <c r="B55" s="42" t="n">
+      <c r="B55" s="41" t="n">
         <v>3172000</v>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -6083,7 +5893,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H55" s="43" t="inlineStr">
+      <c r="H55" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); 122 объекта, оборудование подрядчика</t>
         </is>
@@ -6095,7 +5905,7 @@
           <t>Pest Hunters · площадки, декабрь — февраль</t>
         </is>
       </c>
-      <c r="B56" s="42" t="n">
+      <c r="B56" s="41" t="n">
         <v>2074000</v>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -6103,7 +5913,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H56" s="43" t="inlineStr">
+      <c r="H56" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); 122 объекта, оборудование подрядчика</t>
         </is>
@@ -6115,7 +5925,7 @@
           <t>Pest Hunters · площадки альт., март — ноябрь</t>
         </is>
       </c>
-      <c r="B57" s="42" t="n">
+      <c r="B57" s="41" t="n">
         <v>2806000</v>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -6123,7 +5933,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H57" s="43" t="inlineStr">
+      <c r="H57" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); оборудование заказчика</t>
         </is>
@@ -6135,7 +5945,7 @@
           <t>Pest Hunters · площадки альт., дек. — февраль</t>
         </is>
       </c>
-      <c r="B58" s="42" t="n">
+      <c r="B58" s="41" t="n">
         <v>1830000</v>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -6143,7 +5953,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H58" s="43" t="inlineStr">
+      <c r="H58" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС); оборудование заказчика</t>
         </is>
@@ -6155,7 +5965,7 @@
           <t>Pest Hunters · ЗПП</t>
         </is>
       </c>
-      <c r="B59" s="42" t="n">
+      <c r="B59" s="41" t="n">
         <v>180000</v>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -6163,7 +5973,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H59" s="43" t="inlineStr">
+      <c r="H59" s="42" t="inlineStr">
         <is>
           <t>договор №88 от 01.01.2026; дератизация + дезинсекция, 8 309 м², 3 обхода в месяц</t>
         </is>
@@ -6175,7 +5985,7 @@
           <t>Pest Hunters · склад ТМЦ</t>
         </is>
       </c>
-      <c r="B60" s="42" t="n">
+      <c r="B60" s="41" t="n">
         <v>80000</v>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -6183,7 +5993,7 @@
           <t>₸/мес</t>
         </is>
       </c>
-      <c r="H60" s="43" t="inlineStr">
+      <c r="H60" s="42" t="inlineStr">
         <is>
           <t>договор №921 от 01.04.2026; дератизация + дезинсекция, 1 обход в месяц</t>
         </is>
@@ -6195,7 +6005,7 @@
           <t>Месяцев высокого тарифа площадок (мар — ноя)</t>
         </is>
       </c>
-      <c r="B61" s="42" t="n">
+      <c r="B61" s="41" t="n">
         <v>9</v>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -6203,7 +6013,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H61" s="43" t="inlineStr">
+      <c r="H61" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -6215,7 +6025,7 @@
           <t>Месяцев низкого тарифа площадок (дек — фев)</t>
         </is>
       </c>
-      <c r="B62" s="42" t="n">
+      <c r="B62" s="41" t="n">
         <v>3</v>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -6223,7 +6033,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H62" s="43" t="inlineStr">
+      <c r="H62" s="42" t="inlineStr">
         <is>
           <t>Pest Hunters, КП №26/12 на 2026–2027 (без НДС)</t>
         </is>
@@ -6235,7 +6045,7 @@
           <t>Месяцев действия договора по складу ТМЦ</t>
         </is>
       </c>
-      <c r="B63" s="42" t="n">
+      <c r="B63" s="41" t="n">
         <v>9</v>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -6243,7 +6053,7 @@
           <t>мес.</t>
         </is>
       </c>
-      <c r="H63" s="43" t="inlineStr">
+      <c r="H63" s="42" t="inlineStr">
         <is>
           <t>апрель — декабрь 2026</t>
         </is>
@@ -6255,7 +6065,7 @@
           <t>Скидка Indigo за всю территорию фабрики</t>
         </is>
       </c>
-      <c r="B64" s="57" t="n">
+      <c r="B64" s="56" t="n">
         <v>0.15</v>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -6263,7 +6073,7 @@
           <t>доля</t>
         </is>
       </c>
-      <c r="H64" s="43" t="inlineStr">
+      <c r="H64" s="42" t="inlineStr">
         <is>
           <t>КП от 19.08.2026, условия предоставления скидок</t>
         </is>
@@ -6275,7 +6085,7 @@
           <t>Скидка Indigo за 100 % предоплату за год</t>
         </is>
       </c>
-      <c r="B65" s="57" t="n">
+      <c r="B65" s="56" t="n">
         <v>0.15</v>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -6283,7 +6093,7 @@
           <t>доля</t>
         </is>
       </c>
-      <c r="H65" s="43" t="inlineStr">
+      <c r="H65" s="42" t="inlineStr">
         <is>
           <t>КП от 19.08.2026, дополнительно к предыдущей</t>
         </is>
@@ -6295,7 +6105,7 @@
           <t>Скидка Indigo неплательщику НДС</t>
         </is>
       </c>
-      <c r="B66" s="57" t="n">
+      <c r="B66" s="56" t="n">
         <v>0.16</v>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -6303,7 +6113,7 @@
           <t>доля</t>
         </is>
       </c>
-      <c r="H66" s="43" t="inlineStr">
+      <c r="H66" s="42" t="inlineStr">
         <is>
           <t>КП от 19.08.2026; цены КП уже включают НДС</t>
         </is>

</xml_diff>